<commit_message>
Update testcases.xlsx to reflect new SIPS event types and structure
</commit_message>
<xml_diff>
--- a/testcases.xlsx
+++ b/testcases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://energinet-my.sharepoint.com/personal/prw_energinet_dk/Documents/Dokumenter/GitHub/MTB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_710D79F8E8F49B720F18F8F5A5BEAA4096265349" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D01AC370-765D-420F-9498-03240C275AF9}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="11_710D79F8E8F49B720F18F8F5A5BEAA4096265349" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D68397F5-7546-4295-817C-D589CC648AF5}"/>
   <bookViews>
-    <workbookView xWindow="21465" yWindow="-21720" windowWidth="38640" windowHeight="21120" tabRatio="822" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16935" yWindow="-21720" windowWidth="38640" windowHeight="21120" tabRatio="822" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="29" r:id="rId1"/>
@@ -31,8 +31,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Co-located cases'!$A$2:$BQ$178</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Custom cases'!$A$2:$BK$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'DCC cases'!$A$2:$BJ$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RfG cases'!$A$2:$BK$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'DCC cases'!$A$2:$BJ$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RfG cases'!$A$2:$BK$183</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Settings!$A$5:$E$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Unit cases'!$A$2:$BK$2</definedName>
     <definedName name="inp_Area" localSheetId="0">Settings!$B$28</definedName>
@@ -165,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5513" uniqueCount="948">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5513" uniqueCount="947">
   <si>
     <t>Comment</t>
   </si>
@@ -3702,9 +3702,6 @@
   </si>
   <si>
     <t>Maximum power available change (unit D, Co-Located)</t>
-  </si>
-  <si>
-    <t>SIPS</t>
   </si>
   <si>
     <t>equivalent binary value</t>
@@ -5784,9 +5781,6 @@
     <xf numFmtId="164" fontId="7" fillId="8" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5797,6 +5791,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5820,22 +5832,7 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5859,17 +5856,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -6426,23 +6423,23 @@
         <v>322</v>
       </c>
       <c r="G3" s="124"/>
-      <c r="H3" s="404" t="s">
+      <c r="H3" s="409" t="s">
         <v>339</v>
       </c>
-      <c r="I3" s="404"/>
-      <c r="J3" s="404"/>
-      <c r="K3" s="404" t="s">
+      <c r="I3" s="409"/>
+      <c r="J3" s="409"/>
+      <c r="K3" s="409" t="s">
         <v>340</v>
       </c>
-      <c r="L3" s="404"/>
-      <c r="M3" s="405"/>
+      <c r="L3" s="409"/>
+      <c r="M3" s="410"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4" s="248" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="247" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="C4" s="249" t="s">
         <v>10</v>
@@ -8361,13 +8358,13 @@
         <v>1087</v>
       </c>
       <c r="B88" s="281" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="C88" s="418" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="D88" s="146" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="29.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -8375,11 +8372,11 @@
         <v>1088</v>
       </c>
       <c r="B89" s="283" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="C89" s="420"/>
       <c r="D89" s="143" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.4">
@@ -9414,102 +9411,102 @@
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="333"/>
       <c r="B2" s="333"/>
-      <c r="C2" s="424" t="s">
+      <c r="C2" s="426" t="s">
         <v>843</v>
       </c>
-      <c r="D2" s="426" t="s">
+      <c r="D2" s="424" t="s">
         <v>907</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="333"/>
       <c r="B3" s="333"/>
-      <c r="C3" s="424"/>
-      <c r="D3" s="426"/>
+      <c r="C3" s="426"/>
+      <c r="D3" s="424"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="333"/>
       <c r="B4" s="333"/>
-      <c r="C4" s="424"/>
-      <c r="D4" s="426"/>
+      <c r="C4" s="426"/>
+      <c r="D4" s="424"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="333"/>
       <c r="B5" s="333"/>
-      <c r="C5" s="424"/>
-      <c r="D5" s="426"/>
+      <c r="C5" s="426"/>
+      <c r="D5" s="424"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="333"/>
       <c r="B6" s="333"/>
-      <c r="C6" s="424"/>
-      <c r="D6" s="426"/>
+      <c r="C6" s="426"/>
+      <c r="D6" s="424"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="333"/>
       <c r="B7" s="333"/>
-      <c r="C7" s="424"/>
-      <c r="D7" s="426"/>
+      <c r="C7" s="426"/>
+      <c r="D7" s="424"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="333"/>
       <c r="B8" s="333"/>
-      <c r="C8" s="424"/>
-      <c r="D8" s="426"/>
+      <c r="C8" s="426"/>
+      <c r="D8" s="424"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="333"/>
       <c r="B9" s="333"/>
-      <c r="C9" s="424"/>
-      <c r="D9" s="426"/>
+      <c r="C9" s="426"/>
+      <c r="D9" s="424"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="333"/>
       <c r="B10" s="333"/>
-      <c r="C10" s="424"/>
-      <c r="D10" s="426"/>
+      <c r="C10" s="426"/>
+      <c r="D10" s="424"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="333"/>
       <c r="B11" s="333"/>
-      <c r="C11" s="424"/>
-      <c r="D11" s="426"/>
+      <c r="C11" s="426"/>
+      <c r="D11" s="424"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="333"/>
       <c r="B12" s="333"/>
-      <c r="C12" s="424"/>
-      <c r="D12" s="426"/>
+      <c r="C12" s="426"/>
+      <c r="D12" s="424"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="333"/>
       <c r="B13" s="333"/>
-      <c r="C13" s="424"/>
-      <c r="D13" s="426"/>
+      <c r="C13" s="426"/>
+      <c r="D13" s="424"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="333"/>
       <c r="B14" s="333"/>
-      <c r="C14" s="424"/>
-      <c r="D14" s="426"/>
+      <c r="C14" s="426"/>
+      <c r="D14" s="424"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="333"/>
       <c r="B15" s="333"/>
-      <c r="C15" s="424"/>
-      <c r="D15" s="426"/>
+      <c r="C15" s="426"/>
+      <c r="D15" s="424"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="333"/>
       <c r="B16" s="333"/>
-      <c r="C16" s="424"/>
-      <c r="D16" s="426"/>
+      <c r="C16" s="426"/>
+      <c r="D16" s="424"/>
     </row>
     <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A17" s="315"/>
       <c r="B17" s="315"/>
-      <c r="C17" s="425"/>
-      <c r="D17" s="427"/>
+      <c r="C17" s="427"/>
+      <c r="D17" s="425"/>
     </row>
     <row r="18" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="335"/>
@@ -9517,7 +9514,7 @@
       <c r="C18" s="419" t="s">
         <v>361</v>
       </c>
-      <c r="D18" s="426" t="s">
+      <c r="D18" s="424" t="s">
         <v>844</v>
       </c>
     </row>
@@ -9525,115 +9522,115 @@
       <c r="A19" s="335"/>
       <c r="B19" s="335"/>
       <c r="C19" s="419"/>
-      <c r="D19" s="426"/>
+      <c r="D19" s="424"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="335"/>
       <c r="B20" s="335"/>
       <c r="C20" s="419"/>
-      <c r="D20" s="426"/>
+      <c r="D20" s="424"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="335"/>
       <c r="B21" s="335"/>
       <c r="C21" s="419"/>
-      <c r="D21" s="426"/>
+      <c r="D21" s="424"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="335"/>
       <c r="B22" s="335"/>
       <c r="C22" s="419"/>
-      <c r="D22" s="426"/>
+      <c r="D22" s="424"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="335"/>
       <c r="B23" s="335"/>
       <c r="C23" s="419"/>
-      <c r="D23" s="426"/>
+      <c r="D23" s="424"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" s="335"/>
       <c r="B24" s="335"/>
       <c r="C24" s="419"/>
-      <c r="D24" s="426"/>
+      <c r="D24" s="424"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" s="335"/>
       <c r="B25" s="335"/>
       <c r="C25" s="419"/>
-      <c r="D25" s="426"/>
+      <c r="D25" s="424"/>
     </row>
     <row r="26" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="335"/>
       <c r="B26" s="335"/>
       <c r="C26" s="419"/>
-      <c r="D26" s="426"/>
+      <c r="D26" s="424"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="335"/>
       <c r="B27" s="335"/>
       <c r="C27" s="419"/>
-      <c r="D27" s="426"/>
+      <c r="D27" s="424"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="335"/>
       <c r="B28" s="335"/>
       <c r="C28" s="419"/>
-      <c r="D28" s="426"/>
+      <c r="D28" s="424"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="335"/>
       <c r="B29" s="335"/>
       <c r="C29" s="419"/>
-      <c r="D29" s="426"/>
+      <c r="D29" s="424"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="335"/>
       <c r="B30" s="335"/>
       <c r="C30" s="419"/>
-      <c r="D30" s="426"/>
+      <c r="D30" s="424"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="335"/>
       <c r="B31" s="335"/>
       <c r="C31" s="419"/>
-      <c r="D31" s="426"/>
+      <c r="D31" s="424"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="335"/>
       <c r="B32" s="335"/>
       <c r="C32" s="419"/>
-      <c r="D32" s="426"/>
+      <c r="D32" s="424"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="335"/>
       <c r="B33" s="335"/>
       <c r="C33" s="419"/>
-      <c r="D33" s="426"/>
+      <c r="D33" s="424"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="335"/>
       <c r="B34" s="335"/>
       <c r="C34" s="419"/>
-      <c r="D34" s="426"/>
+      <c r="D34" s="424"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="335"/>
       <c r="B35" s="335"/>
       <c r="C35" s="419"/>
-      <c r="D35" s="426"/>
+      <c r="D35" s="424"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="335"/>
       <c r="B36" s="335"/>
       <c r="C36" s="419"/>
-      <c r="D36" s="426"/>
+      <c r="D36" s="424"/>
     </row>
     <row r="37" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A37" s="316"/>
       <c r="B37" s="316"/>
       <c r="C37" s="420"/>
-      <c r="D37" s="427"/>
+      <c r="D37" s="425"/>
     </row>
     <row r="38" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="334"/>
@@ -9641,7 +9638,7 @@
       <c r="C38" s="419" t="s">
         <v>845</v>
       </c>
-      <c r="D38" s="426" t="s">
+      <c r="D38" s="424" t="s">
         <v>846</v>
       </c>
     </row>
@@ -9649,115 +9646,115 @@
       <c r="A39" s="334"/>
       <c r="B39" s="334"/>
       <c r="C39" s="419"/>
-      <c r="D39" s="426"/>
+      <c r="D39" s="424"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A40" s="334"/>
       <c r="B40" s="334"/>
       <c r="C40" s="419"/>
-      <c r="D40" s="426"/>
+      <c r="D40" s="424"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A41" s="334"/>
       <c r="B41" s="334"/>
       <c r="C41" s="419"/>
-      <c r="D41" s="426"/>
+      <c r="D41" s="424"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A42" s="334"/>
       <c r="B42" s="334"/>
       <c r="C42" s="419"/>
-      <c r="D42" s="426"/>
+      <c r="D42" s="424"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A43" s="334"/>
       <c r="B43" s="334"/>
       <c r="C43" s="419"/>
-      <c r="D43" s="426"/>
+      <c r="D43" s="424"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A44" s="334"/>
       <c r="B44" s="334"/>
       <c r="C44" s="419"/>
-      <c r="D44" s="426"/>
+      <c r="D44" s="424"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A45" s="334"/>
       <c r="B45" s="334"/>
       <c r="C45" s="419"/>
-      <c r="D45" s="426"/>
+      <c r="D45" s="424"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A46" s="334"/>
       <c r="B46" s="334"/>
       <c r="C46" s="419"/>
-      <c r="D46" s="426"/>
+      <c r="D46" s="424"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A47" s="334"/>
       <c r="B47" s="334"/>
       <c r="C47" s="419"/>
-      <c r="D47" s="426"/>
+      <c r="D47" s="424"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A48" s="334"/>
       <c r="B48" s="334"/>
       <c r="C48" s="419"/>
-      <c r="D48" s="426"/>
+      <c r="D48" s="424"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A49" s="334"/>
       <c r="B49" s="334"/>
       <c r="C49" s="419"/>
-      <c r="D49" s="426"/>
+      <c r="D49" s="424"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A50" s="334"/>
       <c r="B50" s="334"/>
       <c r="C50" s="419"/>
-      <c r="D50" s="426"/>
+      <c r="D50" s="424"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A51" s="334"/>
       <c r="B51" s="334"/>
       <c r="C51" s="419"/>
-      <c r="D51" s="426"/>
+      <c r="D51" s="424"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A52" s="334"/>
       <c r="B52" s="334"/>
       <c r="C52" s="419"/>
-      <c r="D52" s="426"/>
+      <c r="D52" s="424"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" s="334"/>
       <c r="B53" s="334"/>
       <c r="C53" s="419"/>
-      <c r="D53" s="426"/>
+      <c r="D53" s="424"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A54" s="334"/>
       <c r="B54" s="334"/>
       <c r="C54" s="419"/>
-      <c r="D54" s="426"/>
+      <c r="D54" s="424"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A55" s="334"/>
       <c r="B55" s="334"/>
       <c r="C55" s="419"/>
-      <c r="D55" s="426"/>
+      <c r="D55" s="424"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A56" s="334"/>
       <c r="B56" s="334"/>
       <c r="C56" s="419"/>
-      <c r="D56" s="426"/>
+      <c r="D56" s="424"/>
     </row>
     <row r="57" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A57" s="317"/>
       <c r="B57" s="317"/>
       <c r="C57" s="420"/>
-      <c r="D57" s="427"/>
+      <c r="D57" s="425"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A58" s="336"/>
@@ -9765,7 +9762,7 @@
       <c r="C58" s="419" t="s">
         <v>847</v>
       </c>
-      <c r="D58" s="426" t="s">
+      <c r="D58" s="424" t="s">
         <v>848</v>
       </c>
     </row>
@@ -9773,85 +9770,85 @@
       <c r="A59" s="336"/>
       <c r="B59" s="336"/>
       <c r="C59" s="419"/>
-      <c r="D59" s="426"/>
+      <c r="D59" s="424"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A60" s="336"/>
       <c r="B60" s="336"/>
       <c r="C60" s="419"/>
-      <c r="D60" s="426"/>
+      <c r="D60" s="424"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A61" s="336"/>
       <c r="B61" s="336"/>
       <c r="C61" s="419"/>
-      <c r="D61" s="426"/>
+      <c r="D61" s="424"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A62" s="336"/>
       <c r="B62" s="336"/>
       <c r="C62" s="419"/>
-      <c r="D62" s="426"/>
+      <c r="D62" s="424"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A63" s="336"/>
       <c r="B63" s="336"/>
       <c r="C63" s="419"/>
-      <c r="D63" s="426"/>
+      <c r="D63" s="424"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A64" s="336"/>
       <c r="B64" s="336"/>
       <c r="C64" s="419"/>
-      <c r="D64" s="426"/>
+      <c r="D64" s="424"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A65" s="336"/>
       <c r="B65" s="336"/>
       <c r="C65" s="419"/>
-      <c r="D65" s="426"/>
+      <c r="D65" s="424"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A66" s="336"/>
       <c r="B66" s="336"/>
       <c r="C66" s="419"/>
-      <c r="D66" s="426"/>
+      <c r="D66" s="424"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A67" s="336"/>
       <c r="B67" s="336"/>
       <c r="C67" s="419"/>
-      <c r="D67" s="426"/>
+      <c r="D67" s="424"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A68" s="336"/>
       <c r="B68" s="336"/>
       <c r="C68" s="419"/>
-      <c r="D68" s="426"/>
+      <c r="D68" s="424"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A69" s="336"/>
       <c r="B69" s="336"/>
       <c r="C69" s="419"/>
-      <c r="D69" s="426"/>
+      <c r="D69" s="424"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A70" s="336"/>
       <c r="B70" s="336"/>
       <c r="C70" s="419"/>
-      <c r="D70" s="426"/>
+      <c r="D70" s="424"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A71" s="336"/>
       <c r="B71" s="336"/>
       <c r="C71" s="419"/>
-      <c r="D71" s="426"/>
+      <c r="D71" s="424"/>
     </row>
     <row r="72" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A72" s="318"/>
       <c r="B72" s="318"/>
       <c r="C72" s="420"/>
-      <c r="D72" s="427"/>
+      <c r="D72" s="425"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A73" s="338"/>
@@ -9859,7 +9856,7 @@
       <c r="C73" s="419" t="s">
         <v>849</v>
       </c>
-      <c r="D73" s="426" t="s">
+      <c r="D73" s="424" t="s">
         <v>850</v>
       </c>
     </row>
@@ -9867,97 +9864,97 @@
       <c r="A74" s="338"/>
       <c r="B74" s="338"/>
       <c r="C74" s="419"/>
-      <c r="D74" s="426"/>
+      <c r="D74" s="424"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A75" s="338"/>
       <c r="B75" s="338"/>
       <c r="C75" s="419"/>
-      <c r="D75" s="426"/>
+      <c r="D75" s="424"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A76" s="338"/>
       <c r="B76" s="338"/>
       <c r="C76" s="419"/>
-      <c r="D76" s="426"/>
+      <c r="D76" s="424"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A77" s="338"/>
       <c r="B77" s="338"/>
       <c r="C77" s="419"/>
-      <c r="D77" s="426"/>
+      <c r="D77" s="424"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A78" s="338"/>
       <c r="B78" s="338"/>
       <c r="C78" s="419"/>
-      <c r="D78" s="426"/>
+      <c r="D78" s="424"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A79" s="338"/>
       <c r="B79" s="338"/>
       <c r="C79" s="419"/>
-      <c r="D79" s="426"/>
+      <c r="D79" s="424"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A80" s="338"/>
       <c r="B80" s="338"/>
       <c r="C80" s="419"/>
-      <c r="D80" s="426"/>
+      <c r="D80" s="424"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A81" s="338"/>
       <c r="B81" s="338"/>
       <c r="C81" s="419"/>
-      <c r="D81" s="426"/>
+      <c r="D81" s="424"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A82" s="338"/>
       <c r="B82" s="338"/>
       <c r="C82" s="419"/>
-      <c r="D82" s="426"/>
+      <c r="D82" s="424"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A83" s="338"/>
       <c r="B83" s="338"/>
       <c r="C83" s="419"/>
-      <c r="D83" s="426"/>
+      <c r="D83" s="424"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A84" s="338"/>
       <c r="B84" s="338"/>
       <c r="C84" s="419"/>
-      <c r="D84" s="426"/>
+      <c r="D84" s="424"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A85" s="338"/>
       <c r="B85" s="338"/>
       <c r="C85" s="419"/>
-      <c r="D85" s="426"/>
+      <c r="D85" s="424"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A86" s="338"/>
       <c r="B86" s="338"/>
       <c r="C86" s="419"/>
-      <c r="D86" s="426"/>
+      <c r="D86" s="424"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A87" s="338"/>
       <c r="B87" s="338"/>
       <c r="C87" s="419"/>
-      <c r="D87" s="426"/>
+      <c r="D87" s="424"/>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A88" s="338"/>
       <c r="B88" s="338"/>
       <c r="C88" s="419"/>
-      <c r="D88" s="426"/>
+      <c r="D88" s="424"/>
     </row>
     <row r="89" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A89" s="319"/>
       <c r="B89" s="319"/>
       <c r="C89" s="420"/>
-      <c r="D89" s="427"/>
+      <c r="D89" s="425"/>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A90" s="337"/>
@@ -9965,7 +9962,7 @@
       <c r="C90" s="419" t="s">
         <v>851</v>
       </c>
-      <c r="D90" s="426" t="s">
+      <c r="D90" s="424" t="s">
         <v>852</v>
       </c>
     </row>
@@ -9973,49 +9970,49 @@
       <c r="A91" s="337"/>
       <c r="B91" s="337"/>
       <c r="C91" s="419"/>
-      <c r="D91" s="426"/>
+      <c r="D91" s="424"/>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A92" s="337"/>
       <c r="B92" s="337"/>
       <c r="C92" s="419"/>
-      <c r="D92" s="426"/>
+      <c r="D92" s="424"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A93" s="337"/>
       <c r="B93" s="337"/>
       <c r="C93" s="419"/>
-      <c r="D93" s="426"/>
+      <c r="D93" s="424"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A94" s="337"/>
       <c r="B94" s="337"/>
       <c r="C94" s="419"/>
-      <c r="D94" s="426"/>
+      <c r="D94" s="424"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A95" s="337"/>
       <c r="B95" s="337"/>
       <c r="C95" s="419"/>
-      <c r="D95" s="426"/>
+      <c r="D95" s="424"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A96" s="337"/>
       <c r="B96" s="337"/>
       <c r="C96" s="419"/>
-      <c r="D96" s="426"/>
+      <c r="D96" s="424"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A97" s="337"/>
       <c r="B97" s="337"/>
       <c r="C97" s="419"/>
-      <c r="D97" s="426"/>
+      <c r="D97" s="424"/>
     </row>
     <row r="98" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A98" s="320"/>
       <c r="B98" s="320"/>
       <c r="C98" s="420"/>
-      <c r="D98" s="427"/>
+      <c r="D98" s="425"/>
     </row>
     <row r="99" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A99" s="339"/>
@@ -10023,7 +10020,7 @@
       <c r="C99" s="422" t="s">
         <v>853</v>
       </c>
-      <c r="D99" s="426" t="s">
+      <c r="D99" s="424" t="s">
         <v>854</v>
       </c>
     </row>
@@ -10031,73 +10028,73 @@
       <c r="A100" s="339"/>
       <c r="B100" s="339"/>
       <c r="C100" s="422"/>
-      <c r="D100" s="426"/>
+      <c r="D100" s="424"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A101" s="339"/>
       <c r="B101" s="339"/>
       <c r="C101" s="422"/>
-      <c r="D101" s="426"/>
+      <c r="D101" s="424"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A102" s="339"/>
       <c r="B102" s="339"/>
       <c r="C102" s="422"/>
-      <c r="D102" s="426"/>
+      <c r="D102" s="424"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A103" s="339"/>
       <c r="B103" s="339"/>
       <c r="C103" s="422"/>
-      <c r="D103" s="426"/>
+      <c r="D103" s="424"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A104" s="339"/>
       <c r="B104" s="339"/>
       <c r="C104" s="422"/>
-      <c r="D104" s="426"/>
+      <c r="D104" s="424"/>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A105" s="339"/>
       <c r="B105" s="339"/>
       <c r="C105" s="422"/>
-      <c r="D105" s="426"/>
+      <c r="D105" s="424"/>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A106" s="339"/>
       <c r="B106" s="339"/>
       <c r="C106" s="422"/>
-      <c r="D106" s="426"/>
+      <c r="D106" s="424"/>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A107" s="339"/>
       <c r="B107" s="339"/>
       <c r="C107" s="422"/>
-      <c r="D107" s="426"/>
+      <c r="D107" s="424"/>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A108" s="339"/>
       <c r="B108" s="339"/>
       <c r="C108" s="422"/>
-      <c r="D108" s="426"/>
+      <c r="D108" s="424"/>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A109" s="339"/>
       <c r="B109" s="339"/>
       <c r="C109" s="422"/>
-      <c r="D109" s="426"/>
+      <c r="D109" s="424"/>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A110" s="339"/>
       <c r="B110" s="339"/>
       <c r="C110" s="422"/>
-      <c r="D110" s="426"/>
+      <c r="D110" s="424"/>
     </row>
     <row r="111" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A111" s="321"/>
       <c r="B111" s="321"/>
       <c r="C111" s="423"/>
-      <c r="D111" s="427"/>
+      <c r="D111" s="425"/>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A112" s="335"/>
@@ -10105,7 +10102,7 @@
       <c r="C112" s="419" t="s">
         <v>855</v>
       </c>
-      <c r="D112" s="426" t="s">
+      <c r="D112" s="424" t="s">
         <v>856</v>
       </c>
     </row>
@@ -10113,67 +10110,67 @@
       <c r="A113" s="335"/>
       <c r="B113" s="335"/>
       <c r="C113" s="419"/>
-      <c r="D113" s="426"/>
+      <c r="D113" s="424"/>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A114" s="335"/>
       <c r="B114" s="335"/>
       <c r="C114" s="419"/>
-      <c r="D114" s="426"/>
+      <c r="D114" s="424"/>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A115" s="335"/>
       <c r="B115" s="335"/>
       <c r="C115" s="419"/>
-      <c r="D115" s="426"/>
+      <c r="D115" s="424"/>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A116" s="335"/>
       <c r="B116" s="335"/>
       <c r="C116" s="419"/>
-      <c r="D116" s="426"/>
+      <c r="D116" s="424"/>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A117" s="335"/>
       <c r="B117" s="335"/>
       <c r="C117" s="419"/>
-      <c r="D117" s="426"/>
+      <c r="D117" s="424"/>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A118" s="335"/>
       <c r="B118" s="335"/>
       <c r="C118" s="419"/>
-      <c r="D118" s="426"/>
+      <c r="D118" s="424"/>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A119" s="335"/>
       <c r="B119" s="335"/>
       <c r="C119" s="419"/>
-      <c r="D119" s="426"/>
+      <c r="D119" s="424"/>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A120" s="335"/>
       <c r="B120" s="335"/>
       <c r="C120" s="419"/>
-      <c r="D120" s="426"/>
+      <c r="D120" s="424"/>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A121" s="335"/>
       <c r="B121" s="335"/>
       <c r="C121" s="419"/>
-      <c r="D121" s="426"/>
+      <c r="D121" s="424"/>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A122" s="335"/>
       <c r="B122" s="335"/>
       <c r="C122" s="419"/>
-      <c r="D122" s="426"/>
+      <c r="D122" s="424"/>
     </row>
     <row r="123" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A123" s="316"/>
       <c r="B123" s="316"/>
       <c r="C123" s="420"/>
-      <c r="D123" s="427"/>
+      <c r="D123" s="425"/>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A124" s="334"/>
@@ -10181,7 +10178,7 @@
       <c r="C124" s="419" t="s">
         <v>857</v>
       </c>
-      <c r="D124" s="426" t="s">
+      <c r="D124" s="424" t="s">
         <v>858</v>
       </c>
     </row>
@@ -10189,31 +10186,31 @@
       <c r="A125" s="334"/>
       <c r="B125" s="334"/>
       <c r="C125" s="419"/>
-      <c r="D125" s="426"/>
+      <c r="D125" s="424"/>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A126" s="334"/>
       <c r="B126" s="334"/>
       <c r="C126" s="419"/>
-      <c r="D126" s="426"/>
+      <c r="D126" s="424"/>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A127" s="334"/>
       <c r="B127" s="334"/>
       <c r="C127" s="419"/>
-      <c r="D127" s="426"/>
+      <c r="D127" s="424"/>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A128" s="334"/>
       <c r="B128" s="334"/>
       <c r="C128" s="419"/>
-      <c r="D128" s="426"/>
+      <c r="D128" s="424"/>
     </row>
     <row r="129" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A129" s="317"/>
       <c r="B129" s="317"/>
       <c r="C129" s="420"/>
-      <c r="D129" s="427"/>
+      <c r="D129" s="425"/>
     </row>
     <row r="130" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A130" s="33"/>
@@ -10221,7 +10218,7 @@
       <c r="C130" s="419" t="s">
         <v>859</v>
       </c>
-      <c r="D130" s="426" t="s">
+      <c r="D130" s="424" t="s">
         <v>860</v>
       </c>
     </row>
@@ -10229,19 +10226,19 @@
       <c r="A131" s="33"/>
       <c r="B131" s="33"/>
       <c r="C131" s="419"/>
-      <c r="D131" s="426"/>
+      <c r="D131" s="424"/>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A132" s="33"/>
       <c r="B132" s="33"/>
       <c r="C132" s="419"/>
-      <c r="D132" s="426"/>
+      <c r="D132" s="424"/>
     </row>
     <row r="133" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A133" s="322"/>
       <c r="B133" s="322"/>
       <c r="C133" s="420"/>
-      <c r="D133" s="427"/>
+      <c r="D133" s="425"/>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A134" s="338"/>
@@ -10249,7 +10246,7 @@
       <c r="C134" s="419" t="s">
         <v>861</v>
       </c>
-      <c r="D134" s="426" t="s">
+      <c r="D134" s="424" t="s">
         <v>862</v>
       </c>
     </row>
@@ -10257,103 +10254,103 @@
       <c r="A135" s="338"/>
       <c r="B135" s="338"/>
       <c r="C135" s="419"/>
-      <c r="D135" s="426"/>
+      <c r="D135" s="424"/>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A136" s="338"/>
       <c r="B136" s="338"/>
       <c r="C136" s="419"/>
-      <c r="D136" s="426"/>
+      <c r="D136" s="424"/>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A137" s="338"/>
       <c r="B137" s="338"/>
       <c r="C137" s="419"/>
-      <c r="D137" s="426"/>
+      <c r="D137" s="424"/>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A138" s="338"/>
       <c r="B138" s="338"/>
       <c r="C138" s="419"/>
-      <c r="D138" s="426"/>
+      <c r="D138" s="424"/>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A139" s="338"/>
       <c r="B139" s="338"/>
       <c r="C139" s="419"/>
-      <c r="D139" s="426"/>
+      <c r="D139" s="424"/>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A140" s="338"/>
       <c r="B140" s="338"/>
       <c r="C140" s="419"/>
-      <c r="D140" s="426"/>
+      <c r="D140" s="424"/>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A141" s="338"/>
       <c r="B141" s="338"/>
       <c r="C141" s="419"/>
-      <c r="D141" s="426"/>
+      <c r="D141" s="424"/>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A142" s="338"/>
       <c r="B142" s="338"/>
       <c r="C142" s="419"/>
-      <c r="D142" s="426"/>
+      <c r="D142" s="424"/>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A143" s="338"/>
       <c r="B143" s="338"/>
       <c r="C143" s="419"/>
-      <c r="D143" s="426"/>
+      <c r="D143" s="424"/>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A144" s="338"/>
       <c r="B144" s="338"/>
       <c r="C144" s="419"/>
-      <c r="D144" s="426"/>
+      <c r="D144" s="424"/>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A145" s="338"/>
       <c r="B145" s="338"/>
       <c r="C145" s="419"/>
-      <c r="D145" s="426"/>
+      <c r="D145" s="424"/>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A146" s="338"/>
       <c r="B146" s="338"/>
       <c r="C146" s="419"/>
-      <c r="D146" s="426"/>
+      <c r="D146" s="424"/>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A147" s="338"/>
       <c r="B147" s="338"/>
       <c r="C147" s="419"/>
-      <c r="D147" s="426"/>
+      <c r="D147" s="424"/>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A148" s="338"/>
       <c r="B148" s="338"/>
       <c r="C148" s="419"/>
-      <c r="D148" s="426"/>
+      <c r="D148" s="424"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A149" s="338"/>
       <c r="B149" s="338"/>
       <c r="C149" s="419"/>
-      <c r="D149" s="426"/>
+      <c r="D149" s="424"/>
     </row>
     <row r="150" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A150" s="338"/>
       <c r="B150" s="338"/>
       <c r="C150" s="419"/>
-      <c r="D150" s="426"/>
+      <c r="D150" s="424"/>
     </row>
     <row r="151" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A151" s="319"/>
       <c r="B151" s="319"/>
       <c r="C151" s="420"/>
-      <c r="D151" s="427"/>
+      <c r="D151" s="425"/>
     </row>
     <row r="152" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A152" s="340"/>
@@ -10361,7 +10358,7 @@
       <c r="C152" s="419" t="s">
         <v>863</v>
       </c>
-      <c r="D152" s="426" t="s">
+      <c r="D152" s="424" t="s">
         <v>864</v>
       </c>
     </row>
@@ -10369,47 +10366,47 @@
       <c r="A153" s="340"/>
       <c r="B153" s="340"/>
       <c r="C153" s="419"/>
-      <c r="D153" s="426"/>
+      <c r="D153" s="424"/>
     </row>
     <row r="154" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A154" s="340"/>
       <c r="B154" s="340"/>
       <c r="C154" s="419"/>
-      <c r="D154" s="426"/>
+      <c r="D154" s="424"/>
     </row>
     <row r="155" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A155" s="323"/>
       <c r="B155" s="323"/>
       <c r="C155" s="420"/>
-      <c r="D155" s="427"/>
+      <c r="D155" s="425"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="24">
+    <mergeCell ref="C2:C17"/>
+    <mergeCell ref="D2:D17"/>
+    <mergeCell ref="C18:C37"/>
+    <mergeCell ref="D18:D37"/>
+    <mergeCell ref="C38:C57"/>
+    <mergeCell ref="D38:D57"/>
+    <mergeCell ref="C58:C72"/>
+    <mergeCell ref="D58:D72"/>
+    <mergeCell ref="C73:C89"/>
+    <mergeCell ref="D73:D89"/>
+    <mergeCell ref="C90:C98"/>
+    <mergeCell ref="D90:D98"/>
+    <mergeCell ref="C99:C111"/>
+    <mergeCell ref="D99:D111"/>
+    <mergeCell ref="C112:C123"/>
+    <mergeCell ref="D112:D123"/>
+    <mergeCell ref="C124:C129"/>
+    <mergeCell ref="D124:D129"/>
     <mergeCell ref="C130:C133"/>
     <mergeCell ref="D130:D133"/>
     <mergeCell ref="C134:C151"/>
     <mergeCell ref="D134:D151"/>
     <mergeCell ref="C152:C155"/>
     <mergeCell ref="D152:D155"/>
-    <mergeCell ref="C99:C111"/>
-    <mergeCell ref="D99:D111"/>
-    <mergeCell ref="C112:C123"/>
-    <mergeCell ref="D112:D123"/>
-    <mergeCell ref="C124:C129"/>
-    <mergeCell ref="D124:D129"/>
-    <mergeCell ref="C58:C72"/>
-    <mergeCell ref="D58:D72"/>
-    <mergeCell ref="C73:C89"/>
-    <mergeCell ref="D73:D89"/>
-    <mergeCell ref="C90:C98"/>
-    <mergeCell ref="D90:D98"/>
-    <mergeCell ref="C2:C17"/>
-    <mergeCell ref="D2:D17"/>
-    <mergeCell ref="C18:C37"/>
-    <mergeCell ref="D18:D37"/>
-    <mergeCell ref="C38:C57"/>
-    <mergeCell ref="D38:D57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -11747,21 +11744,21 @@
   <sheetData>
     <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="33"/>
-      <c r="B1" s="406" t="s">
+      <c r="B1" s="411" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="407"/>
-      <c r="D1" s="408"/>
-      <c r="E1" s="406" t="s">
+      <c r="C1" s="412"/>
+      <c r="D1" s="413"/>
+      <c r="E1" s="411" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="407"/>
-      <c r="G1" s="407"/>
+      <c r="F1" s="412"/>
+      <c r="G1" s="412"/>
       <c r="H1" s="309"/>
-      <c r="K1" s="409" t="s">
+      <c r="K1" s="414" t="s">
         <v>836</v>
       </c>
-      <c r="L1" s="410"/>
+      <c r="L1" s="415"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A2" s="61" t="s">
@@ -12793,31 +12790,31 @@
     <col min="13" max="13" width="8.3828125" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14.69140625" style="1" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20.69140625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="22.84375" style="96" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.3828125" style="96" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="9.69140625" style="96" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="35" style="96" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="16.53515625" style="96" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.53515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.3828125" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="9.69140625" style="1" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="25" style="1" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="16.53515625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="12" style="96" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.3828125" style="96" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="9.69140625" style="96" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="12.3828125" style="96" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="16.53515625" style="96" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.3828125" style="1" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="9.69140625" style="1" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="12.3828125" style="1" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="16.53515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12" style="96" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="14.3828125" style="96" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="9.69140625" style="96" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="12.3828125" style="96" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="16.53515625" style="96" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="14.3828125" style="1" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="9.69140625" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="12.3828125" style="1" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="16.53515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="10.69140625" style="96" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="14.3828125" style="96" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="9.69140625" style="96" bestFit="1" customWidth="1"/>
     <col min="42" max="42" width="12.3828125" style="96" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="16.53515625" style="96" bestFit="1" customWidth="1"/>
@@ -12849,103 +12846,103 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:67" x14ac:dyDescent="0.4">
-      <c r="A1" s="400" t="s">
+      <c r="A1" s="399" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="400"/>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="401" t="s">
+      <c r="B1" s="399"/>
+      <c r="C1" s="399"/>
+      <c r="D1" s="399"/>
+      <c r="E1" s="400" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="402"/>
-      <c r="I1" s="402"/>
-      <c r="J1" s="402"/>
-      <c r="K1" s="402"/>
-      <c r="L1" s="402"/>
-      <c r="M1" s="402"/>
-      <c r="N1" s="402"/>
-      <c r="O1" s="403"/>
-      <c r="P1" s="399" t="s">
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="401"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="401"/>
+      <c r="O1" s="402"/>
+      <c r="P1" s="416" t="s">
         <v>77</v>
       </c>
-      <c r="Q1" s="399"/>
-      <c r="R1" s="399"/>
-      <c r="S1" s="399"/>
-      <c r="T1" s="400" t="s">
+      <c r="Q1" s="416"/>
+      <c r="R1" s="416"/>
+      <c r="S1" s="416"/>
+      <c r="T1" s="399" t="s">
         <v>78</v>
       </c>
-      <c r="U1" s="400"/>
-      <c r="V1" s="400"/>
-      <c r="W1" s="400"/>
-      <c r="X1" s="399" t="s">
+      <c r="U1" s="399"/>
+      <c r="V1" s="399"/>
+      <c r="W1" s="399"/>
+      <c r="X1" s="416" t="s">
         <v>79</v>
       </c>
-      <c r="Y1" s="399"/>
-      <c r="Z1" s="399"/>
-      <c r="AA1" s="399"/>
-      <c r="AB1" s="400" t="s">
+      <c r="Y1" s="416"/>
+      <c r="Z1" s="416"/>
+      <c r="AA1" s="416"/>
+      <c r="AB1" s="399" t="s">
         <v>80</v>
       </c>
-      <c r="AC1" s="400"/>
-      <c r="AD1" s="400"/>
-      <c r="AE1" s="400"/>
-      <c r="AF1" s="399" t="s">
+      <c r="AC1" s="399"/>
+      <c r="AD1" s="399"/>
+      <c r="AE1" s="399"/>
+      <c r="AF1" s="416" t="s">
         <v>81</v>
       </c>
-      <c r="AG1" s="399"/>
-      <c r="AH1" s="399"/>
-      <c r="AI1" s="399"/>
-      <c r="AJ1" s="400" t="s">
+      <c r="AG1" s="416"/>
+      <c r="AH1" s="416"/>
+      <c r="AI1" s="416"/>
+      <c r="AJ1" s="399" t="s">
         <v>82</v>
       </c>
-      <c r="AK1" s="400"/>
-      <c r="AL1" s="400"/>
-      <c r="AM1" s="400"/>
-      <c r="AN1" s="399" t="s">
+      <c r="AK1" s="399"/>
+      <c r="AL1" s="399"/>
+      <c r="AM1" s="399"/>
+      <c r="AN1" s="416" t="s">
         <v>83</v>
       </c>
-      <c r="AO1" s="399"/>
-      <c r="AP1" s="399"/>
-      <c r="AQ1" s="399"/>
-      <c r="AR1" s="400" t="s">
+      <c r="AO1" s="416"/>
+      <c r="AP1" s="416"/>
+      <c r="AQ1" s="416"/>
+      <c r="AR1" s="399" t="s">
         <v>84</v>
       </c>
-      <c r="AS1" s="400"/>
-      <c r="AT1" s="400"/>
-      <c r="AU1" s="400"/>
-      <c r="AV1" s="399" t="s">
+      <c r="AS1" s="399"/>
+      <c r="AT1" s="399"/>
+      <c r="AU1" s="399"/>
+      <c r="AV1" s="416" t="s">
         <v>85</v>
       </c>
-      <c r="AW1" s="399"/>
-      <c r="AX1" s="399"/>
-      <c r="AY1" s="399"/>
-      <c r="AZ1" s="400" t="s">
+      <c r="AW1" s="416"/>
+      <c r="AX1" s="416"/>
+      <c r="AY1" s="416"/>
+      <c r="AZ1" s="399" t="s">
         <v>86</v>
       </c>
-      <c r="BA1" s="400"/>
-      <c r="BB1" s="400"/>
-      <c r="BC1" s="400"/>
-      <c r="BD1" s="399" t="s">
+      <c r="BA1" s="399"/>
+      <c r="BB1" s="399"/>
+      <c r="BC1" s="399"/>
+      <c r="BD1" s="416" t="s">
         <v>87</v>
       </c>
-      <c r="BE1" s="399"/>
-      <c r="BF1" s="399"/>
-      <c r="BG1" s="399"/>
-      <c r="BH1" s="400" t="s">
+      <c r="BE1" s="416"/>
+      <c r="BF1" s="416"/>
+      <c r="BG1" s="416"/>
+      <c r="BH1" s="399" t="s">
         <v>88</v>
       </c>
-      <c r="BI1" s="400"/>
-      <c r="BJ1" s="400"/>
-      <c r="BK1" s="400"/>
-      <c r="BL1" s="399" t="s">
+      <c r="BI1" s="399"/>
+      <c r="BJ1" s="399"/>
+      <c r="BK1" s="399"/>
+      <c r="BL1" s="416" t="s">
         <v>495</v>
       </c>
-      <c r="BM1" s="399"/>
-      <c r="BN1" s="399"/>
-      <c r="BO1" s="399"/>
+      <c r="BM1" s="416"/>
+      <c r="BN1" s="416"/>
+      <c r="BO1" s="416"/>
     </row>
     <row r="2" spans="1:67" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -20007,7 +20004,7 @@
         <v>90</v>
       </c>
       <c r="P59" s="89" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="Q59" s="89">
         <v>-1</v>
@@ -20017,7 +20014,7 @@
       </c>
       <c r="S59" s="398"/>
       <c r="T59" s="81" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="U59" s="81">
         <v>1</v>
@@ -20027,7 +20024,7 @@
       </c>
       <c r="W59" s="81"/>
       <c r="X59" s="396" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="Y59" s="396">
         <v>16</v>
@@ -20037,7 +20034,7 @@
       </c>
       <c r="AA59" s="396"/>
       <c r="AB59" s="81" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="AC59" s="81">
         <v>31</v>
@@ -20047,7 +20044,7 @@
       </c>
       <c r="AE59" s="81"/>
       <c r="AF59" s="396" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="AG59" s="396">
         <v>46</v>
@@ -20057,7 +20054,7 @@
       </c>
       <c r="AI59" s="396"/>
       <c r="AJ59" s="81" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="AK59" s="81">
         <v>61</v>
@@ -20067,7 +20064,7 @@
       </c>
       <c r="AM59" s="81"/>
       <c r="AN59" s="396" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="AO59" s="396">
         <v>76</v>
@@ -20151,7 +20148,7 @@
         <v>90</v>
       </c>
       <c r="P60" s="89" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="Q60" s="89">
         <v>-1</v>
@@ -20161,7 +20158,7 @@
       </c>
       <c r="S60" s="398"/>
       <c r="T60" s="81" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="U60" s="81">
         <v>1</v>
@@ -20171,7 +20168,7 @@
       </c>
       <c r="W60" s="81"/>
       <c r="X60" s="396" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="Y60" s="396">
         <v>16</v>
@@ -20181,7 +20178,7 @@
       </c>
       <c r="AA60" s="396"/>
       <c r="AB60" s="81" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="AC60" s="81">
         <v>31</v>
@@ -20191,7 +20188,7 @@
       </c>
       <c r="AE60" s="81"/>
       <c r="AF60" s="396" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="AG60" s="396">
         <v>46</v>
@@ -20201,7 +20198,7 @@
       </c>
       <c r="AI60" s="396"/>
       <c r="AJ60" s="81" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="AK60" s="81">
         <v>61</v>
@@ -20211,7 +20208,7 @@
       </c>
       <c r="AM60" s="81"/>
       <c r="AN60" s="396" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="AO60" s="396">
         <v>76</v>
@@ -20295,7 +20292,7 @@
         <v>45</v>
       </c>
       <c r="P61" s="89" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="Q61" s="89">
         <v>-1</v>
@@ -20317,7 +20314,7 @@
         <v>0.45</v>
       </c>
       <c r="X61" s="396" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="Y61" s="396">
         <f>U61+W61+0.2</f>
@@ -20328,7 +20325,7 @@
       </c>
       <c r="AA61" s="396"/>
       <c r="AB61" s="81" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="AC61" s="81">
         <v>30</v>
@@ -34355,7 +34352,7 @@
         <v>1</v>
       </c>
       <c r="D179" s="79" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="E179" s="81">
         <f t="shared" si="72"/>
@@ -34395,7 +34392,7 @@
         <v>40</v>
       </c>
       <c r="P179" s="89" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="Q179" s="89">
         <v>-1</v>
@@ -34405,7 +34402,7 @@
       </c>
       <c r="S179" s="89"/>
       <c r="T179" s="81" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="U179" s="81">
         <v>1</v>
@@ -34415,7 +34412,7 @@
       </c>
       <c r="W179" s="81"/>
       <c r="X179" s="89" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="Y179" s="89">
         <v>16</v>
@@ -34425,7 +34422,7 @@
       </c>
       <c r="AA179" s="89"/>
       <c r="AB179" s="81" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="AC179" s="81">
         <v>31</v>
@@ -34470,7 +34467,7 @@
         <v>1</v>
       </c>
       <c r="D180" s="79" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="E180" s="81">
         <f t="shared" si="72"/>
@@ -34510,7 +34507,7 @@
         <v>20</v>
       </c>
       <c r="P180" s="89" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="Q180" s="89">
         <v>-1</v>
@@ -34520,7 +34517,7 @@
       </c>
       <c r="S180" s="89"/>
       <c r="T180" s="81" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="U180" s="81">
         <v>1</v>
@@ -34530,7 +34527,7 @@
       </c>
       <c r="W180" s="81"/>
       <c r="X180" s="89" t="s">
-        <v>920</v>
+        <v>943</v>
       </c>
       <c r="Y180" s="89">
         <v>16</v>
@@ -34573,7 +34570,7 @@
         <v>1</v>
       </c>
       <c r="D181" s="79" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="E181" s="81">
         <f t="shared" si="72"/>
@@ -34705,7 +34702,7 @@
         <v>1</v>
       </c>
       <c r="D182" s="79" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="E182" s="81">
         <f t="shared" si="72"/>
@@ -34838,7 +34835,7 @@
         <v>1</v>
       </c>
       <c r="D183" s="79" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="E183" s="81">
         <f t="shared" si="72"/>
@@ -35159,7 +35156,7 @@
       <c r="O218" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:BK178" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A2:BK183" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <mergeCells count="15">
     <mergeCell ref="BL1:BO1"/>
     <mergeCell ref="A1:D1"/>
@@ -35306,96 +35303,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:94" x14ac:dyDescent="0.4">
-      <c r="A1" s="400" t="s">
+      <c r="A1" s="399" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="400"/>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="401" t="s">
+      <c r="B1" s="399"/>
+      <c r="C1" s="399"/>
+      <c r="D1" s="399"/>
+      <c r="E1" s="400" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="402"/>
-      <c r="I1" s="402"/>
-      <c r="J1" s="402"/>
-      <c r="K1" s="402"/>
-      <c r="L1" s="402"/>
-      <c r="M1" s="402"/>
-      <c r="N1" s="403"/>
-      <c r="O1" s="414" t="s">
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="401"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="402"/>
+      <c r="O1" s="406" t="s">
         <v>77</v>
       </c>
-      <c r="P1" s="415"/>
-      <c r="Q1" s="415"/>
-      <c r="R1" s="416"/>
-      <c r="S1" s="401" t="s">
+      <c r="P1" s="407"/>
+      <c r="Q1" s="407"/>
+      <c r="R1" s="408"/>
+      <c r="S1" s="400" t="s">
         <v>78</v>
       </c>
-      <c r="T1" s="402"/>
-      <c r="U1" s="402"/>
-      <c r="V1" s="402"/>
-      <c r="W1" s="414" t="s">
+      <c r="T1" s="401"/>
+      <c r="U1" s="401"/>
+      <c r="V1" s="401"/>
+      <c r="W1" s="406" t="s">
         <v>79</v>
       </c>
-      <c r="X1" s="415"/>
-      <c r="Y1" s="415"/>
-      <c r="Z1" s="416"/>
-      <c r="AA1" s="411" t="s">
+      <c r="X1" s="407"/>
+      <c r="Y1" s="407"/>
+      <c r="Z1" s="408"/>
+      <c r="AA1" s="403" t="s">
         <v>80</v>
       </c>
-      <c r="AB1" s="412"/>
-      <c r="AC1" s="412"/>
-      <c r="AD1" s="413"/>
-      <c r="AE1" s="414" t="s">
+      <c r="AB1" s="404"/>
+      <c r="AC1" s="404"/>
+      <c r="AD1" s="405"/>
+      <c r="AE1" s="406" t="s">
         <v>81</v>
       </c>
-      <c r="AF1" s="415"/>
-      <c r="AG1" s="415"/>
-      <c r="AH1" s="416"/>
-      <c r="AI1" s="411" t="s">
+      <c r="AF1" s="407"/>
+      <c r="AG1" s="407"/>
+      <c r="AH1" s="408"/>
+      <c r="AI1" s="403" t="s">
         <v>82</v>
       </c>
-      <c r="AJ1" s="412"/>
-      <c r="AK1" s="412"/>
-      <c r="AL1" s="413"/>
-      <c r="AM1" s="414" t="s">
+      <c r="AJ1" s="404"/>
+      <c r="AK1" s="404"/>
+      <c r="AL1" s="405"/>
+      <c r="AM1" s="406" t="s">
         <v>83</v>
       </c>
-      <c r="AN1" s="415"/>
-      <c r="AO1" s="415"/>
-      <c r="AP1" s="416"/>
-      <c r="AQ1" s="411" t="s">
+      <c r="AN1" s="407"/>
+      <c r="AO1" s="407"/>
+      <c r="AP1" s="408"/>
+      <c r="AQ1" s="403" t="s">
         <v>84</v>
       </c>
-      <c r="AR1" s="412"/>
-      <c r="AS1" s="412"/>
-      <c r="AT1" s="413"/>
-      <c r="AU1" s="414" t="s">
+      <c r="AR1" s="404"/>
+      <c r="AS1" s="404"/>
+      <c r="AT1" s="405"/>
+      <c r="AU1" s="406" t="s">
         <v>85</v>
       </c>
-      <c r="AV1" s="415"/>
-      <c r="AW1" s="415"/>
-      <c r="AX1" s="416"/>
-      <c r="AY1" s="411" t="s">
+      <c r="AV1" s="407"/>
+      <c r="AW1" s="407"/>
+      <c r="AX1" s="408"/>
+      <c r="AY1" s="403" t="s">
         <v>86</v>
       </c>
-      <c r="AZ1" s="412"/>
-      <c r="BA1" s="412"/>
-      <c r="BB1" s="413"/>
-      <c r="BC1" s="414" t="s">
+      <c r="AZ1" s="404"/>
+      <c r="BA1" s="404"/>
+      <c r="BB1" s="405"/>
+      <c r="BC1" s="406" t="s">
         <v>87</v>
       </c>
-      <c r="BD1" s="415"/>
-      <c r="BE1" s="415"/>
-      <c r="BF1" s="416"/>
-      <c r="BG1" s="411" t="s">
+      <c r="BD1" s="407"/>
+      <c r="BE1" s="407"/>
+      <c r="BF1" s="408"/>
+      <c r="BG1" s="403" t="s">
         <v>88</v>
       </c>
-      <c r="BH1" s="412"/>
-      <c r="BI1" s="412"/>
-      <c r="BJ1" s="413"/>
+      <c r="BH1" s="404"/>
+      <c r="BI1" s="404"/>
+      <c r="BJ1" s="405"/>
     </row>
     <row r="2" spans="1:94" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -40067,7 +40064,7 @@
         <v>45</v>
       </c>
       <c r="O45" s="122" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="P45" s="122">
         <v>-1</v>
@@ -40077,7 +40074,7 @@
       </c>
       <c r="R45" s="122"/>
       <c r="S45" s="24" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="T45" s="24">
         <v>0</v>
@@ -40087,7 +40084,7 @@
       </c>
       <c r="V45" s="24"/>
       <c r="W45" s="122" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="X45" s="122">
         <v>1</v>
@@ -40097,7 +40094,7 @@
       </c>
       <c r="Z45" s="122"/>
       <c r="AA45" s="24" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AB45" s="24">
         <v>16</v>
@@ -40107,7 +40104,7 @@
       </c>
       <c r="AD45" s="24"/>
       <c r="AE45" s="122" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AF45" s="122">
         <v>31</v>
@@ -40117,7 +40114,7 @@
       </c>
       <c r="AH45" s="122"/>
       <c r="AI45" s="24" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AJ45" s="24">
         <v>46</v>
@@ -40127,7 +40124,7 @@
       </c>
       <c r="AL45" s="24"/>
       <c r="AM45" s="122" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AN45" s="122">
         <v>61</v>
@@ -40137,7 +40134,7 @@
       </c>
       <c r="AP45" s="122"/>
       <c r="AQ45" s="24" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AR45" s="24">
         <v>76</v>
@@ -40210,7 +40207,7 @@
         <v>45</v>
       </c>
       <c r="O46" s="122" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="P46" s="122">
         <v>-1</v>
@@ -40220,7 +40217,7 @@
       </c>
       <c r="R46" s="122"/>
       <c r="S46" s="24" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="T46" s="24">
         <v>0</v>
@@ -40242,7 +40239,7 @@
         <v>0.45</v>
       </c>
       <c r="AA46" s="24" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AB46" s="24">
         <f>X46+Z46+0.2</f>
@@ -40253,7 +40250,7 @@
       </c>
       <c r="AD46" s="24"/>
       <c r="AE46" s="122" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AF46" s="122">
         <v>30</v>
@@ -45222,7 +45219,7 @@
         <v>1</v>
       </c>
       <c r="D89" s="118" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="E89" s="5">
         <f t="shared" si="29"/>
@@ -45258,7 +45255,7 @@
         <v>40</v>
       </c>
       <c r="O89" s="122" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="P89" s="122">
         <v>-1</v>
@@ -45268,7 +45265,7 @@
       </c>
       <c r="R89" s="122"/>
       <c r="S89" s="24" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="T89" s="24">
         <v>0</v>
@@ -45278,7 +45275,7 @@
       </c>
       <c r="V89" s="24"/>
       <c r="W89" s="122" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="X89" s="122">
         <v>1</v>
@@ -45288,7 +45285,7 @@
       </c>
       <c r="Z89" s="122"/>
       <c r="AA89" s="24" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AB89" s="24">
         <v>16</v>
@@ -45298,7 +45295,7 @@
       </c>
       <c r="AD89" s="24"/>
       <c r="AE89" s="122" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AF89" s="122">
         <v>31</v>
@@ -45320,7 +45317,7 @@
         <v>1</v>
       </c>
       <c r="D90" s="118" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="E90" s="5">
         <f t="shared" si="29"/>
@@ -45356,7 +45353,7 @@
         <v>40</v>
       </c>
       <c r="O90" s="122" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="P90" s="122">
         <v>-1</v>
@@ -45366,7 +45363,7 @@
       </c>
       <c r="R90" s="122"/>
       <c r="S90" s="24" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="T90" s="24">
         <v>1</v>
@@ -45376,7 +45373,7 @@
       </c>
       <c r="V90" s="24"/>
       <c r="W90" s="122" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="X90" s="122">
         <v>1</v>
@@ -45386,7 +45383,7 @@
       </c>
       <c r="Z90" s="122"/>
       <c r="AA90" s="24" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AB90" s="24">
         <v>10</v>
@@ -45396,7 +45393,7 @@
       </c>
       <c r="AD90" s="24"/>
       <c r="AE90" s="122" t="s">
-        <v>920</v>
+        <v>944</v>
       </c>
       <c r="AF90" s="122">
         <v>25</v>
@@ -45678,7 +45675,7 @@
       <c r="BJ180" s="68"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:BJ2" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A2:BJ90" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <mergeCells count="14">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:N1"/>
@@ -45809,97 +45806,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:63" x14ac:dyDescent="0.4">
-      <c r="A1" s="400" t="s">
+      <c r="A1" s="399" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="400"/>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="401" t="s">
+      <c r="B1" s="399"/>
+      <c r="C1" s="399"/>
+      <c r="D1" s="399"/>
+      <c r="E1" s="400" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="402"/>
-      <c r="I1" s="402"/>
-      <c r="J1" s="402"/>
-      <c r="K1" s="402"/>
-      <c r="L1" s="402"/>
-      <c r="M1" s="402"/>
-      <c r="N1" s="402"/>
-      <c r="O1" s="403"/>
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="401"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="401"/>
+      <c r="O1" s="402"/>
       <c r="P1" s="417" t="s">
         <v>77</v>
       </c>
       <c r="Q1" s="417"/>
       <c r="R1" s="417"/>
       <c r="S1" s="417"/>
-      <c r="T1" s="400" t="s">
+      <c r="T1" s="399" t="s">
         <v>78</v>
       </c>
-      <c r="U1" s="400"/>
-      <c r="V1" s="400"/>
-      <c r="W1" s="400"/>
+      <c r="U1" s="399"/>
+      <c r="V1" s="399"/>
+      <c r="W1" s="399"/>
       <c r="X1" s="417" t="s">
         <v>79</v>
       </c>
       <c r="Y1" s="417"/>
       <c r="Z1" s="417"/>
       <c r="AA1" s="417"/>
-      <c r="AB1" s="400" t="s">
+      <c r="AB1" s="399" t="s">
         <v>80</v>
       </c>
-      <c r="AC1" s="400"/>
-      <c r="AD1" s="400"/>
-      <c r="AE1" s="400"/>
+      <c r="AC1" s="399"/>
+      <c r="AD1" s="399"/>
+      <c r="AE1" s="399"/>
       <c r="AF1" s="417" t="s">
         <v>81</v>
       </c>
       <c r="AG1" s="417"/>
       <c r="AH1" s="417"/>
       <c r="AI1" s="417"/>
-      <c r="AJ1" s="400" t="s">
+      <c r="AJ1" s="399" t="s">
         <v>82</v>
       </c>
-      <c r="AK1" s="400"/>
-      <c r="AL1" s="400"/>
-      <c r="AM1" s="400"/>
+      <c r="AK1" s="399"/>
+      <c r="AL1" s="399"/>
+      <c r="AM1" s="399"/>
       <c r="AN1" s="417" t="s">
         <v>83</v>
       </c>
       <c r="AO1" s="417"/>
       <c r="AP1" s="417"/>
       <c r="AQ1" s="417"/>
-      <c r="AR1" s="400" t="s">
+      <c r="AR1" s="399" t="s">
         <v>84</v>
       </c>
-      <c r="AS1" s="400"/>
-      <c r="AT1" s="400"/>
-      <c r="AU1" s="400"/>
+      <c r="AS1" s="399"/>
+      <c r="AT1" s="399"/>
+      <c r="AU1" s="399"/>
       <c r="AV1" s="417" t="s">
         <v>85</v>
       </c>
       <c r="AW1" s="417"/>
       <c r="AX1" s="417"/>
       <c r="AY1" s="417"/>
-      <c r="AZ1" s="400" t="s">
+      <c r="AZ1" s="399" t="s">
         <v>86</v>
       </c>
-      <c r="BA1" s="400"/>
-      <c r="BB1" s="400"/>
-      <c r="BC1" s="400"/>
+      <c r="BA1" s="399"/>
+      <c r="BB1" s="399"/>
+      <c r="BC1" s="399"/>
       <c r="BD1" s="417" t="s">
         <v>87</v>
       </c>
       <c r="BE1" s="417"/>
       <c r="BF1" s="417"/>
       <c r="BG1" s="417"/>
-      <c r="BH1" s="400" t="s">
+      <c r="BH1" s="399" t="s">
         <v>88</v>
       </c>
-      <c r="BI1" s="400"/>
-      <c r="BJ1" s="400"/>
-      <c r="BK1" s="400"/>
+      <c r="BI1" s="399"/>
+      <c r="BJ1" s="399"/>
+      <c r="BK1" s="399"/>
     </row>
     <row r="2" spans="1:63" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -55207,109 +55204,109 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:73" x14ac:dyDescent="0.4">
-      <c r="A1" s="400" t="s">
+      <c r="A1" s="399" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="400"/>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="401" t="s">
+      <c r="B1" s="399"/>
+      <c r="C1" s="399"/>
+      <c r="D1" s="399"/>
+      <c r="E1" s="400" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="402"/>
-      <c r="I1" s="402"/>
-      <c r="J1" s="402"/>
-      <c r="K1" s="402"/>
-      <c r="L1" s="402"/>
-      <c r="M1" s="402"/>
-      <c r="N1" s="402"/>
-      <c r="O1" s="402"/>
-      <c r="P1" s="402"/>
-      <c r="Q1" s="402"/>
-      <c r="R1" s="402"/>
-      <c r="S1" s="402"/>
-      <c r="T1" s="402"/>
-      <c r="U1" s="403"/>
-      <c r="V1" s="399" t="s">
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="401"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="401"/>
+      <c r="O1" s="401"/>
+      <c r="P1" s="401"/>
+      <c r="Q1" s="401"/>
+      <c r="R1" s="401"/>
+      <c r="S1" s="401"/>
+      <c r="T1" s="401"/>
+      <c r="U1" s="402"/>
+      <c r="V1" s="416" t="s">
         <v>77</v>
       </c>
-      <c r="W1" s="399"/>
-      <c r="X1" s="399"/>
-      <c r="Y1" s="399"/>
-      <c r="Z1" s="400" t="s">
+      <c r="W1" s="416"/>
+      <c r="X1" s="416"/>
+      <c r="Y1" s="416"/>
+      <c r="Z1" s="399" t="s">
         <v>78</v>
       </c>
-      <c r="AA1" s="400"/>
-      <c r="AB1" s="400"/>
-      <c r="AC1" s="400"/>
-      <c r="AD1" s="399" t="s">
+      <c r="AA1" s="399"/>
+      <c r="AB1" s="399"/>
+      <c r="AC1" s="399"/>
+      <c r="AD1" s="416" t="s">
         <v>79</v>
       </c>
-      <c r="AE1" s="399"/>
-      <c r="AF1" s="399"/>
-      <c r="AG1" s="399"/>
-      <c r="AH1" s="400" t="s">
+      <c r="AE1" s="416"/>
+      <c r="AF1" s="416"/>
+      <c r="AG1" s="416"/>
+      <c r="AH1" s="399" t="s">
         <v>80</v>
       </c>
-      <c r="AI1" s="400"/>
-      <c r="AJ1" s="400"/>
-      <c r="AK1" s="400"/>
-      <c r="AL1" s="399" t="s">
+      <c r="AI1" s="399"/>
+      <c r="AJ1" s="399"/>
+      <c r="AK1" s="399"/>
+      <c r="AL1" s="416" t="s">
         <v>81</v>
       </c>
-      <c r="AM1" s="399"/>
-      <c r="AN1" s="399"/>
-      <c r="AO1" s="399"/>
-      <c r="AP1" s="400" t="s">
+      <c r="AM1" s="416"/>
+      <c r="AN1" s="416"/>
+      <c r="AO1" s="416"/>
+      <c r="AP1" s="399" t="s">
         <v>82</v>
       </c>
-      <c r="AQ1" s="400"/>
-      <c r="AR1" s="400"/>
-      <c r="AS1" s="400"/>
-      <c r="AT1" s="399" t="s">
+      <c r="AQ1" s="399"/>
+      <c r="AR1" s="399"/>
+      <c r="AS1" s="399"/>
+      <c r="AT1" s="416" t="s">
         <v>83</v>
       </c>
-      <c r="AU1" s="399"/>
-      <c r="AV1" s="399"/>
-      <c r="AW1" s="399"/>
-      <c r="AX1" s="400" t="s">
+      <c r="AU1" s="416"/>
+      <c r="AV1" s="416"/>
+      <c r="AW1" s="416"/>
+      <c r="AX1" s="399" t="s">
         <v>84</v>
       </c>
-      <c r="AY1" s="400"/>
-      <c r="AZ1" s="400"/>
-      <c r="BA1" s="400"/>
-      <c r="BB1" s="399" t="s">
+      <c r="AY1" s="399"/>
+      <c r="AZ1" s="399"/>
+      <c r="BA1" s="399"/>
+      <c r="BB1" s="416" t="s">
         <v>85</v>
       </c>
-      <c r="BC1" s="399"/>
-      <c r="BD1" s="399"/>
-      <c r="BE1" s="399"/>
-      <c r="BF1" s="400" t="s">
+      <c r="BC1" s="416"/>
+      <c r="BD1" s="416"/>
+      <c r="BE1" s="416"/>
+      <c r="BF1" s="399" t="s">
         <v>86</v>
       </c>
-      <c r="BG1" s="400"/>
-      <c r="BH1" s="400"/>
-      <c r="BI1" s="400"/>
-      <c r="BJ1" s="399" t="s">
+      <c r="BG1" s="399"/>
+      <c r="BH1" s="399"/>
+      <c r="BI1" s="399"/>
+      <c r="BJ1" s="416" t="s">
         <v>87</v>
       </c>
-      <c r="BK1" s="399"/>
-      <c r="BL1" s="399"/>
-      <c r="BM1" s="399"/>
-      <c r="BN1" s="400" t="s">
+      <c r="BK1" s="416"/>
+      <c r="BL1" s="416"/>
+      <c r="BM1" s="416"/>
+      <c r="BN1" s="399" t="s">
         <v>88</v>
       </c>
-      <c r="BO1" s="400"/>
-      <c r="BP1" s="400"/>
-      <c r="BQ1" s="400"/>
-      <c r="BR1" s="399" t="s">
+      <c r="BO1" s="399"/>
+      <c r="BP1" s="399"/>
+      <c r="BQ1" s="399"/>
+      <c r="BR1" s="416" t="s">
         <v>495</v>
       </c>
-      <c r="BS1" s="399"/>
-      <c r="BT1" s="399"/>
-      <c r="BU1" s="399"/>
+      <c r="BS1" s="416"/>
+      <c r="BT1" s="416"/>
+      <c r="BU1" s="416"/>
     </row>
     <row r="2" spans="1:73" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -68351,6 +68348,12 @@
   </sheetData>
   <autoFilter ref="A2:BQ178" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="15">
+    <mergeCell ref="AH1:AK1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:U1"/>
+    <mergeCell ref="V1:Y1"/>
+    <mergeCell ref="Z1:AC1"/>
+    <mergeCell ref="AD1:AG1"/>
     <mergeCell ref="BJ1:BM1"/>
     <mergeCell ref="BN1:BQ1"/>
     <mergeCell ref="BR1:BU1"/>
@@ -68360,12 +68363,6 @@
     <mergeCell ref="AX1:BA1"/>
     <mergeCell ref="BB1:BE1"/>
     <mergeCell ref="BF1:BI1"/>
-    <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:U1"/>
-    <mergeCell ref="V1:Y1"/>
-    <mergeCell ref="Z1:AC1"/>
-    <mergeCell ref="AD1:AG1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -68495,97 +68492,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:63" x14ac:dyDescent="0.4">
-      <c r="A1" s="400" t="s">
+      <c r="A1" s="399" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="400"/>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="401" t="s">
+      <c r="B1" s="399"/>
+      <c r="C1" s="399"/>
+      <c r="D1" s="399"/>
+      <c r="E1" s="400" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="402"/>
-      <c r="I1" s="402"/>
-      <c r="J1" s="402"/>
-      <c r="K1" s="402"/>
-      <c r="L1" s="402"/>
-      <c r="M1" s="402"/>
-      <c r="N1" s="402"/>
-      <c r="O1" s="403"/>
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="401"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="401"/>
+      <c r="O1" s="402"/>
       <c r="P1" s="417" t="s">
         <v>77</v>
       </c>
       <c r="Q1" s="417"/>
       <c r="R1" s="417"/>
       <c r="S1" s="417"/>
-      <c r="T1" s="401" t="s">
+      <c r="T1" s="400" t="s">
         <v>78</v>
       </c>
-      <c r="U1" s="402"/>
-      <c r="V1" s="402"/>
-      <c r="W1" s="402"/>
+      <c r="U1" s="401"/>
+      <c r="V1" s="401"/>
+      <c r="W1" s="401"/>
       <c r="X1" s="417" t="s">
         <v>79</v>
       </c>
       <c r="Y1" s="417"/>
       <c r="Z1" s="417"/>
       <c r="AA1" s="417"/>
-      <c r="AB1" s="401" t="s">
+      <c r="AB1" s="400" t="s">
         <v>80</v>
       </c>
-      <c r="AC1" s="402"/>
-      <c r="AD1" s="402"/>
-      <c r="AE1" s="402"/>
+      <c r="AC1" s="401"/>
+      <c r="AD1" s="401"/>
+      <c r="AE1" s="401"/>
       <c r="AF1" s="417" t="s">
         <v>81</v>
       </c>
       <c r="AG1" s="417"/>
       <c r="AH1" s="417"/>
       <c r="AI1" s="417"/>
-      <c r="AJ1" s="401" t="s">
+      <c r="AJ1" s="400" t="s">
         <v>82</v>
       </c>
-      <c r="AK1" s="402"/>
-      <c r="AL1" s="402"/>
-      <c r="AM1" s="402"/>
+      <c r="AK1" s="401"/>
+      <c r="AL1" s="401"/>
+      <c r="AM1" s="401"/>
       <c r="AN1" s="417" t="s">
         <v>83</v>
       </c>
       <c r="AO1" s="417"/>
       <c r="AP1" s="417"/>
       <c r="AQ1" s="417"/>
-      <c r="AR1" s="401" t="s">
+      <c r="AR1" s="400" t="s">
         <v>84</v>
       </c>
-      <c r="AS1" s="402"/>
-      <c r="AT1" s="402"/>
-      <c r="AU1" s="402"/>
+      <c r="AS1" s="401"/>
+      <c r="AT1" s="401"/>
+      <c r="AU1" s="401"/>
       <c r="AV1" s="417" t="s">
         <v>85</v>
       </c>
       <c r="AW1" s="417"/>
       <c r="AX1" s="417"/>
       <c r="AY1" s="417"/>
-      <c r="AZ1" s="401" t="s">
+      <c r="AZ1" s="400" t="s">
         <v>86</v>
       </c>
-      <c r="BA1" s="402"/>
-      <c r="BB1" s="402"/>
-      <c r="BC1" s="402"/>
+      <c r="BA1" s="401"/>
+      <c r="BB1" s="401"/>
+      <c r="BC1" s="401"/>
       <c r="BD1" s="417" t="s">
         <v>87</v>
       </c>
       <c r="BE1" s="417"/>
       <c r="BF1" s="417"/>
       <c r="BG1" s="417"/>
-      <c r="BH1" s="401" t="s">
+      <c r="BH1" s="400" t="s">
         <v>88</v>
       </c>
-      <c r="BI1" s="402"/>
-      <c r="BJ1" s="402"/>
-      <c r="BK1" s="402"/>
+      <c r="BI1" s="401"/>
+      <c r="BJ1" s="401"/>
+      <c r="BK1" s="401"/>
     </row>
     <row r="2" spans="1:63" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -76167,13 +76164,13 @@
     </row>
     <row r="34" spans="1:6" s="123" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="382" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="B34" s="383" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="C34" s="382" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="D34" s="382" t="s">
         <v>166</v>
@@ -76187,13 +76184,13 @@
     </row>
     <row r="35" spans="1:6" s="123" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="382" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="B35" s="383" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="C35" s="382" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="D35" s="382" t="s">
         <v>166</v>
@@ -76897,7 +76894,7 @@
       </c>
       <c r="C19" s="419"/>
       <c r="D19" s="139" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
@@ -77371,10 +77368,10 @@
         <v>728</v>
       </c>
       <c r="C58" s="418" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="D58" s="146" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="29.15" x14ac:dyDescent="0.4">
@@ -77386,7 +77383,7 @@
       </c>
       <c r="C59" s="419"/>
       <c r="D59" s="238" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="87.9" thickBot="1" x14ac:dyDescent="0.45">
@@ -77534,7 +77531,7 @@
         <v>406</v>
       </c>
       <c r="D71" s="146" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.4">
@@ -77750,7 +77747,7 @@
       </c>
       <c r="C89" s="419"/>
       <c r="D89" s="139" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.4">
@@ -78826,13 +78823,13 @@
         <v>177</v>
       </c>
       <c r="B178" s="194" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="C178" s="418" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="D178" s="146" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="179" spans="1:4" ht="29.6" thickBot="1" x14ac:dyDescent="0.45">
@@ -78840,11 +78837,11 @@
         <v>178</v>
       </c>
       <c r="B179" s="150" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="C179" s="420"/>
       <c r="D179" s="143" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.4">
@@ -78852,13 +78849,13 @@
         <v>179</v>
       </c>
       <c r="B180" s="393" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="C180" s="418" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="D180" s="146" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.4">
@@ -78866,11 +78863,11 @@
         <v>180</v>
       </c>
       <c r="B181" s="134" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="C181" s="419"/>
       <c r="D181" s="270" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="182" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
@@ -78878,23 +78875,16 @@
         <v>181</v>
       </c>
       <c r="B182" s="394" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="C182" s="420"/>
       <c r="D182" s="143" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="16">
-    <mergeCell ref="C58:C60"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="C2:C11"/>
-    <mergeCell ref="C12:C17"/>
-    <mergeCell ref="C18:C28"/>
-    <mergeCell ref="C44:C53"/>
-    <mergeCell ref="C29:C43"/>
     <mergeCell ref="C180:C182"/>
     <mergeCell ref="C178:C179"/>
     <mergeCell ref="C163:C176"/>
@@ -78904,6 +78894,13 @@
     <mergeCell ref="C99:C108"/>
     <mergeCell ref="C109:C115"/>
     <mergeCell ref="C116:C162"/>
+    <mergeCell ref="C58:C60"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="C2:C11"/>
+    <mergeCell ref="C12:C17"/>
+    <mergeCell ref="C18:C28"/>
+    <mergeCell ref="C44:C53"/>
+    <mergeCell ref="C29:C43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -78911,14 +78908,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="107e75b3-53cc-4838-92d2-ebc011bd4832">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="888ccf44-0d39-41a2-ab17-f7efb2bf6977" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -79171,27 +79166,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="107e75b3-53cc-4838-92d2-ebc011bd4832">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="888ccf44-0d39-41a2-ab17-f7efb2bf6977" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2288FB7-E85A-4FE8-9E7A-FE572FF16064}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74B21D61-7BBD-4BD3-A9A5-1E8F98F2F686}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="107e75b3-53cc-4838-92d2-ebc011bd4832"/>
-    <ds:schemaRef ds:uri="888ccf44-0d39-41a2-ab17-f7efb2bf6977"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -79216,9 +79204,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74B21D61-7BBD-4BD3-A9A5-1E8F98F2F686}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2288FB7-E85A-4FE8-9E7A-FE572FF16064}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="107e75b3-53cc-4838-92d2-ebc011bd4832"/>
+    <ds:schemaRef ds:uri="888ccf44-0d39-41a2-ab17-f7efb2bf6977"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix DCC testcase 1043's Simulationtime to 90 s
</commit_message>
<xml_diff>
--- a/testcases.xlsx
+++ b/testcases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://energinet-my.sharepoint.com/personal/prw_energinet_dk/Documents/Dokumenter/GitHub/MTB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="11_710D79F8E8F49B720F18F8F5A5BEAA4096265349" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D68397F5-7546-4295-817C-D589CC648AF5}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="11_710D79F8E8F49B720F18F8F5A5BEAA4096265349" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A65F2381-AA06-4215-A715-A4C5EA7B4ECF}"/>
   <bookViews>
-    <workbookView xWindow="-16935" yWindow="-21720" windowWidth="38640" windowHeight="21120" tabRatio="822" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16935" yWindow="-21720" windowWidth="38640" windowHeight="21120" tabRatio="822" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="29" r:id="rId1"/>
@@ -5781,6 +5781,9 @@
     <xf numFmtId="164" fontId="7" fillId="8" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5791,24 +5794,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5832,7 +5817,22 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5856,17 +5856,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -6423,16 +6423,16 @@
         <v>322</v>
       </c>
       <c r="G3" s="124"/>
-      <c r="H3" s="409" t="s">
+      <c r="H3" s="404" t="s">
         <v>339</v>
       </c>
-      <c r="I3" s="409"/>
-      <c r="J3" s="409"/>
-      <c r="K3" s="409" t="s">
+      <c r="I3" s="404"/>
+      <c r="J3" s="404"/>
+      <c r="K3" s="404" t="s">
         <v>340</v>
       </c>
-      <c r="L3" s="409"/>
-      <c r="M3" s="410"/>
+      <c r="L3" s="404"/>
+      <c r="M3" s="405"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4" s="248" t="s">
@@ -9411,102 +9411,102 @@
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="333"/>
       <c r="B2" s="333"/>
-      <c r="C2" s="426" t="s">
+      <c r="C2" s="424" t="s">
         <v>843</v>
       </c>
-      <c r="D2" s="424" t="s">
+      <c r="D2" s="426" t="s">
         <v>907</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="333"/>
       <c r="B3" s="333"/>
-      <c r="C3" s="426"/>
-      <c r="D3" s="424"/>
+      <c r="C3" s="424"/>
+      <c r="D3" s="426"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="333"/>
       <c r="B4" s="333"/>
-      <c r="C4" s="426"/>
-      <c r="D4" s="424"/>
+      <c r="C4" s="424"/>
+      <c r="D4" s="426"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="333"/>
       <c r="B5" s="333"/>
-      <c r="C5" s="426"/>
-      <c r="D5" s="424"/>
+      <c r="C5" s="424"/>
+      <c r="D5" s="426"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="333"/>
       <c r="B6" s="333"/>
-      <c r="C6" s="426"/>
-      <c r="D6" s="424"/>
+      <c r="C6" s="424"/>
+      <c r="D6" s="426"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="333"/>
       <c r="B7" s="333"/>
-      <c r="C7" s="426"/>
-      <c r="D7" s="424"/>
+      <c r="C7" s="424"/>
+      <c r="D7" s="426"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="333"/>
       <c r="B8" s="333"/>
-      <c r="C8" s="426"/>
-      <c r="D8" s="424"/>
+      <c r="C8" s="424"/>
+      <c r="D8" s="426"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="333"/>
       <c r="B9" s="333"/>
-      <c r="C9" s="426"/>
-      <c r="D9" s="424"/>
+      <c r="C9" s="424"/>
+      <c r="D9" s="426"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="333"/>
       <c r="B10" s="333"/>
-      <c r="C10" s="426"/>
-      <c r="D10" s="424"/>
+      <c r="C10" s="424"/>
+      <c r="D10" s="426"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="333"/>
       <c r="B11" s="333"/>
-      <c r="C11" s="426"/>
-      <c r="D11" s="424"/>
+      <c r="C11" s="424"/>
+      <c r="D11" s="426"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="333"/>
       <c r="B12" s="333"/>
-      <c r="C12" s="426"/>
-      <c r="D12" s="424"/>
+      <c r="C12" s="424"/>
+      <c r="D12" s="426"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="333"/>
       <c r="B13" s="333"/>
-      <c r="C13" s="426"/>
-      <c r="D13" s="424"/>
+      <c r="C13" s="424"/>
+      <c r="D13" s="426"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="333"/>
       <c r="B14" s="333"/>
-      <c r="C14" s="426"/>
-      <c r="D14" s="424"/>
+      <c r="C14" s="424"/>
+      <c r="D14" s="426"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="333"/>
       <c r="B15" s="333"/>
-      <c r="C15" s="426"/>
-      <c r="D15" s="424"/>
+      <c r="C15" s="424"/>
+      <c r="D15" s="426"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="333"/>
       <c r="B16" s="333"/>
-      <c r="C16" s="426"/>
-      <c r="D16" s="424"/>
+      <c r="C16" s="424"/>
+      <c r="D16" s="426"/>
     </row>
     <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A17" s="315"/>
       <c r="B17" s="315"/>
-      <c r="C17" s="427"/>
-      <c r="D17" s="425"/>
+      <c r="C17" s="425"/>
+      <c r="D17" s="427"/>
     </row>
     <row r="18" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="335"/>
@@ -9514,7 +9514,7 @@
       <c r="C18" s="419" t="s">
         <v>361</v>
       </c>
-      <c r="D18" s="424" t="s">
+      <c r="D18" s="426" t="s">
         <v>844</v>
       </c>
     </row>
@@ -9522,115 +9522,115 @@
       <c r="A19" s="335"/>
       <c r="B19" s="335"/>
       <c r="C19" s="419"/>
-      <c r="D19" s="424"/>
+      <c r="D19" s="426"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="335"/>
       <c r="B20" s="335"/>
       <c r="C20" s="419"/>
-      <c r="D20" s="424"/>
+      <c r="D20" s="426"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="335"/>
       <c r="B21" s="335"/>
       <c r="C21" s="419"/>
-      <c r="D21" s="424"/>
+      <c r="D21" s="426"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="335"/>
       <c r="B22" s="335"/>
       <c r="C22" s="419"/>
-      <c r="D22" s="424"/>
+      <c r="D22" s="426"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="335"/>
       <c r="B23" s="335"/>
       <c r="C23" s="419"/>
-      <c r="D23" s="424"/>
+      <c r="D23" s="426"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" s="335"/>
       <c r="B24" s="335"/>
       <c r="C24" s="419"/>
-      <c r="D24" s="424"/>
+      <c r="D24" s="426"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" s="335"/>
       <c r="B25" s="335"/>
       <c r="C25" s="419"/>
-      <c r="D25" s="424"/>
+      <c r="D25" s="426"/>
     </row>
     <row r="26" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="335"/>
       <c r="B26" s="335"/>
       <c r="C26" s="419"/>
-      <c r="D26" s="424"/>
+      <c r="D26" s="426"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="335"/>
       <c r="B27" s="335"/>
       <c r="C27" s="419"/>
-      <c r="D27" s="424"/>
+      <c r="D27" s="426"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="335"/>
       <c r="B28" s="335"/>
       <c r="C28" s="419"/>
-      <c r="D28" s="424"/>
+      <c r="D28" s="426"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="335"/>
       <c r="B29" s="335"/>
       <c r="C29" s="419"/>
-      <c r="D29" s="424"/>
+      <c r="D29" s="426"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="335"/>
       <c r="B30" s="335"/>
       <c r="C30" s="419"/>
-      <c r="D30" s="424"/>
+      <c r="D30" s="426"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="335"/>
       <c r="B31" s="335"/>
       <c r="C31" s="419"/>
-      <c r="D31" s="424"/>
+      <c r="D31" s="426"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="335"/>
       <c r="B32" s="335"/>
       <c r="C32" s="419"/>
-      <c r="D32" s="424"/>
+      <c r="D32" s="426"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="335"/>
       <c r="B33" s="335"/>
       <c r="C33" s="419"/>
-      <c r="D33" s="424"/>
+      <c r="D33" s="426"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="335"/>
       <c r="B34" s="335"/>
       <c r="C34" s="419"/>
-      <c r="D34" s="424"/>
+      <c r="D34" s="426"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="335"/>
       <c r="B35" s="335"/>
       <c r="C35" s="419"/>
-      <c r="D35" s="424"/>
+      <c r="D35" s="426"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="335"/>
       <c r="B36" s="335"/>
       <c r="C36" s="419"/>
-      <c r="D36" s="424"/>
+      <c r="D36" s="426"/>
     </row>
     <row r="37" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A37" s="316"/>
       <c r="B37" s="316"/>
       <c r="C37" s="420"/>
-      <c r="D37" s="425"/>
+      <c r="D37" s="427"/>
     </row>
     <row r="38" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="334"/>
@@ -9638,7 +9638,7 @@
       <c r="C38" s="419" t="s">
         <v>845</v>
       </c>
-      <c r="D38" s="424" t="s">
+      <c r="D38" s="426" t="s">
         <v>846</v>
       </c>
     </row>
@@ -9646,115 +9646,115 @@
       <c r="A39" s="334"/>
       <c r="B39" s="334"/>
       <c r="C39" s="419"/>
-      <c r="D39" s="424"/>
+      <c r="D39" s="426"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A40" s="334"/>
       <c r="B40" s="334"/>
       <c r="C40" s="419"/>
-      <c r="D40" s="424"/>
+      <c r="D40" s="426"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A41" s="334"/>
       <c r="B41" s="334"/>
       <c r="C41" s="419"/>
-      <c r="D41" s="424"/>
+      <c r="D41" s="426"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A42" s="334"/>
       <c r="B42" s="334"/>
       <c r="C42" s="419"/>
-      <c r="D42" s="424"/>
+      <c r="D42" s="426"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A43" s="334"/>
       <c r="B43" s="334"/>
       <c r="C43" s="419"/>
-      <c r="D43" s="424"/>
+      <c r="D43" s="426"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A44" s="334"/>
       <c r="B44" s="334"/>
       <c r="C44" s="419"/>
-      <c r="D44" s="424"/>
+      <c r="D44" s="426"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A45" s="334"/>
       <c r="B45" s="334"/>
       <c r="C45" s="419"/>
-      <c r="D45" s="424"/>
+      <c r="D45" s="426"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A46" s="334"/>
       <c r="B46" s="334"/>
       <c r="C46" s="419"/>
-      <c r="D46" s="424"/>
+      <c r="D46" s="426"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A47" s="334"/>
       <c r="B47" s="334"/>
       <c r="C47" s="419"/>
-      <c r="D47" s="424"/>
+      <c r="D47" s="426"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A48" s="334"/>
       <c r="B48" s="334"/>
       <c r="C48" s="419"/>
-      <c r="D48" s="424"/>
+      <c r="D48" s="426"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A49" s="334"/>
       <c r="B49" s="334"/>
       <c r="C49" s="419"/>
-      <c r="D49" s="424"/>
+      <c r="D49" s="426"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A50" s="334"/>
       <c r="B50" s="334"/>
       <c r="C50" s="419"/>
-      <c r="D50" s="424"/>
+      <c r="D50" s="426"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A51" s="334"/>
       <c r="B51" s="334"/>
       <c r="C51" s="419"/>
-      <c r="D51" s="424"/>
+      <c r="D51" s="426"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A52" s="334"/>
       <c r="B52" s="334"/>
       <c r="C52" s="419"/>
-      <c r="D52" s="424"/>
+      <c r="D52" s="426"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" s="334"/>
       <c r="B53" s="334"/>
       <c r="C53" s="419"/>
-      <c r="D53" s="424"/>
+      <c r="D53" s="426"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A54" s="334"/>
       <c r="B54" s="334"/>
       <c r="C54" s="419"/>
-      <c r="D54" s="424"/>
+      <c r="D54" s="426"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A55" s="334"/>
       <c r="B55" s="334"/>
       <c r="C55" s="419"/>
-      <c r="D55" s="424"/>
+      <c r="D55" s="426"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A56" s="334"/>
       <c r="B56" s="334"/>
       <c r="C56" s="419"/>
-      <c r="D56" s="424"/>
+      <c r="D56" s="426"/>
     </row>
     <row r="57" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A57" s="317"/>
       <c r="B57" s="317"/>
       <c r="C57" s="420"/>
-      <c r="D57" s="425"/>
+      <c r="D57" s="427"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A58" s="336"/>
@@ -9762,7 +9762,7 @@
       <c r="C58" s="419" t="s">
         <v>847</v>
       </c>
-      <c r="D58" s="424" t="s">
+      <c r="D58" s="426" t="s">
         <v>848</v>
       </c>
     </row>
@@ -9770,85 +9770,85 @@
       <c r="A59" s="336"/>
       <c r="B59" s="336"/>
       <c r="C59" s="419"/>
-      <c r="D59" s="424"/>
+      <c r="D59" s="426"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A60" s="336"/>
       <c r="B60" s="336"/>
       <c r="C60" s="419"/>
-      <c r="D60" s="424"/>
+      <c r="D60" s="426"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A61" s="336"/>
       <c r="B61" s="336"/>
       <c r="C61" s="419"/>
-      <c r="D61" s="424"/>
+      <c r="D61" s="426"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A62" s="336"/>
       <c r="B62" s="336"/>
       <c r="C62" s="419"/>
-      <c r="D62" s="424"/>
+      <c r="D62" s="426"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A63" s="336"/>
       <c r="B63" s="336"/>
       <c r="C63" s="419"/>
-      <c r="D63" s="424"/>
+      <c r="D63" s="426"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A64" s="336"/>
       <c r="B64" s="336"/>
       <c r="C64" s="419"/>
-      <c r="D64" s="424"/>
+      <c r="D64" s="426"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A65" s="336"/>
       <c r="B65" s="336"/>
       <c r="C65" s="419"/>
-      <c r="D65" s="424"/>
+      <c r="D65" s="426"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A66" s="336"/>
       <c r="B66" s="336"/>
       <c r="C66" s="419"/>
-      <c r="D66" s="424"/>
+      <c r="D66" s="426"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A67" s="336"/>
       <c r="B67" s="336"/>
       <c r="C67" s="419"/>
-      <c r="D67" s="424"/>
+      <c r="D67" s="426"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A68" s="336"/>
       <c r="B68" s="336"/>
       <c r="C68" s="419"/>
-      <c r="D68" s="424"/>
+      <c r="D68" s="426"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A69" s="336"/>
       <c r="B69" s="336"/>
       <c r="C69" s="419"/>
-      <c r="D69" s="424"/>
+      <c r="D69" s="426"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A70" s="336"/>
       <c r="B70" s="336"/>
       <c r="C70" s="419"/>
-      <c r="D70" s="424"/>
+      <c r="D70" s="426"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A71" s="336"/>
       <c r="B71" s="336"/>
       <c r="C71" s="419"/>
-      <c r="D71" s="424"/>
+      <c r="D71" s="426"/>
     </row>
     <row r="72" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A72" s="318"/>
       <c r="B72" s="318"/>
       <c r="C72" s="420"/>
-      <c r="D72" s="425"/>
+      <c r="D72" s="427"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A73" s="338"/>
@@ -9856,7 +9856,7 @@
       <c r="C73" s="419" t="s">
         <v>849</v>
       </c>
-      <c r="D73" s="424" t="s">
+      <c r="D73" s="426" t="s">
         <v>850</v>
       </c>
     </row>
@@ -9864,97 +9864,97 @@
       <c r="A74" s="338"/>
       <c r="B74" s="338"/>
       <c r="C74" s="419"/>
-      <c r="D74" s="424"/>
+      <c r="D74" s="426"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A75" s="338"/>
       <c r="B75" s="338"/>
       <c r="C75" s="419"/>
-      <c r="D75" s="424"/>
+      <c r="D75" s="426"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A76" s="338"/>
       <c r="B76" s="338"/>
       <c r="C76" s="419"/>
-      <c r="D76" s="424"/>
+      <c r="D76" s="426"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A77" s="338"/>
       <c r="B77" s="338"/>
       <c r="C77" s="419"/>
-      <c r="D77" s="424"/>
+      <c r="D77" s="426"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A78" s="338"/>
       <c r="B78" s="338"/>
       <c r="C78" s="419"/>
-      <c r="D78" s="424"/>
+      <c r="D78" s="426"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A79" s="338"/>
       <c r="B79" s="338"/>
       <c r="C79" s="419"/>
-      <c r="D79" s="424"/>
+      <c r="D79" s="426"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A80" s="338"/>
       <c r="B80" s="338"/>
       <c r="C80" s="419"/>
-      <c r="D80" s="424"/>
+      <c r="D80" s="426"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A81" s="338"/>
       <c r="B81" s="338"/>
       <c r="C81" s="419"/>
-      <c r="D81" s="424"/>
+      <c r="D81" s="426"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A82" s="338"/>
       <c r="B82" s="338"/>
       <c r="C82" s="419"/>
-      <c r="D82" s="424"/>
+      <c r="D82" s="426"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A83" s="338"/>
       <c r="B83" s="338"/>
       <c r="C83" s="419"/>
-      <c r="D83" s="424"/>
+      <c r="D83" s="426"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A84" s="338"/>
       <c r="B84" s="338"/>
       <c r="C84" s="419"/>
-      <c r="D84" s="424"/>
+      <c r="D84" s="426"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A85" s="338"/>
       <c r="B85" s="338"/>
       <c r="C85" s="419"/>
-      <c r="D85" s="424"/>
+      <c r="D85" s="426"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A86" s="338"/>
       <c r="B86" s="338"/>
       <c r="C86" s="419"/>
-      <c r="D86" s="424"/>
+      <c r="D86" s="426"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A87" s="338"/>
       <c r="B87" s="338"/>
       <c r="C87" s="419"/>
-      <c r="D87" s="424"/>
+      <c r="D87" s="426"/>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A88" s="338"/>
       <c r="B88" s="338"/>
       <c r="C88" s="419"/>
-      <c r="D88" s="424"/>
+      <c r="D88" s="426"/>
     </row>
     <row r="89" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A89" s="319"/>
       <c r="B89" s="319"/>
       <c r="C89" s="420"/>
-      <c r="D89" s="425"/>
+      <c r="D89" s="427"/>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A90" s="337"/>
@@ -9962,7 +9962,7 @@
       <c r="C90" s="419" t="s">
         <v>851</v>
       </c>
-      <c r="D90" s="424" t="s">
+      <c r="D90" s="426" t="s">
         <v>852</v>
       </c>
     </row>
@@ -9970,49 +9970,49 @@
       <c r="A91" s="337"/>
       <c r="B91" s="337"/>
       <c r="C91" s="419"/>
-      <c r="D91" s="424"/>
+      <c r="D91" s="426"/>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A92" s="337"/>
       <c r="B92" s="337"/>
       <c r="C92" s="419"/>
-      <c r="D92" s="424"/>
+      <c r="D92" s="426"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A93" s="337"/>
       <c r="B93" s="337"/>
       <c r="C93" s="419"/>
-      <c r="D93" s="424"/>
+      <c r="D93" s="426"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A94" s="337"/>
       <c r="B94" s="337"/>
       <c r="C94" s="419"/>
-      <c r="D94" s="424"/>
+      <c r="D94" s="426"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A95" s="337"/>
       <c r="B95" s="337"/>
       <c r="C95" s="419"/>
-      <c r="D95" s="424"/>
+      <c r="D95" s="426"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A96" s="337"/>
       <c r="B96" s="337"/>
       <c r="C96" s="419"/>
-      <c r="D96" s="424"/>
+      <c r="D96" s="426"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A97" s="337"/>
       <c r="B97" s="337"/>
       <c r="C97" s="419"/>
-      <c r="D97" s="424"/>
+      <c r="D97" s="426"/>
     </row>
     <row r="98" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A98" s="320"/>
       <c r="B98" s="320"/>
       <c r="C98" s="420"/>
-      <c r="D98" s="425"/>
+      <c r="D98" s="427"/>
     </row>
     <row r="99" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A99" s="339"/>
@@ -10020,7 +10020,7 @@
       <c r="C99" s="422" t="s">
         <v>853</v>
       </c>
-      <c r="D99" s="424" t="s">
+      <c r="D99" s="426" t="s">
         <v>854</v>
       </c>
     </row>
@@ -10028,73 +10028,73 @@
       <c r="A100" s="339"/>
       <c r="B100" s="339"/>
       <c r="C100" s="422"/>
-      <c r="D100" s="424"/>
+      <c r="D100" s="426"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A101" s="339"/>
       <c r="B101" s="339"/>
       <c r="C101" s="422"/>
-      <c r="D101" s="424"/>
+      <c r="D101" s="426"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A102" s="339"/>
       <c r="B102" s="339"/>
       <c r="C102" s="422"/>
-      <c r="D102" s="424"/>
+      <c r="D102" s="426"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A103" s="339"/>
       <c r="B103" s="339"/>
       <c r="C103" s="422"/>
-      <c r="D103" s="424"/>
+      <c r="D103" s="426"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A104" s="339"/>
       <c r="B104" s="339"/>
       <c r="C104" s="422"/>
-      <c r="D104" s="424"/>
+      <c r="D104" s="426"/>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A105" s="339"/>
       <c r="B105" s="339"/>
       <c r="C105" s="422"/>
-      <c r="D105" s="424"/>
+      <c r="D105" s="426"/>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A106" s="339"/>
       <c r="B106" s="339"/>
       <c r="C106" s="422"/>
-      <c r="D106" s="424"/>
+      <c r="D106" s="426"/>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A107" s="339"/>
       <c r="B107" s="339"/>
       <c r="C107" s="422"/>
-      <c r="D107" s="424"/>
+      <c r="D107" s="426"/>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A108" s="339"/>
       <c r="B108" s="339"/>
       <c r="C108" s="422"/>
-      <c r="D108" s="424"/>
+      <c r="D108" s="426"/>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A109" s="339"/>
       <c r="B109" s="339"/>
       <c r="C109" s="422"/>
-      <c r="D109" s="424"/>
+      <c r="D109" s="426"/>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A110" s="339"/>
       <c r="B110" s="339"/>
       <c r="C110" s="422"/>
-      <c r="D110" s="424"/>
+      <c r="D110" s="426"/>
     </row>
     <row r="111" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A111" s="321"/>
       <c r="B111" s="321"/>
       <c r="C111" s="423"/>
-      <c r="D111" s="425"/>
+      <c r="D111" s="427"/>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A112" s="335"/>
@@ -10102,7 +10102,7 @@
       <c r="C112" s="419" t="s">
         <v>855</v>
       </c>
-      <c r="D112" s="424" t="s">
+      <c r="D112" s="426" t="s">
         <v>856</v>
       </c>
     </row>
@@ -10110,67 +10110,67 @@
       <c r="A113" s="335"/>
       <c r="B113" s="335"/>
       <c r="C113" s="419"/>
-      <c r="D113" s="424"/>
+      <c r="D113" s="426"/>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A114" s="335"/>
       <c r="B114" s="335"/>
       <c r="C114" s="419"/>
-      <c r="D114" s="424"/>
+      <c r="D114" s="426"/>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A115" s="335"/>
       <c r="B115" s="335"/>
       <c r="C115" s="419"/>
-      <c r="D115" s="424"/>
+      <c r="D115" s="426"/>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A116" s="335"/>
       <c r="B116" s="335"/>
       <c r="C116" s="419"/>
-      <c r="D116" s="424"/>
+      <c r="D116" s="426"/>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A117" s="335"/>
       <c r="B117" s="335"/>
       <c r="C117" s="419"/>
-      <c r="D117" s="424"/>
+      <c r="D117" s="426"/>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A118" s="335"/>
       <c r="B118" s="335"/>
       <c r="C118" s="419"/>
-      <c r="D118" s="424"/>
+      <c r="D118" s="426"/>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A119" s="335"/>
       <c r="B119" s="335"/>
       <c r="C119" s="419"/>
-      <c r="D119" s="424"/>
+      <c r="D119" s="426"/>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A120" s="335"/>
       <c r="B120" s="335"/>
       <c r="C120" s="419"/>
-      <c r="D120" s="424"/>
+      <c r="D120" s="426"/>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A121" s="335"/>
       <c r="B121" s="335"/>
       <c r="C121" s="419"/>
-      <c r="D121" s="424"/>
+      <c r="D121" s="426"/>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A122" s="335"/>
       <c r="B122" s="335"/>
       <c r="C122" s="419"/>
-      <c r="D122" s="424"/>
+      <c r="D122" s="426"/>
     </row>
     <row r="123" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A123" s="316"/>
       <c r="B123" s="316"/>
       <c r="C123" s="420"/>
-      <c r="D123" s="425"/>
+      <c r="D123" s="427"/>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A124" s="334"/>
@@ -10178,7 +10178,7 @@
       <c r="C124" s="419" t="s">
         <v>857</v>
       </c>
-      <c r="D124" s="424" t="s">
+      <c r="D124" s="426" t="s">
         <v>858</v>
       </c>
     </row>
@@ -10186,31 +10186,31 @@
       <c r="A125" s="334"/>
       <c r="B125" s="334"/>
       <c r="C125" s="419"/>
-      <c r="D125" s="424"/>
+      <c r="D125" s="426"/>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A126" s="334"/>
       <c r="B126" s="334"/>
       <c r="C126" s="419"/>
-      <c r="D126" s="424"/>
+      <c r="D126" s="426"/>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A127" s="334"/>
       <c r="B127" s="334"/>
       <c r="C127" s="419"/>
-      <c r="D127" s="424"/>
+      <c r="D127" s="426"/>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A128" s="334"/>
       <c r="B128" s="334"/>
       <c r="C128" s="419"/>
-      <c r="D128" s="424"/>
+      <c r="D128" s="426"/>
     </row>
     <row r="129" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A129" s="317"/>
       <c r="B129" s="317"/>
       <c r="C129" s="420"/>
-      <c r="D129" s="425"/>
+      <c r="D129" s="427"/>
     </row>
     <row r="130" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A130" s="33"/>
@@ -10218,7 +10218,7 @@
       <c r="C130" s="419" t="s">
         <v>859</v>
       </c>
-      <c r="D130" s="424" t="s">
+      <c r="D130" s="426" t="s">
         <v>860</v>
       </c>
     </row>
@@ -10226,19 +10226,19 @@
       <c r="A131" s="33"/>
       <c r="B131" s="33"/>
       <c r="C131" s="419"/>
-      <c r="D131" s="424"/>
+      <c r="D131" s="426"/>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A132" s="33"/>
       <c r="B132" s="33"/>
       <c r="C132" s="419"/>
-      <c r="D132" s="424"/>
+      <c r="D132" s="426"/>
     </row>
     <row r="133" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A133" s="322"/>
       <c r="B133" s="322"/>
       <c r="C133" s="420"/>
-      <c r="D133" s="425"/>
+      <c r="D133" s="427"/>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A134" s="338"/>
@@ -10246,7 +10246,7 @@
       <c r="C134" s="419" t="s">
         <v>861</v>
       </c>
-      <c r="D134" s="424" t="s">
+      <c r="D134" s="426" t="s">
         <v>862</v>
       </c>
     </row>
@@ -10254,103 +10254,103 @@
       <c r="A135" s="338"/>
       <c r="B135" s="338"/>
       <c r="C135" s="419"/>
-      <c r="D135" s="424"/>
+      <c r="D135" s="426"/>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A136" s="338"/>
       <c r="B136" s="338"/>
       <c r="C136" s="419"/>
-      <c r="D136" s="424"/>
+      <c r="D136" s="426"/>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A137" s="338"/>
       <c r="B137" s="338"/>
       <c r="C137" s="419"/>
-      <c r="D137" s="424"/>
+      <c r="D137" s="426"/>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A138" s="338"/>
       <c r="B138" s="338"/>
       <c r="C138" s="419"/>
-      <c r="D138" s="424"/>
+      <c r="D138" s="426"/>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A139" s="338"/>
       <c r="B139" s="338"/>
       <c r="C139" s="419"/>
-      <c r="D139" s="424"/>
+      <c r="D139" s="426"/>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A140" s="338"/>
       <c r="B140" s="338"/>
       <c r="C140" s="419"/>
-      <c r="D140" s="424"/>
+      <c r="D140" s="426"/>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A141" s="338"/>
       <c r="B141" s="338"/>
       <c r="C141" s="419"/>
-      <c r="D141" s="424"/>
+      <c r="D141" s="426"/>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A142" s="338"/>
       <c r="B142" s="338"/>
       <c r="C142" s="419"/>
-      <c r="D142" s="424"/>
+      <c r="D142" s="426"/>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A143" s="338"/>
       <c r="B143" s="338"/>
       <c r="C143" s="419"/>
-      <c r="D143" s="424"/>
+      <c r="D143" s="426"/>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A144" s="338"/>
       <c r="B144" s="338"/>
       <c r="C144" s="419"/>
-      <c r="D144" s="424"/>
+      <c r="D144" s="426"/>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A145" s="338"/>
       <c r="B145" s="338"/>
       <c r="C145" s="419"/>
-      <c r="D145" s="424"/>
+      <c r="D145" s="426"/>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A146" s="338"/>
       <c r="B146" s="338"/>
       <c r="C146" s="419"/>
-      <c r="D146" s="424"/>
+      <c r="D146" s="426"/>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A147" s="338"/>
       <c r="B147" s="338"/>
       <c r="C147" s="419"/>
-      <c r="D147" s="424"/>
+      <c r="D147" s="426"/>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A148" s="338"/>
       <c r="B148" s="338"/>
       <c r="C148" s="419"/>
-      <c r="D148" s="424"/>
+      <c r="D148" s="426"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A149" s="338"/>
       <c r="B149" s="338"/>
       <c r="C149" s="419"/>
-      <c r="D149" s="424"/>
+      <c r="D149" s="426"/>
     </row>
     <row r="150" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A150" s="338"/>
       <c r="B150" s="338"/>
       <c r="C150" s="419"/>
-      <c r="D150" s="424"/>
+      <c r="D150" s="426"/>
     </row>
     <row r="151" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A151" s="319"/>
       <c r="B151" s="319"/>
       <c r="C151" s="420"/>
-      <c r="D151" s="425"/>
+      <c r="D151" s="427"/>
     </row>
     <row r="152" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A152" s="340"/>
@@ -10358,7 +10358,7 @@
       <c r="C152" s="419" t="s">
         <v>863</v>
       </c>
-      <c r="D152" s="424" t="s">
+      <c r="D152" s="426" t="s">
         <v>864</v>
       </c>
     </row>
@@ -10366,47 +10366,47 @@
       <c r="A153" s="340"/>
       <c r="B153" s="340"/>
       <c r="C153" s="419"/>
-      <c r="D153" s="424"/>
+      <c r="D153" s="426"/>
     </row>
     <row r="154" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A154" s="340"/>
       <c r="B154" s="340"/>
       <c r="C154" s="419"/>
-      <c r="D154" s="424"/>
+      <c r="D154" s="426"/>
     </row>
     <row r="155" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A155" s="323"/>
       <c r="B155" s="323"/>
       <c r="C155" s="420"/>
-      <c r="D155" s="425"/>
+      <c r="D155" s="427"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="24">
+    <mergeCell ref="C130:C133"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="C134:C151"/>
+    <mergeCell ref="D134:D151"/>
+    <mergeCell ref="C152:C155"/>
+    <mergeCell ref="D152:D155"/>
+    <mergeCell ref="C99:C111"/>
+    <mergeCell ref="D99:D111"/>
+    <mergeCell ref="C112:C123"/>
+    <mergeCell ref="D112:D123"/>
+    <mergeCell ref="C124:C129"/>
+    <mergeCell ref="D124:D129"/>
+    <mergeCell ref="C58:C72"/>
+    <mergeCell ref="D58:D72"/>
+    <mergeCell ref="C73:C89"/>
+    <mergeCell ref="D73:D89"/>
+    <mergeCell ref="C90:C98"/>
+    <mergeCell ref="D90:D98"/>
     <mergeCell ref="C2:C17"/>
     <mergeCell ref="D2:D17"/>
     <mergeCell ref="C18:C37"/>
     <mergeCell ref="D18:D37"/>
     <mergeCell ref="C38:C57"/>
     <mergeCell ref="D38:D57"/>
-    <mergeCell ref="C58:C72"/>
-    <mergeCell ref="D58:D72"/>
-    <mergeCell ref="C73:C89"/>
-    <mergeCell ref="D73:D89"/>
-    <mergeCell ref="C90:C98"/>
-    <mergeCell ref="D90:D98"/>
-    <mergeCell ref="C99:C111"/>
-    <mergeCell ref="D99:D111"/>
-    <mergeCell ref="C112:C123"/>
-    <mergeCell ref="D112:D123"/>
-    <mergeCell ref="C124:C129"/>
-    <mergeCell ref="D124:D129"/>
-    <mergeCell ref="C130:C133"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="C134:C151"/>
-    <mergeCell ref="D134:D151"/>
-    <mergeCell ref="C152:C155"/>
-    <mergeCell ref="D152:D155"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -11744,21 +11744,21 @@
   <sheetData>
     <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="33"/>
-      <c r="B1" s="411" t="s">
+      <c r="B1" s="406" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="412"/>
-      <c r="D1" s="413"/>
-      <c r="E1" s="411" t="s">
+      <c r="C1" s="407"/>
+      <c r="D1" s="408"/>
+      <c r="E1" s="406" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="412"/>
-      <c r="G1" s="412"/>
+      <c r="F1" s="407"/>
+      <c r="G1" s="407"/>
       <c r="H1" s="309"/>
-      <c r="K1" s="414" t="s">
+      <c r="K1" s="409" t="s">
         <v>836</v>
       </c>
-      <c r="L1" s="415"/>
+      <c r="L1" s="410"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A2" s="61" t="s">
@@ -12846,103 +12846,103 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:67" x14ac:dyDescent="0.4">
-      <c r="A1" s="399" t="s">
+      <c r="A1" s="400" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="399"/>
-      <c r="C1" s="399"/>
-      <c r="D1" s="399"/>
-      <c r="E1" s="400" t="s">
+      <c r="B1" s="400"/>
+      <c r="C1" s="400"/>
+      <c r="D1" s="400"/>
+      <c r="E1" s="401" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="401"/>
-      <c r="G1" s="401"/>
-      <c r="H1" s="401"/>
-      <c r="I1" s="401"/>
-      <c r="J1" s="401"/>
-      <c r="K1" s="401"/>
-      <c r="L1" s="401"/>
-      <c r="M1" s="401"/>
-      <c r="N1" s="401"/>
-      <c r="O1" s="402"/>
-      <c r="P1" s="416" t="s">
+      <c r="F1" s="402"/>
+      <c r="G1" s="402"/>
+      <c r="H1" s="402"/>
+      <c r="I1" s="402"/>
+      <c r="J1" s="402"/>
+      <c r="K1" s="402"/>
+      <c r="L1" s="402"/>
+      <c r="M1" s="402"/>
+      <c r="N1" s="402"/>
+      <c r="O1" s="403"/>
+      <c r="P1" s="399" t="s">
         <v>77</v>
       </c>
-      <c r="Q1" s="416"/>
-      <c r="R1" s="416"/>
-      <c r="S1" s="416"/>
-      <c r="T1" s="399" t="s">
+      <c r="Q1" s="399"/>
+      <c r="R1" s="399"/>
+      <c r="S1" s="399"/>
+      <c r="T1" s="400" t="s">
         <v>78</v>
       </c>
-      <c r="U1" s="399"/>
-      <c r="V1" s="399"/>
-      <c r="W1" s="399"/>
-      <c r="X1" s="416" t="s">
+      <c r="U1" s="400"/>
+      <c r="V1" s="400"/>
+      <c r="W1" s="400"/>
+      <c r="X1" s="399" t="s">
         <v>79</v>
       </c>
-      <c r="Y1" s="416"/>
-      <c r="Z1" s="416"/>
-      <c r="AA1" s="416"/>
-      <c r="AB1" s="399" t="s">
+      <c r="Y1" s="399"/>
+      <c r="Z1" s="399"/>
+      <c r="AA1" s="399"/>
+      <c r="AB1" s="400" t="s">
         <v>80</v>
       </c>
-      <c r="AC1" s="399"/>
-      <c r="AD1" s="399"/>
-      <c r="AE1" s="399"/>
-      <c r="AF1" s="416" t="s">
+      <c r="AC1" s="400"/>
+      <c r="AD1" s="400"/>
+      <c r="AE1" s="400"/>
+      <c r="AF1" s="399" t="s">
         <v>81</v>
       </c>
-      <c r="AG1" s="416"/>
-      <c r="AH1" s="416"/>
-      <c r="AI1" s="416"/>
-      <c r="AJ1" s="399" t="s">
+      <c r="AG1" s="399"/>
+      <c r="AH1" s="399"/>
+      <c r="AI1" s="399"/>
+      <c r="AJ1" s="400" t="s">
         <v>82</v>
       </c>
-      <c r="AK1" s="399"/>
-      <c r="AL1" s="399"/>
-      <c r="AM1" s="399"/>
-      <c r="AN1" s="416" t="s">
+      <c r="AK1" s="400"/>
+      <c r="AL1" s="400"/>
+      <c r="AM1" s="400"/>
+      <c r="AN1" s="399" t="s">
         <v>83</v>
       </c>
-      <c r="AO1" s="416"/>
-      <c r="AP1" s="416"/>
-      <c r="AQ1" s="416"/>
-      <c r="AR1" s="399" t="s">
+      <c r="AO1" s="399"/>
+      <c r="AP1" s="399"/>
+      <c r="AQ1" s="399"/>
+      <c r="AR1" s="400" t="s">
         <v>84</v>
       </c>
-      <c r="AS1" s="399"/>
-      <c r="AT1" s="399"/>
-      <c r="AU1" s="399"/>
-      <c r="AV1" s="416" t="s">
+      <c r="AS1" s="400"/>
+      <c r="AT1" s="400"/>
+      <c r="AU1" s="400"/>
+      <c r="AV1" s="399" t="s">
         <v>85</v>
       </c>
-      <c r="AW1" s="416"/>
-      <c r="AX1" s="416"/>
-      <c r="AY1" s="416"/>
-      <c r="AZ1" s="399" t="s">
+      <c r="AW1" s="399"/>
+      <c r="AX1" s="399"/>
+      <c r="AY1" s="399"/>
+      <c r="AZ1" s="400" t="s">
         <v>86</v>
       </c>
-      <c r="BA1" s="399"/>
-      <c r="BB1" s="399"/>
-      <c r="BC1" s="399"/>
-      <c r="BD1" s="416" t="s">
+      <c r="BA1" s="400"/>
+      <c r="BB1" s="400"/>
+      <c r="BC1" s="400"/>
+      <c r="BD1" s="399" t="s">
         <v>87</v>
       </c>
-      <c r="BE1" s="416"/>
-      <c r="BF1" s="416"/>
-      <c r="BG1" s="416"/>
-      <c r="BH1" s="399" t="s">
+      <c r="BE1" s="399"/>
+      <c r="BF1" s="399"/>
+      <c r="BG1" s="399"/>
+      <c r="BH1" s="400" t="s">
         <v>88</v>
       </c>
-      <c r="BI1" s="399"/>
-      <c r="BJ1" s="399"/>
-      <c r="BK1" s="399"/>
-      <c r="BL1" s="416" t="s">
+      <c r="BI1" s="400"/>
+      <c r="BJ1" s="400"/>
+      <c r="BK1" s="400"/>
+      <c r="BL1" s="399" t="s">
         <v>495</v>
       </c>
-      <c r="BM1" s="416"/>
-      <c r="BN1" s="416"/>
-      <c r="BO1" s="416"/>
+      <c r="BM1" s="399"/>
+      <c r="BN1" s="399"/>
+      <c r="BO1" s="399"/>
     </row>
     <row r="2" spans="1:67" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -35303,96 +35303,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:94" x14ac:dyDescent="0.4">
-      <c r="A1" s="399" t="s">
+      <c r="A1" s="400" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="399"/>
-      <c r="C1" s="399"/>
-      <c r="D1" s="399"/>
-      <c r="E1" s="400" t="s">
+      <c r="B1" s="400"/>
+      <c r="C1" s="400"/>
+      <c r="D1" s="400"/>
+      <c r="E1" s="401" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="401"/>
-      <c r="G1" s="401"/>
-      <c r="H1" s="401"/>
-      <c r="I1" s="401"/>
-      <c r="J1" s="401"/>
-      <c r="K1" s="401"/>
-      <c r="L1" s="401"/>
-      <c r="M1" s="401"/>
-      <c r="N1" s="402"/>
-      <c r="O1" s="406" t="s">
+      <c r="F1" s="402"/>
+      <c r="G1" s="402"/>
+      <c r="H1" s="402"/>
+      <c r="I1" s="402"/>
+      <c r="J1" s="402"/>
+      <c r="K1" s="402"/>
+      <c r="L1" s="402"/>
+      <c r="M1" s="402"/>
+      <c r="N1" s="403"/>
+      <c r="O1" s="414" t="s">
         <v>77</v>
       </c>
-      <c r="P1" s="407"/>
-      <c r="Q1" s="407"/>
-      <c r="R1" s="408"/>
-      <c r="S1" s="400" t="s">
+      <c r="P1" s="415"/>
+      <c r="Q1" s="415"/>
+      <c r="R1" s="416"/>
+      <c r="S1" s="401" t="s">
         <v>78</v>
       </c>
-      <c r="T1" s="401"/>
-      <c r="U1" s="401"/>
-      <c r="V1" s="401"/>
-      <c r="W1" s="406" t="s">
+      <c r="T1" s="402"/>
+      <c r="U1" s="402"/>
+      <c r="V1" s="402"/>
+      <c r="W1" s="414" t="s">
         <v>79</v>
       </c>
-      <c r="X1" s="407"/>
-      <c r="Y1" s="407"/>
-      <c r="Z1" s="408"/>
-      <c r="AA1" s="403" t="s">
+      <c r="X1" s="415"/>
+      <c r="Y1" s="415"/>
+      <c r="Z1" s="416"/>
+      <c r="AA1" s="411" t="s">
         <v>80</v>
       </c>
-      <c r="AB1" s="404"/>
-      <c r="AC1" s="404"/>
-      <c r="AD1" s="405"/>
-      <c r="AE1" s="406" t="s">
+      <c r="AB1" s="412"/>
+      <c r="AC1" s="412"/>
+      <c r="AD1" s="413"/>
+      <c r="AE1" s="414" t="s">
         <v>81</v>
       </c>
-      <c r="AF1" s="407"/>
-      <c r="AG1" s="407"/>
-      <c r="AH1" s="408"/>
-      <c r="AI1" s="403" t="s">
+      <c r="AF1" s="415"/>
+      <c r="AG1" s="415"/>
+      <c r="AH1" s="416"/>
+      <c r="AI1" s="411" t="s">
         <v>82</v>
       </c>
-      <c r="AJ1" s="404"/>
-      <c r="AK1" s="404"/>
-      <c r="AL1" s="405"/>
-      <c r="AM1" s="406" t="s">
+      <c r="AJ1" s="412"/>
+      <c r="AK1" s="412"/>
+      <c r="AL1" s="413"/>
+      <c r="AM1" s="414" t="s">
         <v>83</v>
       </c>
-      <c r="AN1" s="407"/>
-      <c r="AO1" s="407"/>
-      <c r="AP1" s="408"/>
-      <c r="AQ1" s="403" t="s">
+      <c r="AN1" s="415"/>
+      <c r="AO1" s="415"/>
+      <c r="AP1" s="416"/>
+      <c r="AQ1" s="411" t="s">
         <v>84</v>
       </c>
-      <c r="AR1" s="404"/>
-      <c r="AS1" s="404"/>
-      <c r="AT1" s="405"/>
-      <c r="AU1" s="406" t="s">
+      <c r="AR1" s="412"/>
+      <c r="AS1" s="412"/>
+      <c r="AT1" s="413"/>
+      <c r="AU1" s="414" t="s">
         <v>85</v>
       </c>
-      <c r="AV1" s="407"/>
-      <c r="AW1" s="407"/>
-      <c r="AX1" s="408"/>
-      <c r="AY1" s="403" t="s">
+      <c r="AV1" s="415"/>
+      <c r="AW1" s="415"/>
+      <c r="AX1" s="416"/>
+      <c r="AY1" s="411" t="s">
         <v>86</v>
       </c>
-      <c r="AZ1" s="404"/>
-      <c r="BA1" s="404"/>
-      <c r="BB1" s="405"/>
-      <c r="BC1" s="406" t="s">
+      <c r="AZ1" s="412"/>
+      <c r="BA1" s="412"/>
+      <c r="BB1" s="413"/>
+      <c r="BC1" s="414" t="s">
         <v>87</v>
       </c>
-      <c r="BD1" s="407"/>
-      <c r="BE1" s="407"/>
-      <c r="BF1" s="408"/>
-      <c r="BG1" s="403" t="s">
+      <c r="BD1" s="415"/>
+      <c r="BE1" s="415"/>
+      <c r="BF1" s="416"/>
+      <c r="BG1" s="411" t="s">
         <v>88</v>
       </c>
-      <c r="BH1" s="404"/>
-      <c r="BI1" s="404"/>
-      <c r="BJ1" s="405"/>
+      <c r="BH1" s="412"/>
+      <c r="BI1" s="412"/>
+      <c r="BJ1" s="413"/>
     </row>
     <row r="2" spans="1:94" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -40061,7 +40061,7 @@
         <v>105</v>
       </c>
       <c r="N45" s="22">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="O45" s="122" t="s">
         <v>944</v>
@@ -45806,97 +45806,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:63" x14ac:dyDescent="0.4">
-      <c r="A1" s="399" t="s">
+      <c r="A1" s="400" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="399"/>
-      <c r="C1" s="399"/>
-      <c r="D1" s="399"/>
-      <c r="E1" s="400" t="s">
+      <c r="B1" s="400"/>
+      <c r="C1" s="400"/>
+      <c r="D1" s="400"/>
+      <c r="E1" s="401" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="401"/>
-      <c r="G1" s="401"/>
-      <c r="H1" s="401"/>
-      <c r="I1" s="401"/>
-      <c r="J1" s="401"/>
-      <c r="K1" s="401"/>
-      <c r="L1" s="401"/>
-      <c r="M1" s="401"/>
-      <c r="N1" s="401"/>
-      <c r="O1" s="402"/>
+      <c r="F1" s="402"/>
+      <c r="G1" s="402"/>
+      <c r="H1" s="402"/>
+      <c r="I1" s="402"/>
+      <c r="J1" s="402"/>
+      <c r="K1" s="402"/>
+      <c r="L1" s="402"/>
+      <c r="M1" s="402"/>
+      <c r="N1" s="402"/>
+      <c r="O1" s="403"/>
       <c r="P1" s="417" t="s">
         <v>77</v>
       </c>
       <c r="Q1" s="417"/>
       <c r="R1" s="417"/>
       <c r="S1" s="417"/>
-      <c r="T1" s="399" t="s">
+      <c r="T1" s="400" t="s">
         <v>78</v>
       </c>
-      <c r="U1" s="399"/>
-      <c r="V1" s="399"/>
-      <c r="W1" s="399"/>
+      <c r="U1" s="400"/>
+      <c r="V1" s="400"/>
+      <c r="W1" s="400"/>
       <c r="X1" s="417" t="s">
         <v>79</v>
       </c>
       <c r="Y1" s="417"/>
       <c r="Z1" s="417"/>
       <c r="AA1" s="417"/>
-      <c r="AB1" s="399" t="s">
+      <c r="AB1" s="400" t="s">
         <v>80</v>
       </c>
-      <c r="AC1" s="399"/>
-      <c r="AD1" s="399"/>
-      <c r="AE1" s="399"/>
+      <c r="AC1" s="400"/>
+      <c r="AD1" s="400"/>
+      <c r="AE1" s="400"/>
       <c r="AF1" s="417" t="s">
         <v>81</v>
       </c>
       <c r="AG1" s="417"/>
       <c r="AH1" s="417"/>
       <c r="AI1" s="417"/>
-      <c r="AJ1" s="399" t="s">
+      <c r="AJ1" s="400" t="s">
         <v>82</v>
       </c>
-      <c r="AK1" s="399"/>
-      <c r="AL1" s="399"/>
-      <c r="AM1" s="399"/>
+      <c r="AK1" s="400"/>
+      <c r="AL1" s="400"/>
+      <c r="AM1" s="400"/>
       <c r="AN1" s="417" t="s">
         <v>83</v>
       </c>
       <c r="AO1" s="417"/>
       <c r="AP1" s="417"/>
       <c r="AQ1" s="417"/>
-      <c r="AR1" s="399" t="s">
+      <c r="AR1" s="400" t="s">
         <v>84</v>
       </c>
-      <c r="AS1" s="399"/>
-      <c r="AT1" s="399"/>
-      <c r="AU1" s="399"/>
+      <c r="AS1" s="400"/>
+      <c r="AT1" s="400"/>
+      <c r="AU1" s="400"/>
       <c r="AV1" s="417" t="s">
         <v>85</v>
       </c>
       <c r="AW1" s="417"/>
       <c r="AX1" s="417"/>
       <c r="AY1" s="417"/>
-      <c r="AZ1" s="399" t="s">
+      <c r="AZ1" s="400" t="s">
         <v>86</v>
       </c>
-      <c r="BA1" s="399"/>
-      <c r="BB1" s="399"/>
-      <c r="BC1" s="399"/>
+      <c r="BA1" s="400"/>
+      <c r="BB1" s="400"/>
+      <c r="BC1" s="400"/>
       <c r="BD1" s="417" t="s">
         <v>87</v>
       </c>
       <c r="BE1" s="417"/>
       <c r="BF1" s="417"/>
       <c r="BG1" s="417"/>
-      <c r="BH1" s="399" t="s">
+      <c r="BH1" s="400" t="s">
         <v>88</v>
       </c>
-      <c r="BI1" s="399"/>
-      <c r="BJ1" s="399"/>
-      <c r="BK1" s="399"/>
+      <c r="BI1" s="400"/>
+      <c r="BJ1" s="400"/>
+      <c r="BK1" s="400"/>
     </row>
     <row r="2" spans="1:63" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -55204,109 +55204,109 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:73" x14ac:dyDescent="0.4">
-      <c r="A1" s="399" t="s">
+      <c r="A1" s="400" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="399"/>
-      <c r="C1" s="399"/>
-      <c r="D1" s="399"/>
-      <c r="E1" s="400" t="s">
+      <c r="B1" s="400"/>
+      <c r="C1" s="400"/>
+      <c r="D1" s="400"/>
+      <c r="E1" s="401" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="401"/>
-      <c r="G1" s="401"/>
-      <c r="H1" s="401"/>
-      <c r="I1" s="401"/>
-      <c r="J1" s="401"/>
-      <c r="K1" s="401"/>
-      <c r="L1" s="401"/>
-      <c r="M1" s="401"/>
-      <c r="N1" s="401"/>
-      <c r="O1" s="401"/>
-      <c r="P1" s="401"/>
-      <c r="Q1" s="401"/>
-      <c r="R1" s="401"/>
-      <c r="S1" s="401"/>
-      <c r="T1" s="401"/>
-      <c r="U1" s="402"/>
-      <c r="V1" s="416" t="s">
+      <c r="F1" s="402"/>
+      <c r="G1" s="402"/>
+      <c r="H1" s="402"/>
+      <c r="I1" s="402"/>
+      <c r="J1" s="402"/>
+      <c r="K1" s="402"/>
+      <c r="L1" s="402"/>
+      <c r="M1" s="402"/>
+      <c r="N1" s="402"/>
+      <c r="O1" s="402"/>
+      <c r="P1" s="402"/>
+      <c r="Q1" s="402"/>
+      <c r="R1" s="402"/>
+      <c r="S1" s="402"/>
+      <c r="T1" s="402"/>
+      <c r="U1" s="403"/>
+      <c r="V1" s="399" t="s">
         <v>77</v>
       </c>
-      <c r="W1" s="416"/>
-      <c r="X1" s="416"/>
-      <c r="Y1" s="416"/>
-      <c r="Z1" s="399" t="s">
+      <c r="W1" s="399"/>
+      <c r="X1" s="399"/>
+      <c r="Y1" s="399"/>
+      <c r="Z1" s="400" t="s">
         <v>78</v>
       </c>
-      <c r="AA1" s="399"/>
-      <c r="AB1" s="399"/>
-      <c r="AC1" s="399"/>
-      <c r="AD1" s="416" t="s">
+      <c r="AA1" s="400"/>
+      <c r="AB1" s="400"/>
+      <c r="AC1" s="400"/>
+      <c r="AD1" s="399" t="s">
         <v>79</v>
       </c>
-      <c r="AE1" s="416"/>
-      <c r="AF1" s="416"/>
-      <c r="AG1" s="416"/>
-      <c r="AH1" s="399" t="s">
+      <c r="AE1" s="399"/>
+      <c r="AF1" s="399"/>
+      <c r="AG1" s="399"/>
+      <c r="AH1" s="400" t="s">
         <v>80</v>
       </c>
-      <c r="AI1" s="399"/>
-      <c r="AJ1" s="399"/>
-      <c r="AK1" s="399"/>
-      <c r="AL1" s="416" t="s">
+      <c r="AI1" s="400"/>
+      <c r="AJ1" s="400"/>
+      <c r="AK1" s="400"/>
+      <c r="AL1" s="399" t="s">
         <v>81</v>
       </c>
-      <c r="AM1" s="416"/>
-      <c r="AN1" s="416"/>
-      <c r="AO1" s="416"/>
-      <c r="AP1" s="399" t="s">
+      <c r="AM1" s="399"/>
+      <c r="AN1" s="399"/>
+      <c r="AO1" s="399"/>
+      <c r="AP1" s="400" t="s">
         <v>82</v>
       </c>
-      <c r="AQ1" s="399"/>
-      <c r="AR1" s="399"/>
-      <c r="AS1" s="399"/>
-      <c r="AT1" s="416" t="s">
+      <c r="AQ1" s="400"/>
+      <c r="AR1" s="400"/>
+      <c r="AS1" s="400"/>
+      <c r="AT1" s="399" t="s">
         <v>83</v>
       </c>
-      <c r="AU1" s="416"/>
-      <c r="AV1" s="416"/>
-      <c r="AW1" s="416"/>
-      <c r="AX1" s="399" t="s">
+      <c r="AU1" s="399"/>
+      <c r="AV1" s="399"/>
+      <c r="AW1" s="399"/>
+      <c r="AX1" s="400" t="s">
         <v>84</v>
       </c>
-      <c r="AY1" s="399"/>
-      <c r="AZ1" s="399"/>
-      <c r="BA1" s="399"/>
-      <c r="BB1" s="416" t="s">
+      <c r="AY1" s="400"/>
+      <c r="AZ1" s="400"/>
+      <c r="BA1" s="400"/>
+      <c r="BB1" s="399" t="s">
         <v>85</v>
       </c>
-      <c r="BC1" s="416"/>
-      <c r="BD1" s="416"/>
-      <c r="BE1" s="416"/>
-      <c r="BF1" s="399" t="s">
+      <c r="BC1" s="399"/>
+      <c r="BD1" s="399"/>
+      <c r="BE1" s="399"/>
+      <c r="BF1" s="400" t="s">
         <v>86</v>
       </c>
-      <c r="BG1" s="399"/>
-      <c r="BH1" s="399"/>
-      <c r="BI1" s="399"/>
-      <c r="BJ1" s="416" t="s">
+      <c r="BG1" s="400"/>
+      <c r="BH1" s="400"/>
+      <c r="BI1" s="400"/>
+      <c r="BJ1" s="399" t="s">
         <v>87</v>
       </c>
-      <c r="BK1" s="416"/>
-      <c r="BL1" s="416"/>
-      <c r="BM1" s="416"/>
-      <c r="BN1" s="399" t="s">
+      <c r="BK1" s="399"/>
+      <c r="BL1" s="399"/>
+      <c r="BM1" s="399"/>
+      <c r="BN1" s="400" t="s">
         <v>88</v>
       </c>
-      <c r="BO1" s="399"/>
-      <c r="BP1" s="399"/>
-      <c r="BQ1" s="399"/>
-      <c r="BR1" s="416" t="s">
+      <c r="BO1" s="400"/>
+      <c r="BP1" s="400"/>
+      <c r="BQ1" s="400"/>
+      <c r="BR1" s="399" t="s">
         <v>495</v>
       </c>
-      <c r="BS1" s="416"/>
-      <c r="BT1" s="416"/>
-      <c r="BU1" s="416"/>
+      <c r="BS1" s="399"/>
+      <c r="BT1" s="399"/>
+      <c r="BU1" s="399"/>
     </row>
     <row r="2" spans="1:73" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -68348,12 +68348,6 @@
   </sheetData>
   <autoFilter ref="A2:BQ178" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="15">
-    <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:U1"/>
-    <mergeCell ref="V1:Y1"/>
-    <mergeCell ref="Z1:AC1"/>
-    <mergeCell ref="AD1:AG1"/>
     <mergeCell ref="BJ1:BM1"/>
     <mergeCell ref="BN1:BQ1"/>
     <mergeCell ref="BR1:BU1"/>
@@ -68363,6 +68357,12 @@
     <mergeCell ref="AX1:BA1"/>
     <mergeCell ref="BB1:BE1"/>
     <mergeCell ref="BF1:BI1"/>
+    <mergeCell ref="AH1:AK1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:U1"/>
+    <mergeCell ref="V1:Y1"/>
+    <mergeCell ref="Z1:AC1"/>
+    <mergeCell ref="AD1:AG1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -68492,97 +68492,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:63" x14ac:dyDescent="0.4">
-      <c r="A1" s="399" t="s">
+      <c r="A1" s="400" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="399"/>
-      <c r="C1" s="399"/>
-      <c r="D1" s="399"/>
-      <c r="E1" s="400" t="s">
+      <c r="B1" s="400"/>
+      <c r="C1" s="400"/>
+      <c r="D1" s="400"/>
+      <c r="E1" s="401" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="401"/>
-      <c r="G1" s="401"/>
-      <c r="H1" s="401"/>
-      <c r="I1" s="401"/>
-      <c r="J1" s="401"/>
-      <c r="K1" s="401"/>
-      <c r="L1" s="401"/>
-      <c r="M1" s="401"/>
-      <c r="N1" s="401"/>
-      <c r="O1" s="402"/>
+      <c r="F1" s="402"/>
+      <c r="G1" s="402"/>
+      <c r="H1" s="402"/>
+      <c r="I1" s="402"/>
+      <c r="J1" s="402"/>
+      <c r="K1" s="402"/>
+      <c r="L1" s="402"/>
+      <c r="M1" s="402"/>
+      <c r="N1" s="402"/>
+      <c r="O1" s="403"/>
       <c r="P1" s="417" t="s">
         <v>77</v>
       </c>
       <c r="Q1" s="417"/>
       <c r="R1" s="417"/>
       <c r="S1" s="417"/>
-      <c r="T1" s="400" t="s">
+      <c r="T1" s="401" t="s">
         <v>78</v>
       </c>
-      <c r="U1" s="401"/>
-      <c r="V1" s="401"/>
-      <c r="W1" s="401"/>
+      <c r="U1" s="402"/>
+      <c r="V1" s="402"/>
+      <c r="W1" s="402"/>
       <c r="X1" s="417" t="s">
         <v>79</v>
       </c>
       <c r="Y1" s="417"/>
       <c r="Z1" s="417"/>
       <c r="AA1" s="417"/>
-      <c r="AB1" s="400" t="s">
+      <c r="AB1" s="401" t="s">
         <v>80</v>
       </c>
-      <c r="AC1" s="401"/>
-      <c r="AD1" s="401"/>
-      <c r="AE1" s="401"/>
+      <c r="AC1" s="402"/>
+      <c r="AD1" s="402"/>
+      <c r="AE1" s="402"/>
       <c r="AF1" s="417" t="s">
         <v>81</v>
       </c>
       <c r="AG1" s="417"/>
       <c r="AH1" s="417"/>
       <c r="AI1" s="417"/>
-      <c r="AJ1" s="400" t="s">
+      <c r="AJ1" s="401" t="s">
         <v>82</v>
       </c>
-      <c r="AK1" s="401"/>
-      <c r="AL1" s="401"/>
-      <c r="AM1" s="401"/>
+      <c r="AK1" s="402"/>
+      <c r="AL1" s="402"/>
+      <c r="AM1" s="402"/>
       <c r="AN1" s="417" t="s">
         <v>83</v>
       </c>
       <c r="AO1" s="417"/>
       <c r="AP1" s="417"/>
       <c r="AQ1" s="417"/>
-      <c r="AR1" s="400" t="s">
+      <c r="AR1" s="401" t="s">
         <v>84</v>
       </c>
-      <c r="AS1" s="401"/>
-      <c r="AT1" s="401"/>
-      <c r="AU1" s="401"/>
+      <c r="AS1" s="402"/>
+      <c r="AT1" s="402"/>
+      <c r="AU1" s="402"/>
       <c r="AV1" s="417" t="s">
         <v>85</v>
       </c>
       <c r="AW1" s="417"/>
       <c r="AX1" s="417"/>
       <c r="AY1" s="417"/>
-      <c r="AZ1" s="400" t="s">
+      <c r="AZ1" s="401" t="s">
         <v>86</v>
       </c>
-      <c r="BA1" s="401"/>
-      <c r="BB1" s="401"/>
-      <c r="BC1" s="401"/>
+      <c r="BA1" s="402"/>
+      <c r="BB1" s="402"/>
+      <c r="BC1" s="402"/>
       <c r="BD1" s="417" t="s">
         <v>87</v>
       </c>
       <c r="BE1" s="417"/>
       <c r="BF1" s="417"/>
       <c r="BG1" s="417"/>
-      <c r="BH1" s="400" t="s">
+      <c r="BH1" s="401" t="s">
         <v>88</v>
       </c>
-      <c r="BI1" s="401"/>
-      <c r="BJ1" s="401"/>
-      <c r="BK1" s="401"/>
+      <c r="BI1" s="402"/>
+      <c r="BJ1" s="402"/>
+      <c r="BK1" s="402"/>
     </row>
     <row r="2" spans="1:63" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -78885,6 +78885,13 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="16">
+    <mergeCell ref="C58:C60"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="C2:C11"/>
+    <mergeCell ref="C12:C17"/>
+    <mergeCell ref="C18:C28"/>
+    <mergeCell ref="C44:C53"/>
+    <mergeCell ref="C29:C43"/>
     <mergeCell ref="C180:C182"/>
     <mergeCell ref="C178:C179"/>
     <mergeCell ref="C163:C176"/>
@@ -78894,13 +78901,6 @@
     <mergeCell ref="C99:C108"/>
     <mergeCell ref="C109:C115"/>
     <mergeCell ref="C116:C162"/>
-    <mergeCell ref="C58:C60"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="C2:C11"/>
-    <mergeCell ref="C12:C17"/>
-    <mergeCell ref="C18:C28"/>
-    <mergeCell ref="C44:C53"/>
-    <mergeCell ref="C29:C43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -78908,15 +78908,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FD8CECCB51EC843BF514AFE68379818" ma:contentTypeVersion="18" ma:contentTypeDescription="Opret et nyt dokument." ma:contentTypeScope="" ma:versionID="eda339f53f012ceb64677667a741b441">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="107e75b3-53cc-4838-92d2-ebc011bd4832" xmlns:ns3="888ccf44-0d39-41a2-ab17-f7efb2bf6977" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="04a86f3db711706e561c315688f1c464" ns2:_="" ns3:_="">
     <xsd:import namespace="107e75b3-53cc-4838-92d2-ebc011bd4832"/>
@@ -79165,6 +79156,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -79177,14 +79177,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74B21D61-7BBD-4BD3-A9A5-1E8F98F2F686}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F91B7B9-75FF-4624-B506-952B5B54766C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -79199,6 +79191,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74B21D61-7BBD-4BD3-A9A5-1E8F98F2F686}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update case names with SIPS instead of SystemGuard or SystemProtect in the RfG and DCC cases sheets to be consitent
</commit_message>
<xml_diff>
--- a/testcases.xlsx
+++ b/testcases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://energinet-my.sharepoint.com/personal/prw_energinet_dk/Documents/Dokumenter/GitHub/MTB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="11_710D79F8E8F49B720F18F8F5A5BEAA4096265349" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A65F2381-AA06-4215-A715-A4C5EA7B4ECF}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="11_710D79F8E8F49B720F18F8F5A5BEAA4096265349" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E6167DD-D679-419E-9BB4-72A703004ECA}"/>
   <bookViews>
-    <workbookView xWindow="-16935" yWindow="-21720" windowWidth="38640" windowHeight="21120" tabRatio="822" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15400" yWindow="-21710" windowWidth="51420" windowHeight="21100" tabRatio="822" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="29" r:id="rId1"/>
@@ -165,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5513" uniqueCount="947">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5513" uniqueCount="956">
   <si>
     <t>Comment</t>
   </si>
@@ -3785,6 +3785,33 @@
   <si>
     <t>System Integrity Protection Scheme (SIPS) real signal for Demand facilities
 The real signal will be converted into binary equivalent signal using the MTB SIPS Decoder blocks in PSCAD and PowerFactory</t>
+  </si>
+  <si>
+    <t>RfG_SIPS_Q</t>
+  </si>
+  <si>
+    <t>RfG_SIPS_QU</t>
+  </si>
+  <si>
+    <t>RfG_SIPS+fault</t>
+  </si>
+  <si>
+    <t>RfG_SIPS_StepPriority</t>
+  </si>
+  <si>
+    <t>RfG_SIPS_ControlRobustness</t>
+  </si>
+  <si>
+    <t>DCC_SIPS_StepPriority</t>
+  </si>
+  <si>
+    <t>DCC_SIPS_ControlRobustness</t>
+  </si>
+  <si>
+    <t>DCC_SIPS</t>
+  </si>
+  <si>
+    <t>DCC_SIPS+fault</t>
   </si>
 </sst>
 </file>
@@ -5781,9 +5808,6 @@
     <xf numFmtId="164" fontId="7" fillId="8" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5794,6 +5818,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5817,22 +5859,7 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5856,17 +5883,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -6423,16 +6450,16 @@
         <v>322</v>
       </c>
       <c r="G3" s="124"/>
-      <c r="H3" s="404" t="s">
+      <c r="H3" s="409" t="s">
         <v>339</v>
       </c>
-      <c r="I3" s="404"/>
-      <c r="J3" s="404"/>
-      <c r="K3" s="404" t="s">
+      <c r="I3" s="409"/>
+      <c r="J3" s="409"/>
+      <c r="K3" s="409" t="s">
         <v>340</v>
       </c>
-      <c r="L3" s="404"/>
-      <c r="M3" s="405"/>
+      <c r="L3" s="409"/>
+      <c r="M3" s="410"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4" s="248" t="s">
@@ -9411,102 +9438,102 @@
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="333"/>
       <c r="B2" s="333"/>
-      <c r="C2" s="424" t="s">
+      <c r="C2" s="426" t="s">
         <v>843</v>
       </c>
-      <c r="D2" s="426" t="s">
+      <c r="D2" s="424" t="s">
         <v>907</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="333"/>
       <c r="B3" s="333"/>
-      <c r="C3" s="424"/>
-      <c r="D3" s="426"/>
+      <c r="C3" s="426"/>
+      <c r="D3" s="424"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="333"/>
       <c r="B4" s="333"/>
-      <c r="C4" s="424"/>
-      <c r="D4" s="426"/>
+      <c r="C4" s="426"/>
+      <c r="D4" s="424"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="333"/>
       <c r="B5" s="333"/>
-      <c r="C5" s="424"/>
-      <c r="D5" s="426"/>
+      <c r="C5" s="426"/>
+      <c r="D5" s="424"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="333"/>
       <c r="B6" s="333"/>
-      <c r="C6" s="424"/>
-      <c r="D6" s="426"/>
+      <c r="C6" s="426"/>
+      <c r="D6" s="424"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="333"/>
       <c r="B7" s="333"/>
-      <c r="C7" s="424"/>
-      <c r="D7" s="426"/>
+      <c r="C7" s="426"/>
+      <c r="D7" s="424"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="333"/>
       <c r="B8" s="333"/>
-      <c r="C8" s="424"/>
-      <c r="D8" s="426"/>
+      <c r="C8" s="426"/>
+      <c r="D8" s="424"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="333"/>
       <c r="B9" s="333"/>
-      <c r="C9" s="424"/>
-      <c r="D9" s="426"/>
+      <c r="C9" s="426"/>
+      <c r="D9" s="424"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="333"/>
       <c r="B10" s="333"/>
-      <c r="C10" s="424"/>
-      <c r="D10" s="426"/>
+      <c r="C10" s="426"/>
+      <c r="D10" s="424"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="333"/>
       <c r="B11" s="333"/>
-      <c r="C11" s="424"/>
-      <c r="D11" s="426"/>
+      <c r="C11" s="426"/>
+      <c r="D11" s="424"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="333"/>
       <c r="B12" s="333"/>
-      <c r="C12" s="424"/>
-      <c r="D12" s="426"/>
+      <c r="C12" s="426"/>
+      <c r="D12" s="424"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="333"/>
       <c r="B13" s="333"/>
-      <c r="C13" s="424"/>
-      <c r="D13" s="426"/>
+      <c r="C13" s="426"/>
+      <c r="D13" s="424"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="333"/>
       <c r="B14" s="333"/>
-      <c r="C14" s="424"/>
-      <c r="D14" s="426"/>
+      <c r="C14" s="426"/>
+      <c r="D14" s="424"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="333"/>
       <c r="B15" s="333"/>
-      <c r="C15" s="424"/>
-      <c r="D15" s="426"/>
+      <c r="C15" s="426"/>
+      <c r="D15" s="424"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="333"/>
       <c r="B16" s="333"/>
-      <c r="C16" s="424"/>
-      <c r="D16" s="426"/>
+      <c r="C16" s="426"/>
+      <c r="D16" s="424"/>
     </row>
     <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A17" s="315"/>
       <c r="B17" s="315"/>
-      <c r="C17" s="425"/>
-      <c r="D17" s="427"/>
+      <c r="C17" s="427"/>
+      <c r="D17" s="425"/>
     </row>
     <row r="18" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="335"/>
@@ -9514,7 +9541,7 @@
       <c r="C18" s="419" t="s">
         <v>361</v>
       </c>
-      <c r="D18" s="426" t="s">
+      <c r="D18" s="424" t="s">
         <v>844</v>
       </c>
     </row>
@@ -9522,115 +9549,115 @@
       <c r="A19" s="335"/>
       <c r="B19" s="335"/>
       <c r="C19" s="419"/>
-      <c r="D19" s="426"/>
+      <c r="D19" s="424"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="335"/>
       <c r="B20" s="335"/>
       <c r="C20" s="419"/>
-      <c r="D20" s="426"/>
+      <c r="D20" s="424"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="335"/>
       <c r="B21" s="335"/>
       <c r="C21" s="419"/>
-      <c r="D21" s="426"/>
+      <c r="D21" s="424"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="335"/>
       <c r="B22" s="335"/>
       <c r="C22" s="419"/>
-      <c r="D22" s="426"/>
+      <c r="D22" s="424"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="335"/>
       <c r="B23" s="335"/>
       <c r="C23" s="419"/>
-      <c r="D23" s="426"/>
+      <c r="D23" s="424"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" s="335"/>
       <c r="B24" s="335"/>
       <c r="C24" s="419"/>
-      <c r="D24" s="426"/>
+      <c r="D24" s="424"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" s="335"/>
       <c r="B25" s="335"/>
       <c r="C25" s="419"/>
-      <c r="D25" s="426"/>
+      <c r="D25" s="424"/>
     </row>
     <row r="26" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="335"/>
       <c r="B26" s="335"/>
       <c r="C26" s="419"/>
-      <c r="D26" s="426"/>
+      <c r="D26" s="424"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="335"/>
       <c r="B27" s="335"/>
       <c r="C27" s="419"/>
-      <c r="D27" s="426"/>
+      <c r="D27" s="424"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="335"/>
       <c r="B28" s="335"/>
       <c r="C28" s="419"/>
-      <c r="D28" s="426"/>
+      <c r="D28" s="424"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="335"/>
       <c r="B29" s="335"/>
       <c r="C29" s="419"/>
-      <c r="D29" s="426"/>
+      <c r="D29" s="424"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="335"/>
       <c r="B30" s="335"/>
       <c r="C30" s="419"/>
-      <c r="D30" s="426"/>
+      <c r="D30" s="424"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="335"/>
       <c r="B31" s="335"/>
       <c r="C31" s="419"/>
-      <c r="D31" s="426"/>
+      <c r="D31" s="424"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="335"/>
       <c r="B32" s="335"/>
       <c r="C32" s="419"/>
-      <c r="D32" s="426"/>
+      <c r="D32" s="424"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="335"/>
       <c r="B33" s="335"/>
       <c r="C33" s="419"/>
-      <c r="D33" s="426"/>
+      <c r="D33" s="424"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="335"/>
       <c r="B34" s="335"/>
       <c r="C34" s="419"/>
-      <c r="D34" s="426"/>
+      <c r="D34" s="424"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="335"/>
       <c r="B35" s="335"/>
       <c r="C35" s="419"/>
-      <c r="D35" s="426"/>
+      <c r="D35" s="424"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="335"/>
       <c r="B36" s="335"/>
       <c r="C36" s="419"/>
-      <c r="D36" s="426"/>
+      <c r="D36" s="424"/>
     </row>
     <row r="37" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A37" s="316"/>
       <c r="B37" s="316"/>
       <c r="C37" s="420"/>
-      <c r="D37" s="427"/>
+      <c r="D37" s="425"/>
     </row>
     <row r="38" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="334"/>
@@ -9638,7 +9665,7 @@
       <c r="C38" s="419" t="s">
         <v>845</v>
       </c>
-      <c r="D38" s="426" t="s">
+      <c r="D38" s="424" t="s">
         <v>846</v>
       </c>
     </row>
@@ -9646,115 +9673,115 @@
       <c r="A39" s="334"/>
       <c r="B39" s="334"/>
       <c r="C39" s="419"/>
-      <c r="D39" s="426"/>
+      <c r="D39" s="424"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A40" s="334"/>
       <c r="B40" s="334"/>
       <c r="C40" s="419"/>
-      <c r="D40" s="426"/>
+      <c r="D40" s="424"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A41" s="334"/>
       <c r="B41" s="334"/>
       <c r="C41" s="419"/>
-      <c r="D41" s="426"/>
+      <c r="D41" s="424"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A42" s="334"/>
       <c r="B42" s="334"/>
       <c r="C42" s="419"/>
-      <c r="D42" s="426"/>
+      <c r="D42" s="424"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A43" s="334"/>
       <c r="B43" s="334"/>
       <c r="C43" s="419"/>
-      <c r="D43" s="426"/>
+      <c r="D43" s="424"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A44" s="334"/>
       <c r="B44" s="334"/>
       <c r="C44" s="419"/>
-      <c r="D44" s="426"/>
+      <c r="D44" s="424"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A45" s="334"/>
       <c r="B45" s="334"/>
       <c r="C45" s="419"/>
-      <c r="D45" s="426"/>
+      <c r="D45" s="424"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A46" s="334"/>
       <c r="B46" s="334"/>
       <c r="C46" s="419"/>
-      <c r="D46" s="426"/>
+      <c r="D46" s="424"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A47" s="334"/>
       <c r="B47" s="334"/>
       <c r="C47" s="419"/>
-      <c r="D47" s="426"/>
+      <c r="D47" s="424"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A48" s="334"/>
       <c r="B48" s="334"/>
       <c r="C48" s="419"/>
-      <c r="D48" s="426"/>
+      <c r="D48" s="424"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A49" s="334"/>
       <c r="B49" s="334"/>
       <c r="C49" s="419"/>
-      <c r="D49" s="426"/>
+      <c r="D49" s="424"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A50" s="334"/>
       <c r="B50" s="334"/>
       <c r="C50" s="419"/>
-      <c r="D50" s="426"/>
+      <c r="D50" s="424"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A51" s="334"/>
       <c r="B51" s="334"/>
       <c r="C51" s="419"/>
-      <c r="D51" s="426"/>
+      <c r="D51" s="424"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A52" s="334"/>
       <c r="B52" s="334"/>
       <c r="C52" s="419"/>
-      <c r="D52" s="426"/>
+      <c r="D52" s="424"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" s="334"/>
       <c r="B53" s="334"/>
       <c r="C53" s="419"/>
-      <c r="D53" s="426"/>
+      <c r="D53" s="424"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A54" s="334"/>
       <c r="B54" s="334"/>
       <c r="C54" s="419"/>
-      <c r="D54" s="426"/>
+      <c r="D54" s="424"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A55" s="334"/>
       <c r="B55" s="334"/>
       <c r="C55" s="419"/>
-      <c r="D55" s="426"/>
+      <c r="D55" s="424"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A56" s="334"/>
       <c r="B56" s="334"/>
       <c r="C56" s="419"/>
-      <c r="D56" s="426"/>
+      <c r="D56" s="424"/>
     </row>
     <row r="57" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A57" s="317"/>
       <c r="B57" s="317"/>
       <c r="C57" s="420"/>
-      <c r="D57" s="427"/>
+      <c r="D57" s="425"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A58" s="336"/>
@@ -9762,7 +9789,7 @@
       <c r="C58" s="419" t="s">
         <v>847</v>
       </c>
-      <c r="D58" s="426" t="s">
+      <c r="D58" s="424" t="s">
         <v>848</v>
       </c>
     </row>
@@ -9770,85 +9797,85 @@
       <c r="A59" s="336"/>
       <c r="B59" s="336"/>
       <c r="C59" s="419"/>
-      <c r="D59" s="426"/>
+      <c r="D59" s="424"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A60" s="336"/>
       <c r="B60" s="336"/>
       <c r="C60" s="419"/>
-      <c r="D60" s="426"/>
+      <c r="D60" s="424"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A61" s="336"/>
       <c r="B61" s="336"/>
       <c r="C61" s="419"/>
-      <c r="D61" s="426"/>
+      <c r="D61" s="424"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A62" s="336"/>
       <c r="B62" s="336"/>
       <c r="C62" s="419"/>
-      <c r="D62" s="426"/>
+      <c r="D62" s="424"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A63" s="336"/>
       <c r="B63" s="336"/>
       <c r="C63" s="419"/>
-      <c r="D63" s="426"/>
+      <c r="D63" s="424"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A64" s="336"/>
       <c r="B64" s="336"/>
       <c r="C64" s="419"/>
-      <c r="D64" s="426"/>
+      <c r="D64" s="424"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A65" s="336"/>
       <c r="B65" s="336"/>
       <c r="C65" s="419"/>
-      <c r="D65" s="426"/>
+      <c r="D65" s="424"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A66" s="336"/>
       <c r="B66" s="336"/>
       <c r="C66" s="419"/>
-      <c r="D66" s="426"/>
+      <c r="D66" s="424"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A67" s="336"/>
       <c r="B67" s="336"/>
       <c r="C67" s="419"/>
-      <c r="D67" s="426"/>
+      <c r="D67" s="424"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A68" s="336"/>
       <c r="B68" s="336"/>
       <c r="C68" s="419"/>
-      <c r="D68" s="426"/>
+      <c r="D68" s="424"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A69" s="336"/>
       <c r="B69" s="336"/>
       <c r="C69" s="419"/>
-      <c r="D69" s="426"/>
+      <c r="D69" s="424"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A70" s="336"/>
       <c r="B70" s="336"/>
       <c r="C70" s="419"/>
-      <c r="D70" s="426"/>
+      <c r="D70" s="424"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A71" s="336"/>
       <c r="B71" s="336"/>
       <c r="C71" s="419"/>
-      <c r="D71" s="426"/>
+      <c r="D71" s="424"/>
     </row>
     <row r="72" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A72" s="318"/>
       <c r="B72" s="318"/>
       <c r="C72" s="420"/>
-      <c r="D72" s="427"/>
+      <c r="D72" s="425"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A73" s="338"/>
@@ -9856,7 +9883,7 @@
       <c r="C73" s="419" t="s">
         <v>849</v>
       </c>
-      <c r="D73" s="426" t="s">
+      <c r="D73" s="424" t="s">
         <v>850</v>
       </c>
     </row>
@@ -9864,97 +9891,97 @@
       <c r="A74" s="338"/>
       <c r="B74" s="338"/>
       <c r="C74" s="419"/>
-      <c r="D74" s="426"/>
+      <c r="D74" s="424"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A75" s="338"/>
       <c r="B75" s="338"/>
       <c r="C75" s="419"/>
-      <c r="D75" s="426"/>
+      <c r="D75" s="424"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A76" s="338"/>
       <c r="B76" s="338"/>
       <c r="C76" s="419"/>
-      <c r="D76" s="426"/>
+      <c r="D76" s="424"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A77" s="338"/>
       <c r="B77" s="338"/>
       <c r="C77" s="419"/>
-      <c r="D77" s="426"/>
+      <c r="D77" s="424"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A78" s="338"/>
       <c r="B78" s="338"/>
       <c r="C78" s="419"/>
-      <c r="D78" s="426"/>
+      <c r="D78" s="424"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A79" s="338"/>
       <c r="B79" s="338"/>
       <c r="C79" s="419"/>
-      <c r="D79" s="426"/>
+      <c r="D79" s="424"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A80" s="338"/>
       <c r="B80" s="338"/>
       <c r="C80" s="419"/>
-      <c r="D80" s="426"/>
+      <c r="D80" s="424"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A81" s="338"/>
       <c r="B81" s="338"/>
       <c r="C81" s="419"/>
-      <c r="D81" s="426"/>
+      <c r="D81" s="424"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A82" s="338"/>
       <c r="B82" s="338"/>
       <c r="C82" s="419"/>
-      <c r="D82" s="426"/>
+      <c r="D82" s="424"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A83" s="338"/>
       <c r="B83" s="338"/>
       <c r="C83" s="419"/>
-      <c r="D83" s="426"/>
+      <c r="D83" s="424"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A84" s="338"/>
       <c r="B84" s="338"/>
       <c r="C84" s="419"/>
-      <c r="D84" s="426"/>
+      <c r="D84" s="424"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A85" s="338"/>
       <c r="B85" s="338"/>
       <c r="C85" s="419"/>
-      <c r="D85" s="426"/>
+      <c r="D85" s="424"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A86" s="338"/>
       <c r="B86" s="338"/>
       <c r="C86" s="419"/>
-      <c r="D86" s="426"/>
+      <c r="D86" s="424"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A87" s="338"/>
       <c r="B87" s="338"/>
       <c r="C87" s="419"/>
-      <c r="D87" s="426"/>
+      <c r="D87" s="424"/>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A88" s="338"/>
       <c r="B88" s="338"/>
       <c r="C88" s="419"/>
-      <c r="D88" s="426"/>
+      <c r="D88" s="424"/>
     </row>
     <row r="89" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A89" s="319"/>
       <c r="B89" s="319"/>
       <c r="C89" s="420"/>
-      <c r="D89" s="427"/>
+      <c r="D89" s="425"/>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A90" s="337"/>
@@ -9962,7 +9989,7 @@
       <c r="C90" s="419" t="s">
         <v>851</v>
       </c>
-      <c r="D90" s="426" t="s">
+      <c r="D90" s="424" t="s">
         <v>852</v>
       </c>
     </row>
@@ -9970,49 +9997,49 @@
       <c r="A91" s="337"/>
       <c r="B91" s="337"/>
       <c r="C91" s="419"/>
-      <c r="D91" s="426"/>
+      <c r="D91" s="424"/>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A92" s="337"/>
       <c r="B92" s="337"/>
       <c r="C92" s="419"/>
-      <c r="D92" s="426"/>
+      <c r="D92" s="424"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A93" s="337"/>
       <c r="B93" s="337"/>
       <c r="C93" s="419"/>
-      <c r="D93" s="426"/>
+      <c r="D93" s="424"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A94" s="337"/>
       <c r="B94" s="337"/>
       <c r="C94" s="419"/>
-      <c r="D94" s="426"/>
+      <c r="D94" s="424"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A95" s="337"/>
       <c r="B95" s="337"/>
       <c r="C95" s="419"/>
-      <c r="D95" s="426"/>
+      <c r="D95" s="424"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A96" s="337"/>
       <c r="B96" s="337"/>
       <c r="C96" s="419"/>
-      <c r="D96" s="426"/>
+      <c r="D96" s="424"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A97" s="337"/>
       <c r="B97" s="337"/>
       <c r="C97" s="419"/>
-      <c r="D97" s="426"/>
+      <c r="D97" s="424"/>
     </row>
     <row r="98" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A98" s="320"/>
       <c r="B98" s="320"/>
       <c r="C98" s="420"/>
-      <c r="D98" s="427"/>
+      <c r="D98" s="425"/>
     </row>
     <row r="99" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A99" s="339"/>
@@ -10020,7 +10047,7 @@
       <c r="C99" s="422" t="s">
         <v>853</v>
       </c>
-      <c r="D99" s="426" t="s">
+      <c r="D99" s="424" t="s">
         <v>854</v>
       </c>
     </row>
@@ -10028,73 +10055,73 @@
       <c r="A100" s="339"/>
       <c r="B100" s="339"/>
       <c r="C100" s="422"/>
-      <c r="D100" s="426"/>
+      <c r="D100" s="424"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A101" s="339"/>
       <c r="B101" s="339"/>
       <c r="C101" s="422"/>
-      <c r="D101" s="426"/>
+      <c r="D101" s="424"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A102" s="339"/>
       <c r="B102" s="339"/>
       <c r="C102" s="422"/>
-      <c r="D102" s="426"/>
+      <c r="D102" s="424"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A103" s="339"/>
       <c r="B103" s="339"/>
       <c r="C103" s="422"/>
-      <c r="D103" s="426"/>
+      <c r="D103" s="424"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A104" s="339"/>
       <c r="B104" s="339"/>
       <c r="C104" s="422"/>
-      <c r="D104" s="426"/>
+      <c r="D104" s="424"/>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A105" s="339"/>
       <c r="B105" s="339"/>
       <c r="C105" s="422"/>
-      <c r="D105" s="426"/>
+      <c r="D105" s="424"/>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A106" s="339"/>
       <c r="B106" s="339"/>
       <c r="C106" s="422"/>
-      <c r="D106" s="426"/>
+      <c r="D106" s="424"/>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A107" s="339"/>
       <c r="B107" s="339"/>
       <c r="C107" s="422"/>
-      <c r="D107" s="426"/>
+      <c r="D107" s="424"/>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A108" s="339"/>
       <c r="B108" s="339"/>
       <c r="C108" s="422"/>
-      <c r="D108" s="426"/>
+      <c r="D108" s="424"/>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A109" s="339"/>
       <c r="B109" s="339"/>
       <c r="C109" s="422"/>
-      <c r="D109" s="426"/>
+      <c r="D109" s="424"/>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A110" s="339"/>
       <c r="B110" s="339"/>
       <c r="C110" s="422"/>
-      <c r="D110" s="426"/>
+      <c r="D110" s="424"/>
     </row>
     <row r="111" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A111" s="321"/>
       <c r="B111" s="321"/>
       <c r="C111" s="423"/>
-      <c r="D111" s="427"/>
+      <c r="D111" s="425"/>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A112" s="335"/>
@@ -10102,7 +10129,7 @@
       <c r="C112" s="419" t="s">
         <v>855</v>
       </c>
-      <c r="D112" s="426" t="s">
+      <c r="D112" s="424" t="s">
         <v>856</v>
       </c>
     </row>
@@ -10110,67 +10137,67 @@
       <c r="A113" s="335"/>
       <c r="B113" s="335"/>
       <c r="C113" s="419"/>
-      <c r="D113" s="426"/>
+      <c r="D113" s="424"/>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A114" s="335"/>
       <c r="B114" s="335"/>
       <c r="C114" s="419"/>
-      <c r="D114" s="426"/>
+      <c r="D114" s="424"/>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A115" s="335"/>
       <c r="B115" s="335"/>
       <c r="C115" s="419"/>
-      <c r="D115" s="426"/>
+      <c r="D115" s="424"/>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A116" s="335"/>
       <c r="B116" s="335"/>
       <c r="C116" s="419"/>
-      <c r="D116" s="426"/>
+      <c r="D116" s="424"/>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A117" s="335"/>
       <c r="B117" s="335"/>
       <c r="C117" s="419"/>
-      <c r="D117" s="426"/>
+      <c r="D117" s="424"/>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A118" s="335"/>
       <c r="B118" s="335"/>
       <c r="C118" s="419"/>
-      <c r="D118" s="426"/>
+      <c r="D118" s="424"/>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A119" s="335"/>
       <c r="B119" s="335"/>
       <c r="C119" s="419"/>
-      <c r="D119" s="426"/>
+      <c r="D119" s="424"/>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A120" s="335"/>
       <c r="B120" s="335"/>
       <c r="C120" s="419"/>
-      <c r="D120" s="426"/>
+      <c r="D120" s="424"/>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A121" s="335"/>
       <c r="B121" s="335"/>
       <c r="C121" s="419"/>
-      <c r="D121" s="426"/>
+      <c r="D121" s="424"/>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A122" s="335"/>
       <c r="B122" s="335"/>
       <c r="C122" s="419"/>
-      <c r="D122" s="426"/>
+      <c r="D122" s="424"/>
     </row>
     <row r="123" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A123" s="316"/>
       <c r="B123" s="316"/>
       <c r="C123" s="420"/>
-      <c r="D123" s="427"/>
+      <c r="D123" s="425"/>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A124" s="334"/>
@@ -10178,7 +10205,7 @@
       <c r="C124" s="419" t="s">
         <v>857</v>
       </c>
-      <c r="D124" s="426" t="s">
+      <c r="D124" s="424" t="s">
         <v>858</v>
       </c>
     </row>
@@ -10186,31 +10213,31 @@
       <c r="A125" s="334"/>
       <c r="B125" s="334"/>
       <c r="C125" s="419"/>
-      <c r="D125" s="426"/>
+      <c r="D125" s="424"/>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A126" s="334"/>
       <c r="B126" s="334"/>
       <c r="C126" s="419"/>
-      <c r="D126" s="426"/>
+      <c r="D126" s="424"/>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A127" s="334"/>
       <c r="B127" s="334"/>
       <c r="C127" s="419"/>
-      <c r="D127" s="426"/>
+      <c r="D127" s="424"/>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A128" s="334"/>
       <c r="B128" s="334"/>
       <c r="C128" s="419"/>
-      <c r="D128" s="426"/>
+      <c r="D128" s="424"/>
     </row>
     <row r="129" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A129" s="317"/>
       <c r="B129" s="317"/>
       <c r="C129" s="420"/>
-      <c r="D129" s="427"/>
+      <c r="D129" s="425"/>
     </row>
     <row r="130" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A130" s="33"/>
@@ -10218,7 +10245,7 @@
       <c r="C130" s="419" t="s">
         <v>859</v>
       </c>
-      <c r="D130" s="426" t="s">
+      <c r="D130" s="424" t="s">
         <v>860</v>
       </c>
     </row>
@@ -10226,19 +10253,19 @@
       <c r="A131" s="33"/>
       <c r="B131" s="33"/>
       <c r="C131" s="419"/>
-      <c r="D131" s="426"/>
+      <c r="D131" s="424"/>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A132" s="33"/>
       <c r="B132" s="33"/>
       <c r="C132" s="419"/>
-      <c r="D132" s="426"/>
+      <c r="D132" s="424"/>
     </row>
     <row r="133" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A133" s="322"/>
       <c r="B133" s="322"/>
       <c r="C133" s="420"/>
-      <c r="D133" s="427"/>
+      <c r="D133" s="425"/>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A134" s="338"/>
@@ -10246,7 +10273,7 @@
       <c r="C134" s="419" t="s">
         <v>861</v>
       </c>
-      <c r="D134" s="426" t="s">
+      <c r="D134" s="424" t="s">
         <v>862</v>
       </c>
     </row>
@@ -10254,103 +10281,103 @@
       <c r="A135" s="338"/>
       <c r="B135" s="338"/>
       <c r="C135" s="419"/>
-      <c r="D135" s="426"/>
+      <c r="D135" s="424"/>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A136" s="338"/>
       <c r="B136" s="338"/>
       <c r="C136" s="419"/>
-      <c r="D136" s="426"/>
+      <c r="D136" s="424"/>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A137" s="338"/>
       <c r="B137" s="338"/>
       <c r="C137" s="419"/>
-      <c r="D137" s="426"/>
+      <c r="D137" s="424"/>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A138" s="338"/>
       <c r="B138" s="338"/>
       <c r="C138" s="419"/>
-      <c r="D138" s="426"/>
+      <c r="D138" s="424"/>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A139" s="338"/>
       <c r="B139" s="338"/>
       <c r="C139" s="419"/>
-      <c r="D139" s="426"/>
+      <c r="D139" s="424"/>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A140" s="338"/>
       <c r="B140" s="338"/>
       <c r="C140" s="419"/>
-      <c r="D140" s="426"/>
+      <c r="D140" s="424"/>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A141" s="338"/>
       <c r="B141" s="338"/>
       <c r="C141" s="419"/>
-      <c r="D141" s="426"/>
+      <c r="D141" s="424"/>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A142" s="338"/>
       <c r="B142" s="338"/>
       <c r="C142" s="419"/>
-      <c r="D142" s="426"/>
+      <c r="D142" s="424"/>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A143" s="338"/>
       <c r="B143" s="338"/>
       <c r="C143" s="419"/>
-      <c r="D143" s="426"/>
+      <c r="D143" s="424"/>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A144" s="338"/>
       <c r="B144" s="338"/>
       <c r="C144" s="419"/>
-      <c r="D144" s="426"/>
+      <c r="D144" s="424"/>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A145" s="338"/>
       <c r="B145" s="338"/>
       <c r="C145" s="419"/>
-      <c r="D145" s="426"/>
+      <c r="D145" s="424"/>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A146" s="338"/>
       <c r="B146" s="338"/>
       <c r="C146" s="419"/>
-      <c r="D146" s="426"/>
+      <c r="D146" s="424"/>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A147" s="338"/>
       <c r="B147" s="338"/>
       <c r="C147" s="419"/>
-      <c r="D147" s="426"/>
+      <c r="D147" s="424"/>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A148" s="338"/>
       <c r="B148" s="338"/>
       <c r="C148" s="419"/>
-      <c r="D148" s="426"/>
+      <c r="D148" s="424"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A149" s="338"/>
       <c r="B149" s="338"/>
       <c r="C149" s="419"/>
-      <c r="D149" s="426"/>
+      <c r="D149" s="424"/>
     </row>
     <row r="150" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A150" s="338"/>
       <c r="B150" s="338"/>
       <c r="C150" s="419"/>
-      <c r="D150" s="426"/>
+      <c r="D150" s="424"/>
     </row>
     <row r="151" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A151" s="319"/>
       <c r="B151" s="319"/>
       <c r="C151" s="420"/>
-      <c r="D151" s="427"/>
+      <c r="D151" s="425"/>
     </row>
     <row r="152" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A152" s="340"/>
@@ -10358,7 +10385,7 @@
       <c r="C152" s="419" t="s">
         <v>863</v>
       </c>
-      <c r="D152" s="426" t="s">
+      <c r="D152" s="424" t="s">
         <v>864</v>
       </c>
     </row>
@@ -10366,47 +10393,47 @@
       <c r="A153" s="340"/>
       <c r="B153" s="340"/>
       <c r="C153" s="419"/>
-      <c r="D153" s="426"/>
+      <c r="D153" s="424"/>
     </row>
     <row r="154" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A154" s="340"/>
       <c r="B154" s="340"/>
       <c r="C154" s="419"/>
-      <c r="D154" s="426"/>
+      <c r="D154" s="424"/>
     </row>
     <row r="155" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A155" s="323"/>
       <c r="B155" s="323"/>
       <c r="C155" s="420"/>
-      <c r="D155" s="427"/>
+      <c r="D155" s="425"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="24">
+    <mergeCell ref="C2:C17"/>
+    <mergeCell ref="D2:D17"/>
+    <mergeCell ref="C18:C37"/>
+    <mergeCell ref="D18:D37"/>
+    <mergeCell ref="C38:C57"/>
+    <mergeCell ref="D38:D57"/>
+    <mergeCell ref="C58:C72"/>
+    <mergeCell ref="D58:D72"/>
+    <mergeCell ref="C73:C89"/>
+    <mergeCell ref="D73:D89"/>
+    <mergeCell ref="C90:C98"/>
+    <mergeCell ref="D90:D98"/>
+    <mergeCell ref="C99:C111"/>
+    <mergeCell ref="D99:D111"/>
+    <mergeCell ref="C112:C123"/>
+    <mergeCell ref="D112:D123"/>
+    <mergeCell ref="C124:C129"/>
+    <mergeCell ref="D124:D129"/>
     <mergeCell ref="C130:C133"/>
     <mergeCell ref="D130:D133"/>
     <mergeCell ref="C134:C151"/>
     <mergeCell ref="D134:D151"/>
     <mergeCell ref="C152:C155"/>
     <mergeCell ref="D152:D155"/>
-    <mergeCell ref="C99:C111"/>
-    <mergeCell ref="D99:D111"/>
-    <mergeCell ref="C112:C123"/>
-    <mergeCell ref="D112:D123"/>
-    <mergeCell ref="C124:C129"/>
-    <mergeCell ref="D124:D129"/>
-    <mergeCell ref="C58:C72"/>
-    <mergeCell ref="D58:D72"/>
-    <mergeCell ref="C73:C89"/>
-    <mergeCell ref="D73:D89"/>
-    <mergeCell ref="C90:C98"/>
-    <mergeCell ref="D90:D98"/>
-    <mergeCell ref="C2:C17"/>
-    <mergeCell ref="D2:D17"/>
-    <mergeCell ref="C18:C37"/>
-    <mergeCell ref="D18:D37"/>
-    <mergeCell ref="C38:C57"/>
-    <mergeCell ref="D38:D57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -11744,21 +11771,21 @@
   <sheetData>
     <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="33"/>
-      <c r="B1" s="406" t="s">
+      <c r="B1" s="411" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="407"/>
-      <c r="D1" s="408"/>
-      <c r="E1" s="406" t="s">
+      <c r="C1" s="412"/>
+      <c r="D1" s="413"/>
+      <c r="E1" s="411" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="407"/>
-      <c r="G1" s="407"/>
+      <c r="F1" s="412"/>
+      <c r="G1" s="412"/>
       <c r="H1" s="309"/>
-      <c r="K1" s="409" t="s">
+      <c r="K1" s="414" t="s">
         <v>836</v>
       </c>
-      <c r="L1" s="410"/>
+      <c r="L1" s="415"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A2" s="61" t="s">
@@ -12846,103 +12873,103 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:67" x14ac:dyDescent="0.4">
-      <c r="A1" s="400" t="s">
+      <c r="A1" s="399" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="400"/>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="401" t="s">
+      <c r="B1" s="399"/>
+      <c r="C1" s="399"/>
+      <c r="D1" s="399"/>
+      <c r="E1" s="400" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="402"/>
-      <c r="I1" s="402"/>
-      <c r="J1" s="402"/>
-      <c r="K1" s="402"/>
-      <c r="L1" s="402"/>
-      <c r="M1" s="402"/>
-      <c r="N1" s="402"/>
-      <c r="O1" s="403"/>
-      <c r="P1" s="399" t="s">
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="401"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="401"/>
+      <c r="O1" s="402"/>
+      <c r="P1" s="416" t="s">
         <v>77</v>
       </c>
-      <c r="Q1" s="399"/>
-      <c r="R1" s="399"/>
-      <c r="S1" s="399"/>
-      <c r="T1" s="400" t="s">
+      <c r="Q1" s="416"/>
+      <c r="R1" s="416"/>
+      <c r="S1" s="416"/>
+      <c r="T1" s="399" t="s">
         <v>78</v>
       </c>
-      <c r="U1" s="400"/>
-      <c r="V1" s="400"/>
-      <c r="W1" s="400"/>
-      <c r="X1" s="399" t="s">
+      <c r="U1" s="399"/>
+      <c r="V1" s="399"/>
+      <c r="W1" s="399"/>
+      <c r="X1" s="416" t="s">
         <v>79</v>
       </c>
-      <c r="Y1" s="399"/>
-      <c r="Z1" s="399"/>
-      <c r="AA1" s="399"/>
-      <c r="AB1" s="400" t="s">
+      <c r="Y1" s="416"/>
+      <c r="Z1" s="416"/>
+      <c r="AA1" s="416"/>
+      <c r="AB1" s="399" t="s">
         <v>80</v>
       </c>
-      <c r="AC1" s="400"/>
-      <c r="AD1" s="400"/>
-      <c r="AE1" s="400"/>
-      <c r="AF1" s="399" t="s">
+      <c r="AC1" s="399"/>
+      <c r="AD1" s="399"/>
+      <c r="AE1" s="399"/>
+      <c r="AF1" s="416" t="s">
         <v>81</v>
       </c>
-      <c r="AG1" s="399"/>
-      <c r="AH1" s="399"/>
-      <c r="AI1" s="399"/>
-      <c r="AJ1" s="400" t="s">
+      <c r="AG1" s="416"/>
+      <c r="AH1" s="416"/>
+      <c r="AI1" s="416"/>
+      <c r="AJ1" s="399" t="s">
         <v>82</v>
       </c>
-      <c r="AK1" s="400"/>
-      <c r="AL1" s="400"/>
-      <c r="AM1" s="400"/>
-      <c r="AN1" s="399" t="s">
+      <c r="AK1" s="399"/>
+      <c r="AL1" s="399"/>
+      <c r="AM1" s="399"/>
+      <c r="AN1" s="416" t="s">
         <v>83</v>
       </c>
-      <c r="AO1" s="399"/>
-      <c r="AP1" s="399"/>
-      <c r="AQ1" s="399"/>
-      <c r="AR1" s="400" t="s">
+      <c r="AO1" s="416"/>
+      <c r="AP1" s="416"/>
+      <c r="AQ1" s="416"/>
+      <c r="AR1" s="399" t="s">
         <v>84</v>
       </c>
-      <c r="AS1" s="400"/>
-      <c r="AT1" s="400"/>
-      <c r="AU1" s="400"/>
-      <c r="AV1" s="399" t="s">
+      <c r="AS1" s="399"/>
+      <c r="AT1" s="399"/>
+      <c r="AU1" s="399"/>
+      <c r="AV1" s="416" t="s">
         <v>85</v>
       </c>
-      <c r="AW1" s="399"/>
-      <c r="AX1" s="399"/>
-      <c r="AY1" s="399"/>
-      <c r="AZ1" s="400" t="s">
+      <c r="AW1" s="416"/>
+      <c r="AX1" s="416"/>
+      <c r="AY1" s="416"/>
+      <c r="AZ1" s="399" t="s">
         <v>86</v>
       </c>
-      <c r="BA1" s="400"/>
-      <c r="BB1" s="400"/>
-      <c r="BC1" s="400"/>
-      <c r="BD1" s="399" t="s">
+      <c r="BA1" s="399"/>
+      <c r="BB1" s="399"/>
+      <c r="BC1" s="399"/>
+      <c r="BD1" s="416" t="s">
         <v>87</v>
       </c>
-      <c r="BE1" s="399"/>
-      <c r="BF1" s="399"/>
-      <c r="BG1" s="399"/>
-      <c r="BH1" s="400" t="s">
+      <c r="BE1" s="416"/>
+      <c r="BF1" s="416"/>
+      <c r="BG1" s="416"/>
+      <c r="BH1" s="399" t="s">
         <v>88</v>
       </c>
-      <c r="BI1" s="400"/>
-      <c r="BJ1" s="400"/>
-      <c r="BK1" s="400"/>
-      <c r="BL1" s="399" t="s">
+      <c r="BI1" s="399"/>
+      <c r="BJ1" s="399"/>
+      <c r="BK1" s="399"/>
+      <c r="BL1" s="416" t="s">
         <v>495</v>
       </c>
-      <c r="BM1" s="399"/>
-      <c r="BN1" s="399"/>
-      <c r="BO1" s="399"/>
+      <c r="BM1" s="416"/>
+      <c r="BN1" s="416"/>
+      <c r="BO1" s="416"/>
     </row>
     <row r="2" spans="1:67" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -19965,7 +19992,7 @@
         <v>1</v>
       </c>
       <c r="D59" s="79" t="s">
-        <v>728</v>
+        <v>947</v>
       </c>
       <c r="E59" s="81">
         <f t="shared" si="18"/>
@@ -20108,7 +20135,7 @@
         <v>1</v>
       </c>
       <c r="D60" s="79" t="s">
-        <v>729</v>
+        <v>948</v>
       </c>
       <c r="E60" s="81">
         <f t="shared" si="18"/>
@@ -20252,7 +20279,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="79" t="s">
-        <v>730</v>
+        <v>949</v>
       </c>
       <c r="E61" s="81">
         <f t="shared" si="18"/>
@@ -34352,7 +34379,7 @@
         <v>1</v>
       </c>
       <c r="D179" s="79" t="s">
-        <v>924</v>
+        <v>950</v>
       </c>
       <c r="E179" s="81">
         <f t="shared" si="72"/>
@@ -34467,7 +34494,7 @@
         <v>1</v>
       </c>
       <c r="D180" s="79" t="s">
-        <v>925</v>
+        <v>951</v>
       </c>
       <c r="E180" s="81">
         <f t="shared" si="72"/>
@@ -35303,96 +35330,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:94" x14ac:dyDescent="0.4">
-      <c r="A1" s="400" t="s">
+      <c r="A1" s="399" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="400"/>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="401" t="s">
+      <c r="B1" s="399"/>
+      <c r="C1" s="399"/>
+      <c r="D1" s="399"/>
+      <c r="E1" s="400" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="402"/>
-      <c r="I1" s="402"/>
-      <c r="J1" s="402"/>
-      <c r="K1" s="402"/>
-      <c r="L1" s="402"/>
-      <c r="M1" s="402"/>
-      <c r="N1" s="403"/>
-      <c r="O1" s="414" t="s">
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="401"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="402"/>
+      <c r="O1" s="406" t="s">
         <v>77</v>
       </c>
-      <c r="P1" s="415"/>
-      <c r="Q1" s="415"/>
-      <c r="R1" s="416"/>
-      <c r="S1" s="401" t="s">
+      <c r="P1" s="407"/>
+      <c r="Q1" s="407"/>
+      <c r="R1" s="408"/>
+      <c r="S1" s="400" t="s">
         <v>78</v>
       </c>
-      <c r="T1" s="402"/>
-      <c r="U1" s="402"/>
-      <c r="V1" s="402"/>
-      <c r="W1" s="414" t="s">
+      <c r="T1" s="401"/>
+      <c r="U1" s="401"/>
+      <c r="V1" s="401"/>
+      <c r="W1" s="406" t="s">
         <v>79</v>
       </c>
-      <c r="X1" s="415"/>
-      <c r="Y1" s="415"/>
-      <c r="Z1" s="416"/>
-      <c r="AA1" s="411" t="s">
+      <c r="X1" s="407"/>
+      <c r="Y1" s="407"/>
+      <c r="Z1" s="408"/>
+      <c r="AA1" s="403" t="s">
         <v>80</v>
       </c>
-      <c r="AB1" s="412"/>
-      <c r="AC1" s="412"/>
-      <c r="AD1" s="413"/>
-      <c r="AE1" s="414" t="s">
+      <c r="AB1" s="404"/>
+      <c r="AC1" s="404"/>
+      <c r="AD1" s="405"/>
+      <c r="AE1" s="406" t="s">
         <v>81</v>
       </c>
-      <c r="AF1" s="415"/>
-      <c r="AG1" s="415"/>
-      <c r="AH1" s="416"/>
-      <c r="AI1" s="411" t="s">
+      <c r="AF1" s="407"/>
+      <c r="AG1" s="407"/>
+      <c r="AH1" s="408"/>
+      <c r="AI1" s="403" t="s">
         <v>82</v>
       </c>
-      <c r="AJ1" s="412"/>
-      <c r="AK1" s="412"/>
-      <c r="AL1" s="413"/>
-      <c r="AM1" s="414" t="s">
+      <c r="AJ1" s="404"/>
+      <c r="AK1" s="404"/>
+      <c r="AL1" s="405"/>
+      <c r="AM1" s="406" t="s">
         <v>83</v>
       </c>
-      <c r="AN1" s="415"/>
-      <c r="AO1" s="415"/>
-      <c r="AP1" s="416"/>
-      <c r="AQ1" s="411" t="s">
+      <c r="AN1" s="407"/>
+      <c r="AO1" s="407"/>
+      <c r="AP1" s="408"/>
+      <c r="AQ1" s="403" t="s">
         <v>84</v>
       </c>
-      <c r="AR1" s="412"/>
-      <c r="AS1" s="412"/>
-      <c r="AT1" s="413"/>
-      <c r="AU1" s="414" t="s">
+      <c r="AR1" s="404"/>
+      <c r="AS1" s="404"/>
+      <c r="AT1" s="405"/>
+      <c r="AU1" s="406" t="s">
         <v>85</v>
       </c>
-      <c r="AV1" s="415"/>
-      <c r="AW1" s="415"/>
-      <c r="AX1" s="416"/>
-      <c r="AY1" s="411" t="s">
+      <c r="AV1" s="407"/>
+      <c r="AW1" s="407"/>
+      <c r="AX1" s="408"/>
+      <c r="AY1" s="403" t="s">
         <v>86</v>
       </c>
-      <c r="AZ1" s="412"/>
-      <c r="BA1" s="412"/>
-      <c r="BB1" s="413"/>
-      <c r="BC1" s="414" t="s">
+      <c r="AZ1" s="404"/>
+      <c r="BA1" s="404"/>
+      <c r="BB1" s="405"/>
+      <c r="BC1" s="406" t="s">
         <v>87</v>
       </c>
-      <c r="BD1" s="415"/>
-      <c r="BE1" s="415"/>
-      <c r="BF1" s="416"/>
-      <c r="BG1" s="411" t="s">
+      <c r="BD1" s="407"/>
+      <c r="BE1" s="407"/>
+      <c r="BF1" s="408"/>
+      <c r="BG1" s="403" t="s">
         <v>88</v>
       </c>
-      <c r="BH1" s="412"/>
-      <c r="BI1" s="412"/>
-      <c r="BJ1" s="413"/>
+      <c r="BH1" s="404"/>
+      <c r="BI1" s="404"/>
+      <c r="BJ1" s="405"/>
     </row>
     <row r="2" spans="1:94" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -40028,7 +40055,7 @@
         <v>1</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>252</v>
+        <v>954</v>
       </c>
       <c r="E45" s="5">
         <f t="shared" si="3"/>
@@ -40171,7 +40198,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>748</v>
+        <v>955</v>
       </c>
       <c r="E46" s="5">
         <f t="shared" si="3"/>
@@ -45219,7 +45246,7 @@
         <v>1</v>
       </c>
       <c r="D89" s="118" t="s">
-        <v>926</v>
+        <v>952</v>
       </c>
       <c r="E89" s="5">
         <f t="shared" si="29"/>
@@ -45317,7 +45344,7 @@
         <v>1</v>
       </c>
       <c r="D90" s="118" t="s">
-        <v>927</v>
+        <v>953</v>
       </c>
       <c r="E90" s="5">
         <f t="shared" si="29"/>
@@ -45806,97 +45833,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:63" x14ac:dyDescent="0.4">
-      <c r="A1" s="400" t="s">
+      <c r="A1" s="399" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="400"/>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="401" t="s">
+      <c r="B1" s="399"/>
+      <c r="C1" s="399"/>
+      <c r="D1" s="399"/>
+      <c r="E1" s="400" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="402"/>
-      <c r="I1" s="402"/>
-      <c r="J1" s="402"/>
-      <c r="K1" s="402"/>
-      <c r="L1" s="402"/>
-      <c r="M1" s="402"/>
-      <c r="N1" s="402"/>
-      <c r="O1" s="403"/>
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="401"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="401"/>
+      <c r="O1" s="402"/>
       <c r="P1" s="417" t="s">
         <v>77</v>
       </c>
       <c r="Q1" s="417"/>
       <c r="R1" s="417"/>
       <c r="S1" s="417"/>
-      <c r="T1" s="400" t="s">
+      <c r="T1" s="399" t="s">
         <v>78</v>
       </c>
-      <c r="U1" s="400"/>
-      <c r="V1" s="400"/>
-      <c r="W1" s="400"/>
+      <c r="U1" s="399"/>
+      <c r="V1" s="399"/>
+      <c r="W1" s="399"/>
       <c r="X1" s="417" t="s">
         <v>79</v>
       </c>
       <c r="Y1" s="417"/>
       <c r="Z1" s="417"/>
       <c r="AA1" s="417"/>
-      <c r="AB1" s="400" t="s">
+      <c r="AB1" s="399" t="s">
         <v>80</v>
       </c>
-      <c r="AC1" s="400"/>
-      <c r="AD1" s="400"/>
-      <c r="AE1" s="400"/>
+      <c r="AC1" s="399"/>
+      <c r="AD1" s="399"/>
+      <c r="AE1" s="399"/>
       <c r="AF1" s="417" t="s">
         <v>81</v>
       </c>
       <c r="AG1" s="417"/>
       <c r="AH1" s="417"/>
       <c r="AI1" s="417"/>
-      <c r="AJ1" s="400" t="s">
+      <c r="AJ1" s="399" t="s">
         <v>82</v>
       </c>
-      <c r="AK1" s="400"/>
-      <c r="AL1" s="400"/>
-      <c r="AM1" s="400"/>
+      <c r="AK1" s="399"/>
+      <c r="AL1" s="399"/>
+      <c r="AM1" s="399"/>
       <c r="AN1" s="417" t="s">
         <v>83</v>
       </c>
       <c r="AO1" s="417"/>
       <c r="AP1" s="417"/>
       <c r="AQ1" s="417"/>
-      <c r="AR1" s="400" t="s">
+      <c r="AR1" s="399" t="s">
         <v>84</v>
       </c>
-      <c r="AS1" s="400"/>
-      <c r="AT1" s="400"/>
-      <c r="AU1" s="400"/>
+      <c r="AS1" s="399"/>
+      <c r="AT1" s="399"/>
+      <c r="AU1" s="399"/>
       <c r="AV1" s="417" t="s">
         <v>85</v>
       </c>
       <c r="AW1" s="417"/>
       <c r="AX1" s="417"/>
       <c r="AY1" s="417"/>
-      <c r="AZ1" s="400" t="s">
+      <c r="AZ1" s="399" t="s">
         <v>86</v>
       </c>
-      <c r="BA1" s="400"/>
-      <c r="BB1" s="400"/>
-      <c r="BC1" s="400"/>
+      <c r="BA1" s="399"/>
+      <c r="BB1" s="399"/>
+      <c r="BC1" s="399"/>
       <c r="BD1" s="417" t="s">
         <v>87</v>
       </c>
       <c r="BE1" s="417"/>
       <c r="BF1" s="417"/>
       <c r="BG1" s="417"/>
-      <c r="BH1" s="400" t="s">
+      <c r="BH1" s="399" t="s">
         <v>88</v>
       </c>
-      <c r="BI1" s="400"/>
-      <c r="BJ1" s="400"/>
-      <c r="BK1" s="400"/>
+      <c r="BI1" s="399"/>
+      <c r="BJ1" s="399"/>
+      <c r="BK1" s="399"/>
     </row>
     <row r="2" spans="1:63" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -55204,109 +55231,109 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:73" x14ac:dyDescent="0.4">
-      <c r="A1" s="400" t="s">
+      <c r="A1" s="399" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="400"/>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="401" t="s">
+      <c r="B1" s="399"/>
+      <c r="C1" s="399"/>
+      <c r="D1" s="399"/>
+      <c r="E1" s="400" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="402"/>
-      <c r="I1" s="402"/>
-      <c r="J1" s="402"/>
-      <c r="K1" s="402"/>
-      <c r="L1" s="402"/>
-      <c r="M1" s="402"/>
-      <c r="N1" s="402"/>
-      <c r="O1" s="402"/>
-      <c r="P1" s="402"/>
-      <c r="Q1" s="402"/>
-      <c r="R1" s="402"/>
-      <c r="S1" s="402"/>
-      <c r="T1" s="402"/>
-      <c r="U1" s="403"/>
-      <c r="V1" s="399" t="s">
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="401"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="401"/>
+      <c r="O1" s="401"/>
+      <c r="P1" s="401"/>
+      <c r="Q1" s="401"/>
+      <c r="R1" s="401"/>
+      <c r="S1" s="401"/>
+      <c r="T1" s="401"/>
+      <c r="U1" s="402"/>
+      <c r="V1" s="416" t="s">
         <v>77</v>
       </c>
-      <c r="W1" s="399"/>
-      <c r="X1" s="399"/>
-      <c r="Y1" s="399"/>
-      <c r="Z1" s="400" t="s">
+      <c r="W1" s="416"/>
+      <c r="X1" s="416"/>
+      <c r="Y1" s="416"/>
+      <c r="Z1" s="399" t="s">
         <v>78</v>
       </c>
-      <c r="AA1" s="400"/>
-      <c r="AB1" s="400"/>
-      <c r="AC1" s="400"/>
-      <c r="AD1" s="399" t="s">
+      <c r="AA1" s="399"/>
+      <c r="AB1" s="399"/>
+      <c r="AC1" s="399"/>
+      <c r="AD1" s="416" t="s">
         <v>79</v>
       </c>
-      <c r="AE1" s="399"/>
-      <c r="AF1" s="399"/>
-      <c r="AG1" s="399"/>
-      <c r="AH1" s="400" t="s">
+      <c r="AE1" s="416"/>
+      <c r="AF1" s="416"/>
+      <c r="AG1" s="416"/>
+      <c r="AH1" s="399" t="s">
         <v>80</v>
       </c>
-      <c r="AI1" s="400"/>
-      <c r="AJ1" s="400"/>
-      <c r="AK1" s="400"/>
-      <c r="AL1" s="399" t="s">
+      <c r="AI1" s="399"/>
+      <c r="AJ1" s="399"/>
+      <c r="AK1" s="399"/>
+      <c r="AL1" s="416" t="s">
         <v>81</v>
       </c>
-      <c r="AM1" s="399"/>
-      <c r="AN1" s="399"/>
-      <c r="AO1" s="399"/>
-      <c r="AP1" s="400" t="s">
+      <c r="AM1" s="416"/>
+      <c r="AN1" s="416"/>
+      <c r="AO1" s="416"/>
+      <c r="AP1" s="399" t="s">
         <v>82</v>
       </c>
-      <c r="AQ1" s="400"/>
-      <c r="AR1" s="400"/>
-      <c r="AS1" s="400"/>
-      <c r="AT1" s="399" t="s">
+      <c r="AQ1" s="399"/>
+      <c r="AR1" s="399"/>
+      <c r="AS1" s="399"/>
+      <c r="AT1" s="416" t="s">
         <v>83</v>
       </c>
-      <c r="AU1" s="399"/>
-      <c r="AV1" s="399"/>
-      <c r="AW1" s="399"/>
-      <c r="AX1" s="400" t="s">
+      <c r="AU1" s="416"/>
+      <c r="AV1" s="416"/>
+      <c r="AW1" s="416"/>
+      <c r="AX1" s="399" t="s">
         <v>84</v>
       </c>
-      <c r="AY1" s="400"/>
-      <c r="AZ1" s="400"/>
-      <c r="BA1" s="400"/>
-      <c r="BB1" s="399" t="s">
+      <c r="AY1" s="399"/>
+      <c r="AZ1" s="399"/>
+      <c r="BA1" s="399"/>
+      <c r="BB1" s="416" t="s">
         <v>85</v>
       </c>
-      <c r="BC1" s="399"/>
-      <c r="BD1" s="399"/>
-      <c r="BE1" s="399"/>
-      <c r="BF1" s="400" t="s">
+      <c r="BC1" s="416"/>
+      <c r="BD1" s="416"/>
+      <c r="BE1" s="416"/>
+      <c r="BF1" s="399" t="s">
         <v>86</v>
       </c>
-      <c r="BG1" s="400"/>
-      <c r="BH1" s="400"/>
-      <c r="BI1" s="400"/>
-      <c r="BJ1" s="399" t="s">
+      <c r="BG1" s="399"/>
+      <c r="BH1" s="399"/>
+      <c r="BI1" s="399"/>
+      <c r="BJ1" s="416" t="s">
         <v>87</v>
       </c>
-      <c r="BK1" s="399"/>
-      <c r="BL1" s="399"/>
-      <c r="BM1" s="399"/>
-      <c r="BN1" s="400" t="s">
+      <c r="BK1" s="416"/>
+      <c r="BL1" s="416"/>
+      <c r="BM1" s="416"/>
+      <c r="BN1" s="399" t="s">
         <v>88</v>
       </c>
-      <c r="BO1" s="400"/>
-      <c r="BP1" s="400"/>
-      <c r="BQ1" s="400"/>
-      <c r="BR1" s="399" t="s">
+      <c r="BO1" s="399"/>
+      <c r="BP1" s="399"/>
+      <c r="BQ1" s="399"/>
+      <c r="BR1" s="416" t="s">
         <v>495</v>
       </c>
-      <c r="BS1" s="399"/>
-      <c r="BT1" s="399"/>
-      <c r="BU1" s="399"/>
+      <c r="BS1" s="416"/>
+      <c r="BT1" s="416"/>
+      <c r="BU1" s="416"/>
     </row>
     <row r="2" spans="1:73" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -68348,6 +68375,12 @@
   </sheetData>
   <autoFilter ref="A2:BQ178" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="15">
+    <mergeCell ref="AH1:AK1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:U1"/>
+    <mergeCell ref="V1:Y1"/>
+    <mergeCell ref="Z1:AC1"/>
+    <mergeCell ref="AD1:AG1"/>
     <mergeCell ref="BJ1:BM1"/>
     <mergeCell ref="BN1:BQ1"/>
     <mergeCell ref="BR1:BU1"/>
@@ -68357,12 +68390,6 @@
     <mergeCell ref="AX1:BA1"/>
     <mergeCell ref="BB1:BE1"/>
     <mergeCell ref="BF1:BI1"/>
-    <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:U1"/>
-    <mergeCell ref="V1:Y1"/>
-    <mergeCell ref="Z1:AC1"/>
-    <mergeCell ref="AD1:AG1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -68492,97 +68519,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:63" x14ac:dyDescent="0.4">
-      <c r="A1" s="400" t="s">
+      <c r="A1" s="399" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="400"/>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="401" t="s">
+      <c r="B1" s="399"/>
+      <c r="C1" s="399"/>
+      <c r="D1" s="399"/>
+      <c r="E1" s="400" t="s">
         <v>491</v>
       </c>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="402"/>
-      <c r="I1" s="402"/>
-      <c r="J1" s="402"/>
-      <c r="K1" s="402"/>
-      <c r="L1" s="402"/>
-      <c r="M1" s="402"/>
-      <c r="N1" s="402"/>
-      <c r="O1" s="403"/>
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="401"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="401"/>
+      <c r="O1" s="402"/>
       <c r="P1" s="417" t="s">
         <v>77</v>
       </c>
       <c r="Q1" s="417"/>
       <c r="R1" s="417"/>
       <c r="S1" s="417"/>
-      <c r="T1" s="401" t="s">
+      <c r="T1" s="400" t="s">
         <v>78</v>
       </c>
-      <c r="U1" s="402"/>
-      <c r="V1" s="402"/>
-      <c r="W1" s="402"/>
+      <c r="U1" s="401"/>
+      <c r="V1" s="401"/>
+      <c r="W1" s="401"/>
       <c r="X1" s="417" t="s">
         <v>79</v>
       </c>
       <c r="Y1" s="417"/>
       <c r="Z1" s="417"/>
       <c r="AA1" s="417"/>
-      <c r="AB1" s="401" t="s">
+      <c r="AB1" s="400" t="s">
         <v>80</v>
       </c>
-      <c r="AC1" s="402"/>
-      <c r="AD1" s="402"/>
-      <c r="AE1" s="402"/>
+      <c r="AC1" s="401"/>
+      <c r="AD1" s="401"/>
+      <c r="AE1" s="401"/>
       <c r="AF1" s="417" t="s">
         <v>81</v>
       </c>
       <c r="AG1" s="417"/>
       <c r="AH1" s="417"/>
       <c r="AI1" s="417"/>
-      <c r="AJ1" s="401" t="s">
+      <c r="AJ1" s="400" t="s">
         <v>82</v>
       </c>
-      <c r="AK1" s="402"/>
-      <c r="AL1" s="402"/>
-      <c r="AM1" s="402"/>
+      <c r="AK1" s="401"/>
+      <c r="AL1" s="401"/>
+      <c r="AM1" s="401"/>
       <c r="AN1" s="417" t="s">
         <v>83</v>
       </c>
       <c r="AO1" s="417"/>
       <c r="AP1" s="417"/>
       <c r="AQ1" s="417"/>
-      <c r="AR1" s="401" t="s">
+      <c r="AR1" s="400" t="s">
         <v>84</v>
       </c>
-      <c r="AS1" s="402"/>
-      <c r="AT1" s="402"/>
-      <c r="AU1" s="402"/>
+      <c r="AS1" s="401"/>
+      <c r="AT1" s="401"/>
+      <c r="AU1" s="401"/>
       <c r="AV1" s="417" t="s">
         <v>85</v>
       </c>
       <c r="AW1" s="417"/>
       <c r="AX1" s="417"/>
       <c r="AY1" s="417"/>
-      <c r="AZ1" s="401" t="s">
+      <c r="AZ1" s="400" t="s">
         <v>86</v>
       </c>
-      <c r="BA1" s="402"/>
-      <c r="BB1" s="402"/>
-      <c r="BC1" s="402"/>
+      <c r="BA1" s="401"/>
+      <c r="BB1" s="401"/>
+      <c r="BC1" s="401"/>
       <c r="BD1" s="417" t="s">
         <v>87</v>
       </c>
       <c r="BE1" s="417"/>
       <c r="BF1" s="417"/>
       <c r="BG1" s="417"/>
-      <c r="BH1" s="401" t="s">
+      <c r="BH1" s="400" t="s">
         <v>88</v>
       </c>
-      <c r="BI1" s="402"/>
-      <c r="BJ1" s="402"/>
-      <c r="BK1" s="402"/>
+      <c r="BI1" s="401"/>
+      <c r="BJ1" s="401"/>
+      <c r="BK1" s="401"/>
     </row>
     <row r="2" spans="1:63" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
@@ -78885,13 +78912,6 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="16">
-    <mergeCell ref="C58:C60"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="C2:C11"/>
-    <mergeCell ref="C12:C17"/>
-    <mergeCell ref="C18:C28"/>
-    <mergeCell ref="C44:C53"/>
-    <mergeCell ref="C29:C43"/>
     <mergeCell ref="C180:C182"/>
     <mergeCell ref="C178:C179"/>
     <mergeCell ref="C163:C176"/>
@@ -78901,6 +78921,13 @@
     <mergeCell ref="C99:C108"/>
     <mergeCell ref="C109:C115"/>
     <mergeCell ref="C116:C162"/>
+    <mergeCell ref="C58:C60"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="C2:C11"/>
+    <mergeCell ref="C12:C17"/>
+    <mergeCell ref="C18:C28"/>
+    <mergeCell ref="C44:C53"/>
+    <mergeCell ref="C29:C43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -78908,6 +78935,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="107e75b3-53cc-4838-92d2-ebc011bd4832">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="888ccf44-0d39-41a2-ab17-f7efb2bf6977" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FD8CECCB51EC843BF514AFE68379818" ma:contentTypeVersion="18" ma:contentTypeDescription="Opret et nyt dokument." ma:contentTypeScope="" ma:versionID="eda339f53f012ceb64677667a741b441">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="107e75b3-53cc-4838-92d2-ebc011bd4832" xmlns:ns3="888ccf44-0d39-41a2-ab17-f7efb2bf6977" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="04a86f3db711706e561c315688f1c464" ns2:_="" ns3:_="">
     <xsd:import namespace="107e75b3-53cc-4838-92d2-ebc011bd4832"/>
@@ -79156,27 +79203,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2288FB7-E85A-4FE8-9E7A-FE572FF16064}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="107e75b3-53cc-4838-92d2-ebc011bd4832"/>
+    <ds:schemaRef ds:uri="888ccf44-0d39-41a2-ab17-f7efb2bf6977"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="107e75b3-53cc-4838-92d2-ebc011bd4832">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="888ccf44-0d39-41a2-ab17-f7efb2bf6977" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74B21D61-7BBD-4BD3-A9A5-1E8F98F2F686}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F91B7B9-75FF-4624-B506-952B5B54766C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -79193,29 +79245,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74B21D61-7BBD-4BD3-A9A5-1E8F98F2F686}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2288FB7-E85A-4FE8-9E7A-FE572FF16064}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="107e75b3-53cc-4838-92d2-ebc011bd4832"/>
-    <ds:schemaRef ds:uri="888ccf44-0d39-41a2-ab17-f7efb2bf6977"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update RfG_proc_Fault_3_0.6pu to RfG_proc_Fault_3_0.60pu and RfG_proc_Fault_3_0.8pu to RfG_proc_Fault_3_0.80pu for consistency
</commit_message>
<xml_diff>
--- a/testcases.xlsx
+++ b/testcases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://energinet-my.sharepoint.com/personal/prw_energinet_dk/Documents/Dokumenter/GitHub/MTB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="11_710D79F8E8F49B720F18F8F5A5BEAA4096265349" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C29E74CA-966E-4617-A0B9-A067781CB8F3}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="11_710D79F8E8F49B720F18F8F5A5BEAA4096265349" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9771C8EB-9FEE-4BCA-9478-F65D1BCD5756}"/>
   <bookViews>
     <workbookView xWindow="-15400" yWindow="-21710" windowWidth="51420" windowHeight="21100" tabRatio="822" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -165,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5513" uniqueCount="956">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5513" uniqueCount="958">
   <si>
     <t>Comment</t>
   </si>
@@ -3812,6 +3812,12 @@
   </si>
   <si>
     <t>DCC_SIPS+fault</t>
+  </si>
+  <si>
+    <t>RfG_proc_Fault_3_0.80pu</t>
+  </si>
+  <si>
+    <t>RfG_proc_Fault_3_0.60pu</t>
   </si>
 </sst>
 </file>
@@ -5883,17 +5889,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -9438,102 +9444,102 @@
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="333"/>
       <c r="B2" s="333"/>
-      <c r="C2" s="426" t="s">
+      <c r="C2" s="424" t="s">
         <v>843</v>
       </c>
-      <c r="D2" s="424" t="s">
+      <c r="D2" s="426" t="s">
         <v>907</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="333"/>
       <c r="B3" s="333"/>
-      <c r="C3" s="426"/>
-      <c r="D3" s="424"/>
+      <c r="C3" s="424"/>
+      <c r="D3" s="426"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="333"/>
       <c r="B4" s="333"/>
-      <c r="C4" s="426"/>
-      <c r="D4" s="424"/>
+      <c r="C4" s="424"/>
+      <c r="D4" s="426"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="333"/>
       <c r="B5" s="333"/>
-      <c r="C5" s="426"/>
-      <c r="D5" s="424"/>
+      <c r="C5" s="424"/>
+      <c r="D5" s="426"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="333"/>
       <c r="B6" s="333"/>
-      <c r="C6" s="426"/>
-      <c r="D6" s="424"/>
+      <c r="C6" s="424"/>
+      <c r="D6" s="426"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="333"/>
       <c r="B7" s="333"/>
-      <c r="C7" s="426"/>
-      <c r="D7" s="424"/>
+      <c r="C7" s="424"/>
+      <c r="D7" s="426"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="333"/>
       <c r="B8" s="333"/>
-      <c r="C8" s="426"/>
-      <c r="D8" s="424"/>
+      <c r="C8" s="424"/>
+      <c r="D8" s="426"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="333"/>
       <c r="B9" s="333"/>
-      <c r="C9" s="426"/>
-      <c r="D9" s="424"/>
+      <c r="C9" s="424"/>
+      <c r="D9" s="426"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="333"/>
       <c r="B10" s="333"/>
-      <c r="C10" s="426"/>
-      <c r="D10" s="424"/>
+      <c r="C10" s="424"/>
+      <c r="D10" s="426"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="333"/>
       <c r="B11" s="333"/>
-      <c r="C11" s="426"/>
-      <c r="D11" s="424"/>
+      <c r="C11" s="424"/>
+      <c r="D11" s="426"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="333"/>
       <c r="B12" s="333"/>
-      <c r="C12" s="426"/>
-      <c r="D12" s="424"/>
+      <c r="C12" s="424"/>
+      <c r="D12" s="426"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="333"/>
       <c r="B13" s="333"/>
-      <c r="C13" s="426"/>
-      <c r="D13" s="424"/>
+      <c r="C13" s="424"/>
+      <c r="D13" s="426"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="333"/>
       <c r="B14" s="333"/>
-      <c r="C14" s="426"/>
-      <c r="D14" s="424"/>
+      <c r="C14" s="424"/>
+      <c r="D14" s="426"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="333"/>
       <c r="B15" s="333"/>
-      <c r="C15" s="426"/>
-      <c r="D15" s="424"/>
+      <c r="C15" s="424"/>
+      <c r="D15" s="426"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="333"/>
       <c r="B16" s="333"/>
-      <c r="C16" s="426"/>
-      <c r="D16" s="424"/>
+      <c r="C16" s="424"/>
+      <c r="D16" s="426"/>
     </row>
     <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A17" s="315"/>
       <c r="B17" s="315"/>
-      <c r="C17" s="427"/>
-      <c r="D17" s="425"/>
+      <c r="C17" s="425"/>
+      <c r="D17" s="427"/>
     </row>
     <row r="18" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="335"/>
@@ -9541,7 +9547,7 @@
       <c r="C18" s="419" t="s">
         <v>361</v>
       </c>
-      <c r="D18" s="424" t="s">
+      <c r="D18" s="426" t="s">
         <v>844</v>
       </c>
     </row>
@@ -9549,115 +9555,115 @@
       <c r="A19" s="335"/>
       <c r="B19" s="335"/>
       <c r="C19" s="419"/>
-      <c r="D19" s="424"/>
+      <c r="D19" s="426"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="335"/>
       <c r="B20" s="335"/>
       <c r="C20" s="419"/>
-      <c r="D20" s="424"/>
+      <c r="D20" s="426"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="335"/>
       <c r="B21" s="335"/>
       <c r="C21" s="419"/>
-      <c r="D21" s="424"/>
+      <c r="D21" s="426"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="335"/>
       <c r="B22" s="335"/>
       <c r="C22" s="419"/>
-      <c r="D22" s="424"/>
+      <c r="D22" s="426"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="335"/>
       <c r="B23" s="335"/>
       <c r="C23" s="419"/>
-      <c r="D23" s="424"/>
+      <c r="D23" s="426"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" s="335"/>
       <c r="B24" s="335"/>
       <c r="C24" s="419"/>
-      <c r="D24" s="424"/>
+      <c r="D24" s="426"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" s="335"/>
       <c r="B25" s="335"/>
       <c r="C25" s="419"/>
-      <c r="D25" s="424"/>
+      <c r="D25" s="426"/>
     </row>
     <row r="26" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="335"/>
       <c r="B26" s="335"/>
       <c r="C26" s="419"/>
-      <c r="D26" s="424"/>
+      <c r="D26" s="426"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="335"/>
       <c r="B27" s="335"/>
       <c r="C27" s="419"/>
-      <c r="D27" s="424"/>
+      <c r="D27" s="426"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="335"/>
       <c r="B28" s="335"/>
       <c r="C28" s="419"/>
-      <c r="D28" s="424"/>
+      <c r="D28" s="426"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="335"/>
       <c r="B29" s="335"/>
       <c r="C29" s="419"/>
-      <c r="D29" s="424"/>
+      <c r="D29" s="426"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="335"/>
       <c r="B30" s="335"/>
       <c r="C30" s="419"/>
-      <c r="D30" s="424"/>
+      <c r="D30" s="426"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="335"/>
       <c r="B31" s="335"/>
       <c r="C31" s="419"/>
-      <c r="D31" s="424"/>
+      <c r="D31" s="426"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="335"/>
       <c r="B32" s="335"/>
       <c r="C32" s="419"/>
-      <c r="D32" s="424"/>
+      <c r="D32" s="426"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="335"/>
       <c r="B33" s="335"/>
       <c r="C33" s="419"/>
-      <c r="D33" s="424"/>
+      <c r="D33" s="426"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="335"/>
       <c r="B34" s="335"/>
       <c r="C34" s="419"/>
-      <c r="D34" s="424"/>
+      <c r="D34" s="426"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="335"/>
       <c r="B35" s="335"/>
       <c r="C35" s="419"/>
-      <c r="D35" s="424"/>
+      <c r="D35" s="426"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="335"/>
       <c r="B36" s="335"/>
       <c r="C36" s="419"/>
-      <c r="D36" s="424"/>
+      <c r="D36" s="426"/>
     </row>
     <row r="37" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A37" s="316"/>
       <c r="B37" s="316"/>
       <c r="C37" s="420"/>
-      <c r="D37" s="425"/>
+      <c r="D37" s="427"/>
     </row>
     <row r="38" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="334"/>
@@ -9665,7 +9671,7 @@
       <c r="C38" s="419" t="s">
         <v>845</v>
       </c>
-      <c r="D38" s="424" t="s">
+      <c r="D38" s="426" t="s">
         <v>846</v>
       </c>
     </row>
@@ -9673,115 +9679,115 @@
       <c r="A39" s="334"/>
       <c r="B39" s="334"/>
       <c r="C39" s="419"/>
-      <c r="D39" s="424"/>
+      <c r="D39" s="426"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A40" s="334"/>
       <c r="B40" s="334"/>
       <c r="C40" s="419"/>
-      <c r="D40" s="424"/>
+      <c r="D40" s="426"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A41" s="334"/>
       <c r="B41" s="334"/>
       <c r="C41" s="419"/>
-      <c r="D41" s="424"/>
+      <c r="D41" s="426"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A42" s="334"/>
       <c r="B42" s="334"/>
       <c r="C42" s="419"/>
-      <c r="D42" s="424"/>
+      <c r="D42" s="426"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A43" s="334"/>
       <c r="B43" s="334"/>
       <c r="C43" s="419"/>
-      <c r="D43" s="424"/>
+      <c r="D43" s="426"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A44" s="334"/>
       <c r="B44" s="334"/>
       <c r="C44" s="419"/>
-      <c r="D44" s="424"/>
+      <c r="D44" s="426"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A45" s="334"/>
       <c r="B45" s="334"/>
       <c r="C45" s="419"/>
-      <c r="D45" s="424"/>
+      <c r="D45" s="426"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A46" s="334"/>
       <c r="B46" s="334"/>
       <c r="C46" s="419"/>
-      <c r="D46" s="424"/>
+      <c r="D46" s="426"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A47" s="334"/>
       <c r="B47" s="334"/>
       <c r="C47" s="419"/>
-      <c r="D47" s="424"/>
+      <c r="D47" s="426"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A48" s="334"/>
       <c r="B48" s="334"/>
       <c r="C48" s="419"/>
-      <c r="D48" s="424"/>
+      <c r="D48" s="426"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A49" s="334"/>
       <c r="B49" s="334"/>
       <c r="C49" s="419"/>
-      <c r="D49" s="424"/>
+      <c r="D49" s="426"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A50" s="334"/>
       <c r="B50" s="334"/>
       <c r="C50" s="419"/>
-      <c r="D50" s="424"/>
+      <c r="D50" s="426"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A51" s="334"/>
       <c r="B51" s="334"/>
       <c r="C51" s="419"/>
-      <c r="D51" s="424"/>
+      <c r="D51" s="426"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A52" s="334"/>
       <c r="B52" s="334"/>
       <c r="C52" s="419"/>
-      <c r="D52" s="424"/>
+      <c r="D52" s="426"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" s="334"/>
       <c r="B53" s="334"/>
       <c r="C53" s="419"/>
-      <c r="D53" s="424"/>
+      <c r="D53" s="426"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A54" s="334"/>
       <c r="B54" s="334"/>
       <c r="C54" s="419"/>
-      <c r="D54" s="424"/>
+      <c r="D54" s="426"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A55" s="334"/>
       <c r="B55" s="334"/>
       <c r="C55" s="419"/>
-      <c r="D55" s="424"/>
+      <c r="D55" s="426"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A56" s="334"/>
       <c r="B56" s="334"/>
       <c r="C56" s="419"/>
-      <c r="D56" s="424"/>
+      <c r="D56" s="426"/>
     </row>
     <row r="57" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A57" s="317"/>
       <c r="B57" s="317"/>
       <c r="C57" s="420"/>
-      <c r="D57" s="425"/>
+      <c r="D57" s="427"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A58" s="336"/>
@@ -9789,7 +9795,7 @@
       <c r="C58" s="419" t="s">
         <v>847</v>
       </c>
-      <c r="D58" s="424" t="s">
+      <c r="D58" s="426" t="s">
         <v>848</v>
       </c>
     </row>
@@ -9797,85 +9803,85 @@
       <c r="A59" s="336"/>
       <c r="B59" s="336"/>
       <c r="C59" s="419"/>
-      <c r="D59" s="424"/>
+      <c r="D59" s="426"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A60" s="336"/>
       <c r="B60" s="336"/>
       <c r="C60" s="419"/>
-      <c r="D60" s="424"/>
+      <c r="D60" s="426"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A61" s="336"/>
       <c r="B61" s="336"/>
       <c r="C61" s="419"/>
-      <c r="D61" s="424"/>
+      <c r="D61" s="426"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A62" s="336"/>
       <c r="B62" s="336"/>
       <c r="C62" s="419"/>
-      <c r="D62" s="424"/>
+      <c r="D62" s="426"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A63" s="336"/>
       <c r="B63" s="336"/>
       <c r="C63" s="419"/>
-      <c r="D63" s="424"/>
+      <c r="D63" s="426"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A64" s="336"/>
       <c r="B64" s="336"/>
       <c r="C64" s="419"/>
-      <c r="D64" s="424"/>
+      <c r="D64" s="426"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A65" s="336"/>
       <c r="B65" s="336"/>
       <c r="C65" s="419"/>
-      <c r="D65" s="424"/>
+      <c r="D65" s="426"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A66" s="336"/>
       <c r="B66" s="336"/>
       <c r="C66" s="419"/>
-      <c r="D66" s="424"/>
+      <c r="D66" s="426"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A67" s="336"/>
       <c r="B67" s="336"/>
       <c r="C67" s="419"/>
-      <c r="D67" s="424"/>
+      <c r="D67" s="426"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A68" s="336"/>
       <c r="B68" s="336"/>
       <c r="C68" s="419"/>
-      <c r="D68" s="424"/>
+      <c r="D68" s="426"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A69" s="336"/>
       <c r="B69" s="336"/>
       <c r="C69" s="419"/>
-      <c r="D69" s="424"/>
+      <c r="D69" s="426"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A70" s="336"/>
       <c r="B70" s="336"/>
       <c r="C70" s="419"/>
-      <c r="D70" s="424"/>
+      <c r="D70" s="426"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A71" s="336"/>
       <c r="B71" s="336"/>
       <c r="C71" s="419"/>
-      <c r="D71" s="424"/>
+      <c r="D71" s="426"/>
     </row>
     <row r="72" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A72" s="318"/>
       <c r="B72" s="318"/>
       <c r="C72" s="420"/>
-      <c r="D72" s="425"/>
+      <c r="D72" s="427"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A73" s="338"/>
@@ -9883,7 +9889,7 @@
       <c r="C73" s="419" t="s">
         <v>849</v>
       </c>
-      <c r="D73" s="424" t="s">
+      <c r="D73" s="426" t="s">
         <v>850</v>
       </c>
     </row>
@@ -9891,97 +9897,97 @@
       <c r="A74" s="338"/>
       <c r="B74" s="338"/>
       <c r="C74" s="419"/>
-      <c r="D74" s="424"/>
+      <c r="D74" s="426"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A75" s="338"/>
       <c r="B75" s="338"/>
       <c r="C75" s="419"/>
-      <c r="D75" s="424"/>
+      <c r="D75" s="426"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A76" s="338"/>
       <c r="B76" s="338"/>
       <c r="C76" s="419"/>
-      <c r="D76" s="424"/>
+      <c r="D76" s="426"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A77" s="338"/>
       <c r="B77" s="338"/>
       <c r="C77" s="419"/>
-      <c r="D77" s="424"/>
+      <c r="D77" s="426"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A78" s="338"/>
       <c r="B78" s="338"/>
       <c r="C78" s="419"/>
-      <c r="D78" s="424"/>
+      <c r="D78" s="426"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A79" s="338"/>
       <c r="B79" s="338"/>
       <c r="C79" s="419"/>
-      <c r="D79" s="424"/>
+      <c r="D79" s="426"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A80" s="338"/>
       <c r="B80" s="338"/>
       <c r="C80" s="419"/>
-      <c r="D80" s="424"/>
+      <c r="D80" s="426"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A81" s="338"/>
       <c r="B81" s="338"/>
       <c r="C81" s="419"/>
-      <c r="D81" s="424"/>
+      <c r="D81" s="426"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A82" s="338"/>
       <c r="B82" s="338"/>
       <c r="C82" s="419"/>
-      <c r="D82" s="424"/>
+      <c r="D82" s="426"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A83" s="338"/>
       <c r="B83" s="338"/>
       <c r="C83" s="419"/>
-      <c r="D83" s="424"/>
+      <c r="D83" s="426"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A84" s="338"/>
       <c r="B84" s="338"/>
       <c r="C84" s="419"/>
-      <c r="D84" s="424"/>
+      <c r="D84" s="426"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A85" s="338"/>
       <c r="B85" s="338"/>
       <c r="C85" s="419"/>
-      <c r="D85" s="424"/>
+      <c r="D85" s="426"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A86" s="338"/>
       <c r="B86" s="338"/>
       <c r="C86" s="419"/>
-      <c r="D86" s="424"/>
+      <c r="D86" s="426"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A87" s="338"/>
       <c r="B87" s="338"/>
       <c r="C87" s="419"/>
-      <c r="D87" s="424"/>
+      <c r="D87" s="426"/>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A88" s="338"/>
       <c r="B88" s="338"/>
       <c r="C88" s="419"/>
-      <c r="D88" s="424"/>
+      <c r="D88" s="426"/>
     </row>
     <row r="89" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A89" s="319"/>
       <c r="B89" s="319"/>
       <c r="C89" s="420"/>
-      <c r="D89" s="425"/>
+      <c r="D89" s="427"/>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A90" s="337"/>
@@ -9989,7 +9995,7 @@
       <c r="C90" s="419" t="s">
         <v>851</v>
       </c>
-      <c r="D90" s="424" t="s">
+      <c r="D90" s="426" t="s">
         <v>852</v>
       </c>
     </row>
@@ -9997,49 +10003,49 @@
       <c r="A91" s="337"/>
       <c r="B91" s="337"/>
       <c r="C91" s="419"/>
-      <c r="D91" s="424"/>
+      <c r="D91" s="426"/>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A92" s="337"/>
       <c r="B92" s="337"/>
       <c r="C92" s="419"/>
-      <c r="D92" s="424"/>
+      <c r="D92" s="426"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A93" s="337"/>
       <c r="B93" s="337"/>
       <c r="C93" s="419"/>
-      <c r="D93" s="424"/>
+      <c r="D93" s="426"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A94" s="337"/>
       <c r="B94" s="337"/>
       <c r="C94" s="419"/>
-      <c r="D94" s="424"/>
+      <c r="D94" s="426"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A95" s="337"/>
       <c r="B95" s="337"/>
       <c r="C95" s="419"/>
-      <c r="D95" s="424"/>
+      <c r="D95" s="426"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A96" s="337"/>
       <c r="B96" s="337"/>
       <c r="C96" s="419"/>
-      <c r="D96" s="424"/>
+      <c r="D96" s="426"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A97" s="337"/>
       <c r="B97" s="337"/>
       <c r="C97" s="419"/>
-      <c r="D97" s="424"/>
+      <c r="D97" s="426"/>
     </row>
     <row r="98" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A98" s="320"/>
       <c r="B98" s="320"/>
       <c r="C98" s="420"/>
-      <c r="D98" s="425"/>
+      <c r="D98" s="427"/>
     </row>
     <row r="99" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A99" s="339"/>
@@ -10047,7 +10053,7 @@
       <c r="C99" s="422" t="s">
         <v>853</v>
       </c>
-      <c r="D99" s="424" t="s">
+      <c r="D99" s="426" t="s">
         <v>854</v>
       </c>
     </row>
@@ -10055,73 +10061,73 @@
       <c r="A100" s="339"/>
       <c r="B100" s="339"/>
       <c r="C100" s="422"/>
-      <c r="D100" s="424"/>
+      <c r="D100" s="426"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A101" s="339"/>
       <c r="B101" s="339"/>
       <c r="C101" s="422"/>
-      <c r="D101" s="424"/>
+      <c r="D101" s="426"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A102" s="339"/>
       <c r="B102" s="339"/>
       <c r="C102" s="422"/>
-      <c r="D102" s="424"/>
+      <c r="D102" s="426"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A103" s="339"/>
       <c r="B103" s="339"/>
       <c r="C103" s="422"/>
-      <c r="D103" s="424"/>
+      <c r="D103" s="426"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A104" s="339"/>
       <c r="B104" s="339"/>
       <c r="C104" s="422"/>
-      <c r="D104" s="424"/>
+      <c r="D104" s="426"/>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A105" s="339"/>
       <c r="B105" s="339"/>
       <c r="C105" s="422"/>
-      <c r="D105" s="424"/>
+      <c r="D105" s="426"/>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A106" s="339"/>
       <c r="B106" s="339"/>
       <c r="C106" s="422"/>
-      <c r="D106" s="424"/>
+      <c r="D106" s="426"/>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A107" s="339"/>
       <c r="B107" s="339"/>
       <c r="C107" s="422"/>
-      <c r="D107" s="424"/>
+      <c r="D107" s="426"/>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A108" s="339"/>
       <c r="B108" s="339"/>
       <c r="C108" s="422"/>
-      <c r="D108" s="424"/>
+      <c r="D108" s="426"/>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A109" s="339"/>
       <c r="B109" s="339"/>
       <c r="C109" s="422"/>
-      <c r="D109" s="424"/>
+      <c r="D109" s="426"/>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A110" s="339"/>
       <c r="B110" s="339"/>
       <c r="C110" s="422"/>
-      <c r="D110" s="424"/>
+      <c r="D110" s="426"/>
     </row>
     <row r="111" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A111" s="321"/>
       <c r="B111" s="321"/>
       <c r="C111" s="423"/>
-      <c r="D111" s="425"/>
+      <c r="D111" s="427"/>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A112" s="335"/>
@@ -10129,7 +10135,7 @@
       <c r="C112" s="419" t="s">
         <v>855</v>
       </c>
-      <c r="D112" s="424" t="s">
+      <c r="D112" s="426" t="s">
         <v>856</v>
       </c>
     </row>
@@ -10137,67 +10143,67 @@
       <c r="A113" s="335"/>
       <c r="B113" s="335"/>
       <c r="C113" s="419"/>
-      <c r="D113" s="424"/>
+      <c r="D113" s="426"/>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A114" s="335"/>
       <c r="B114" s="335"/>
       <c r="C114" s="419"/>
-      <c r="D114" s="424"/>
+      <c r="D114" s="426"/>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A115" s="335"/>
       <c r="B115" s="335"/>
       <c r="C115" s="419"/>
-      <c r="D115" s="424"/>
+      <c r="D115" s="426"/>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A116" s="335"/>
       <c r="B116" s="335"/>
       <c r="C116" s="419"/>
-      <c r="D116" s="424"/>
+      <c r="D116" s="426"/>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A117" s="335"/>
       <c r="B117" s="335"/>
       <c r="C117" s="419"/>
-      <c r="D117" s="424"/>
+      <c r="D117" s="426"/>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A118" s="335"/>
       <c r="B118" s="335"/>
       <c r="C118" s="419"/>
-      <c r="D118" s="424"/>
+      <c r="D118" s="426"/>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A119" s="335"/>
       <c r="B119" s="335"/>
       <c r="C119" s="419"/>
-      <c r="D119" s="424"/>
+      <c r="D119" s="426"/>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A120" s="335"/>
       <c r="B120" s="335"/>
       <c r="C120" s="419"/>
-      <c r="D120" s="424"/>
+      <c r="D120" s="426"/>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A121" s="335"/>
       <c r="B121" s="335"/>
       <c r="C121" s="419"/>
-      <c r="D121" s="424"/>
+      <c r="D121" s="426"/>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A122" s="335"/>
       <c r="B122" s="335"/>
       <c r="C122" s="419"/>
-      <c r="D122" s="424"/>
+      <c r="D122" s="426"/>
     </row>
     <row r="123" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A123" s="316"/>
       <c r="B123" s="316"/>
       <c r="C123" s="420"/>
-      <c r="D123" s="425"/>
+      <c r="D123" s="427"/>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A124" s="334"/>
@@ -10205,7 +10211,7 @@
       <c r="C124" s="419" t="s">
         <v>857</v>
       </c>
-      <c r="D124" s="424" t="s">
+      <c r="D124" s="426" t="s">
         <v>858</v>
       </c>
     </row>
@@ -10213,31 +10219,31 @@
       <c r="A125" s="334"/>
       <c r="B125" s="334"/>
       <c r="C125" s="419"/>
-      <c r="D125" s="424"/>
+      <c r="D125" s="426"/>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A126" s="334"/>
       <c r="B126" s="334"/>
       <c r="C126" s="419"/>
-      <c r="D126" s="424"/>
+      <c r="D126" s="426"/>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A127" s="334"/>
       <c r="B127" s="334"/>
       <c r="C127" s="419"/>
-      <c r="D127" s="424"/>
+      <c r="D127" s="426"/>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A128" s="334"/>
       <c r="B128" s="334"/>
       <c r="C128" s="419"/>
-      <c r="D128" s="424"/>
+      <c r="D128" s="426"/>
     </row>
     <row r="129" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A129" s="317"/>
       <c r="B129" s="317"/>
       <c r="C129" s="420"/>
-      <c r="D129" s="425"/>
+      <c r="D129" s="427"/>
     </row>
     <row r="130" spans="1:4" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A130" s="33"/>
@@ -10245,7 +10251,7 @@
       <c r="C130" s="419" t="s">
         <v>859</v>
       </c>
-      <c r="D130" s="424" t="s">
+      <c r="D130" s="426" t="s">
         <v>860</v>
       </c>
     </row>
@@ -10253,19 +10259,19 @@
       <c r="A131" s="33"/>
       <c r="B131" s="33"/>
       <c r="C131" s="419"/>
-      <c r="D131" s="424"/>
+      <c r="D131" s="426"/>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A132" s="33"/>
       <c r="B132" s="33"/>
       <c r="C132" s="419"/>
-      <c r="D132" s="424"/>
+      <c r="D132" s="426"/>
     </row>
     <row r="133" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A133" s="322"/>
       <c r="B133" s="322"/>
       <c r="C133" s="420"/>
-      <c r="D133" s="425"/>
+      <c r="D133" s="427"/>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A134" s="338"/>
@@ -10273,7 +10279,7 @@
       <c r="C134" s="419" t="s">
         <v>861</v>
       </c>
-      <c r="D134" s="424" t="s">
+      <c r="D134" s="426" t="s">
         <v>862</v>
       </c>
     </row>
@@ -10281,103 +10287,103 @@
       <c r="A135" s="338"/>
       <c r="B135" s="338"/>
       <c r="C135" s="419"/>
-      <c r="D135" s="424"/>
+      <c r="D135" s="426"/>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A136" s="338"/>
       <c r="B136" s="338"/>
       <c r="C136" s="419"/>
-      <c r="D136" s="424"/>
+      <c r="D136" s="426"/>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A137" s="338"/>
       <c r="B137" s="338"/>
       <c r="C137" s="419"/>
-      <c r="D137" s="424"/>
+      <c r="D137" s="426"/>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A138" s="338"/>
       <c r="B138" s="338"/>
       <c r="C138" s="419"/>
-      <c r="D138" s="424"/>
+      <c r="D138" s="426"/>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A139" s="338"/>
       <c r="B139" s="338"/>
       <c r="C139" s="419"/>
-      <c r="D139" s="424"/>
+      <c r="D139" s="426"/>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A140" s="338"/>
       <c r="B140" s="338"/>
       <c r="C140" s="419"/>
-      <c r="D140" s="424"/>
+      <c r="D140" s="426"/>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A141" s="338"/>
       <c r="B141" s="338"/>
       <c r="C141" s="419"/>
-      <c r="D141" s="424"/>
+      <c r="D141" s="426"/>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A142" s="338"/>
       <c r="B142" s="338"/>
       <c r="C142" s="419"/>
-      <c r="D142" s="424"/>
+      <c r="D142" s="426"/>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A143" s="338"/>
       <c r="B143" s="338"/>
       <c r="C143" s="419"/>
-      <c r="D143" s="424"/>
+      <c r="D143" s="426"/>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A144" s="338"/>
       <c r="B144" s="338"/>
       <c r="C144" s="419"/>
-      <c r="D144" s="424"/>
+      <c r="D144" s="426"/>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A145" s="338"/>
       <c r="B145" s="338"/>
       <c r="C145" s="419"/>
-      <c r="D145" s="424"/>
+      <c r="D145" s="426"/>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A146" s="338"/>
       <c r="B146" s="338"/>
       <c r="C146" s="419"/>
-      <c r="D146" s="424"/>
+      <c r="D146" s="426"/>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A147" s="338"/>
       <c r="B147" s="338"/>
       <c r="C147" s="419"/>
-      <c r="D147" s="424"/>
+      <c r="D147" s="426"/>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A148" s="338"/>
       <c r="B148" s="338"/>
       <c r="C148" s="419"/>
-      <c r="D148" s="424"/>
+      <c r="D148" s="426"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A149" s="338"/>
       <c r="B149" s="338"/>
       <c r="C149" s="419"/>
-      <c r="D149" s="424"/>
+      <c r="D149" s="426"/>
     </row>
     <row r="150" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A150" s="338"/>
       <c r="B150" s="338"/>
       <c r="C150" s="419"/>
-      <c r="D150" s="424"/>
+      <c r="D150" s="426"/>
     </row>
     <row r="151" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A151" s="319"/>
       <c r="B151" s="319"/>
       <c r="C151" s="420"/>
-      <c r="D151" s="425"/>
+      <c r="D151" s="427"/>
     </row>
     <row r="152" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A152" s="340"/>
@@ -10385,7 +10391,7 @@
       <c r="C152" s="419" t="s">
         <v>863</v>
       </c>
-      <c r="D152" s="424" t="s">
+      <c r="D152" s="426" t="s">
         <v>864</v>
       </c>
     </row>
@@ -10393,47 +10399,47 @@
       <c r="A153" s="340"/>
       <c r="B153" s="340"/>
       <c r="C153" s="419"/>
-      <c r="D153" s="424"/>
+      <c r="D153" s="426"/>
     </row>
     <row r="154" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A154" s="340"/>
       <c r="B154" s="340"/>
       <c r="C154" s="419"/>
-      <c r="D154" s="424"/>
+      <c r="D154" s="426"/>
     </row>
     <row r="155" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A155" s="323"/>
       <c r="B155" s="323"/>
       <c r="C155" s="420"/>
-      <c r="D155" s="425"/>
+      <c r="D155" s="427"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="24">
+    <mergeCell ref="C130:C133"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="C134:C151"/>
+    <mergeCell ref="D134:D151"/>
+    <mergeCell ref="C152:C155"/>
+    <mergeCell ref="D152:D155"/>
+    <mergeCell ref="C99:C111"/>
+    <mergeCell ref="D99:D111"/>
+    <mergeCell ref="C112:C123"/>
+    <mergeCell ref="D112:D123"/>
+    <mergeCell ref="C124:C129"/>
+    <mergeCell ref="D124:D129"/>
+    <mergeCell ref="C58:C72"/>
+    <mergeCell ref="D58:D72"/>
+    <mergeCell ref="C73:C89"/>
+    <mergeCell ref="D73:D89"/>
+    <mergeCell ref="C90:C98"/>
+    <mergeCell ref="D90:D98"/>
     <mergeCell ref="C2:C17"/>
     <mergeCell ref="D2:D17"/>
     <mergeCell ref="C18:C37"/>
     <mergeCell ref="D18:D37"/>
     <mergeCell ref="C38:C57"/>
     <mergeCell ref="D38:D57"/>
-    <mergeCell ref="C58:C72"/>
-    <mergeCell ref="D58:D72"/>
-    <mergeCell ref="C73:C89"/>
-    <mergeCell ref="D73:D89"/>
-    <mergeCell ref="C90:C98"/>
-    <mergeCell ref="D90:D98"/>
-    <mergeCell ref="C99:C111"/>
-    <mergeCell ref="D99:D111"/>
-    <mergeCell ref="C112:C123"/>
-    <mergeCell ref="D112:D123"/>
-    <mergeCell ref="C124:C129"/>
-    <mergeCell ref="D124:D129"/>
-    <mergeCell ref="C130:C133"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="C134:C151"/>
-    <mergeCell ref="D134:D151"/>
-    <mergeCell ref="C152:C155"/>
-    <mergeCell ref="D152:D155"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -33365,7 +33371,7 @@
         <v>1</v>
       </c>
       <c r="D170" s="79" t="s">
-        <v>703</v>
+        <v>956</v>
       </c>
       <c r="E170" s="81">
         <f t="shared" si="72"/>
@@ -33472,7 +33478,7 @@
         <v>1</v>
       </c>
       <c r="D171" s="79" t="s">
-        <v>704</v>
+        <v>957</v>
       </c>
       <c r="E171" s="81">
         <f t="shared" si="72"/>
@@ -68375,12 +68381,6 @@
   </sheetData>
   <autoFilter ref="A2:BQ178" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="15">
-    <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:U1"/>
-    <mergeCell ref="V1:Y1"/>
-    <mergeCell ref="Z1:AC1"/>
-    <mergeCell ref="AD1:AG1"/>
     <mergeCell ref="BJ1:BM1"/>
     <mergeCell ref="BN1:BQ1"/>
     <mergeCell ref="BR1:BU1"/>
@@ -68390,6 +68390,12 @@
     <mergeCell ref="AX1:BA1"/>
     <mergeCell ref="BB1:BE1"/>
     <mergeCell ref="BF1:BI1"/>
+    <mergeCell ref="AH1:AK1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:U1"/>
+    <mergeCell ref="V1:Y1"/>
+    <mergeCell ref="Z1:AC1"/>
+    <mergeCell ref="AD1:AG1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -78912,6 +78918,13 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="16">
+    <mergeCell ref="C58:C60"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="C2:C11"/>
+    <mergeCell ref="C12:C17"/>
+    <mergeCell ref="C18:C28"/>
+    <mergeCell ref="C44:C53"/>
+    <mergeCell ref="C29:C43"/>
     <mergeCell ref="C180:C182"/>
     <mergeCell ref="C178:C179"/>
     <mergeCell ref="C163:C176"/>
@@ -78921,13 +78934,6 @@
     <mergeCell ref="C99:C108"/>
     <mergeCell ref="C109:C115"/>
     <mergeCell ref="C116:C162"/>
-    <mergeCell ref="C58:C60"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="C2:C11"/>
-    <mergeCell ref="C12:C17"/>
-    <mergeCell ref="C18:C28"/>
-    <mergeCell ref="C44:C53"/>
-    <mergeCell ref="C29:C43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -78935,26 +78941,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="107e75b3-53cc-4838-92d2-ebc011bd4832">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="888ccf44-0d39-41a2-ab17-f7efb2bf6977" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FD8CECCB51EC843BF514AFE68379818" ma:contentTypeVersion="18" ma:contentTypeDescription="Opret et nyt dokument." ma:contentTypeScope="" ma:versionID="eda339f53f012ceb64677667a741b441">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="107e75b3-53cc-4838-92d2-ebc011bd4832" xmlns:ns3="888ccf44-0d39-41a2-ab17-f7efb2bf6977" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="04a86f3db711706e561c315688f1c464" ns2:_="" ns3:_="">
     <xsd:import namespace="107e75b3-53cc-4838-92d2-ebc011bd4832"/>
@@ -79203,32 +79189,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2288FB7-E85A-4FE8-9E7A-FE572FF16064}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="107e75b3-53cc-4838-92d2-ebc011bd4832"/>
-    <ds:schemaRef ds:uri="888ccf44-0d39-41a2-ab17-f7efb2bf6977"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74B21D61-7BBD-4BD3-A9A5-1E8F98F2F686}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="107e75b3-53cc-4838-92d2-ebc011bd4832">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="888ccf44-0d39-41a2-ab17-f7efb2bf6977" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F91B7B9-75FF-4624-B506-952B5B54766C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -79245,4 +79226,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74B21D61-7BBD-4BD3-A9A5-1E8F98F2F686}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2288FB7-E85A-4FE8-9E7A-FE572FF16064}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="107e75b3-53cc-4838-92d2-ebc011bd4832"/>
+    <ds:schemaRef ds:uri="888ccf44-0d39-41a2-ab17-f7efb2bf6977"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>